<commit_message>
Add business-specific email features and remove top preview banners
</commit_message>
<xml_diff>
--- a/website-demos/business-contacts.xlsx
+++ b/website-demos/business-contacts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="R3cdc95d0013a4594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="R2d439c0b0b304bba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,8 +97,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BusinessContacts" displayName="BusinessContacts" ref="A6:H106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BusinessContacts" displayName="BusinessContacts" ref="A6:L106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="No."/>
     <x:tableColumn id="2" name="Business name"/>
     <x:tableColumn id="3" name="Contact phone number"/>
@@ -107,6 +107,10 @@
     <x:tableColumn id="6" name="Contact notes"/>
     <x:tableColumn id="7" name="Contact source dates"/>
     <x:tableColumn id="8" name="Contact sources"/>
+    <x:tableColumn id="9" name="Specific demo features"/>
+    <x:tableColumn id="10" name="Customer benefit"/>
+    <x:tableColumn id="11" name="Email paragraph"/>
+    <x:tableColumn id="12" name="Demo limitations"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -315,6 +319,10 @@
     <ns0:col min="6" max="6" width="64" hidden="0" customWidth="1"/>
     <ns0:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
     <ns0:col min="8" max="8" width="72" hidden="0" customWidth="1"/>
+    <ns0:col min="9" max="9" width="68" hidden="0" customWidth="1"/>
+    <ns0:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
+    <ns0:col min="11" max="11" width="100" hidden="0" customWidth="1"/>
+    <ns0:col min="12" max="12" width="72" hidden="0" customWidth="1"/>
   </ns0:cols>
   <ns0:sheetData>
     <ns0:row r="2">
@@ -357,8 +365,20 @@
       <ns0:c r="H6" s="5" t="str">
         <ns0:v>Contact sources</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="7" ht="66" customHeight="1">
+      <ns0:c r="I6" s="5" t="str">
+        <ns0:v>Specific demo features</ns0:v>
+      </ns0:c>
+      <ns0:c r="J6" s="5" t="str">
+        <ns0:v>Customer benefit</ns0:v>
+      </ns0:c>
+      <ns0:c r="K6" s="5" t="str">
+        <ns0:v>Email paragraph</ns0:v>
+      </ns0:c>
+      <ns0:c r="L6" s="5" t="str">
+        <ns0:v>Demo limitations</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7" ht="150" customHeight="1">
       <ns0:c r="A7" s="6" t="n">
         <ns0:v>1</ns0:v>
       </ns0:c>
@@ -381,8 +401,21 @@
       <ns0:c r="H7" s="6" t="str">
         <ns0:v>https://www.yell.com/biz/andrew-leonards-leicester-1610927/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="8" ht="66" customHeight="1">
+      <ns0:c r="I7" s="6" t="str">
+        <ns0:v>Service guide for cuts, colour and occasions
+Appointment discussion notes with a preferred date</ns0:v>
+      </ns0:c>
+      <ns0:c r="J7" s="6" t="str">
+        <ns0:v>Help visitors explain the look and appointment they have in mind before calling.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K7" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Andrew Leonards Hairdressing. it includes service guide for cuts, colour and occasions and appointment discussion notes with a preferred date. the idea is to help visitors explain the look and appointment they have in mind before calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L7" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" ht="150" customHeight="1">
       <ns0:c r="A8" s="6" t="n">
         <ns0:v>2</ns0:v>
       </ns0:c>
@@ -405,8 +438,21 @@
       <ns0:c r="H8" s="6" t="str">
         <ns0:v>https://www.yell.com/biz/bar-sandwich-leicester-2506888/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="9" ht="66" customHeight="1">
+      <ns0:c r="I8" s="6" t="str">
+        <ns0:v>Lunch categories for sandwiches, soup and buffets
+Group lunch planner with headcount, date and dietary questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J8" s="6" t="str">
+        <ns0:v>Make a catering conversation easier to start with the key details already together.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K8" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Bar Sandwich. it includes lunch categories for sandwiches, soup and buffets and group lunch planner with headcount, date and dietary questions. the idea is to make a catering conversation easier to start with the key details already together. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L8" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" ht="150" customHeight="1">
       <ns0:c r="A9" s="6" t="n">
         <ns0:v>3</ns0:v>
       </ns0:c>
@@ -432,8 +478,21 @@
         <ns0:v>https://independentleicester.co.uk/independents/
 https://restaurantguru.com/5-COATS-Coffee-shop-and-Sandwich-bar-Leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="10" ht="66" customHeight="1">
+      <ns0:c r="I9" s="6" t="str">
+        <ns0:v>Lunch, cake and drink category filters
+Café shortlist with item details and a copyable visit note</ns0:v>
+      </ns0:c>
+      <ns0:c r="J9" s="6" t="str">
+        <ns0:v>Let people pick out a lunch or cake idea before visiting High Street.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K9" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for 5 Coats. it includes lunch, cake and drink category filters and café shortlist with item details and a copyable visit note. the idea is to let people pick out a lunch or cake idea before visiting High Street. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L9" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10" ht="150" customHeight="1">
       <ns0:c r="A10" s="6" t="n">
         <ns0:v>4</ns0:v>
       </ns0:c>
@@ -458,8 +517,21 @@
       <ns0:c r="H10" s="6" t="str">
         <ns0:v>https://localbeauty.uk/en-gb/i/2866-chloes-nails-leicester/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="11" ht="66" customHeight="1">
+      <ns0:c r="I10" s="6" t="str">
+        <ns0:v>Acrylic, BIAB, gel and pedicure treatment guide
+Existing product guidance, nail inspiration gallery and Booksy links</ns0:v>
+      </ns0:c>
+      <ns0:c r="J10" s="6" t="str">
+        <ns0:v>Help clients think through their treatment and removal questions before opening Booksy.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K10" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Chloe's Nails. it includes acrylic, BIAB, gel and pedicure treatment guide and existing product guidance, nail inspiration gallery and Booksy links. the idea is to help clients think through their treatment and removal questions before opening Booksy. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L10" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11" ht="150" customHeight="1">
       <ns0:c r="A11" s="6" t="n">
         <ns0:v>5</ns0:v>
       </ns0:c>
@@ -482,8 +554,21 @@
       <ns0:c r="H11" s="6" t="str">
         <ns0:v>https://www.leicestermarket.co.uk/outdoor-market/outdoor-market-directory/kotula-tomasz-2/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="12" ht="66" customHeight="1">
+      <ns0:c r="I11" s="6" t="str">
+        <ns0:v>Product enquiry list with quantities across Polish deli categories
+English or Polish enquiry summaries with collection and delivery questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J11" s="6" t="str">
+        <ns0:v>Help customers explain the products and quantities they want to ask the counter about.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K11" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Tomasz Kotula Butcher. it includes product enquiry list with quantities across Polish deli categories and english or Polish enquiry summaries with collection and delivery questions. the idea is to help customers explain the products and quantities they want to ask the counter about. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L11" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="150" customHeight="1">
       <ns0:c r="A12" s="6" t="n">
         <ns0:v>6</ns0:v>
       </ns0:c>
@@ -506,8 +591,21 @@
       <ns0:c r="H12" s="6" t="str">
         <ns0:v>https://visitleicester.info/point-of-interest/very-bazaar/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="13" ht="66" customHeight="1">
+      <ns0:c r="I12" s="6" t="str">
+        <ns0:v>Discovery guide across jewellery, crystals, clothing, gifts and incense
+Personal shopping or gift choice with a copyable visit list</ns0:v>
+      </ns0:c>
+      <ns0:c r="J12" s="6" t="str">
+        <ns0:v>Give visitors a starting point for browsing the shop or finding a gift.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K12" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for The Very Bazaar. it includes discovery guide across jewellery, crystals, clothing, gifts and incense and personal shopping or gift choice with a copyable visit list. the idea is to give visitors a starting point for browsing the shop or finding a gift. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L12" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13" ht="150" customHeight="1">
       <ns0:c r="A13" s="6" t="n">
         <ns0:v>7</ns0:v>
       </ns0:c>
@@ -530,8 +628,21 @@
       <ns0:c r="H13" s="6" t="str">
         <ns0:v>https://www.bizseek.co.uk/croft-hotel_9I-0116-212-0327</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="14" ht="66" customHeight="1">
+      <ns0:c r="I13" s="6" t="str">
+        <ns0:v>Room search and filters for single, twin, double and family options
+Bed arrangements beside links to the existing Booking.com profile</ns0:v>
+      </ns0:c>
+      <ns0:c r="J13" s="6" t="str">
+        <ns0:v>Help guests compare room types before checking current dates and rates.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K13" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Croft Hotel. it includes room search and filters for single, twin, double and family options and bed arrangements beside links to the existing Booking.com profile. the idea is to help guests compare room types before checking current dates and rates. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L13" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="150" customHeight="1">
       <ns0:c r="A14" s="6" t="n">
         <ns0:v>8</ns0:v>
       </ns0:c>
@@ -554,8 +665,21 @@
       <ns0:c r="H14" s="6" t="str">
         <ns0:v>https://www.bandsintown.com/v/10028541-duffys-bar?came_from=209</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="15" ht="66" customHeight="1">
+      <ns0:c r="I14" s="6" t="str">
+        <ns0:v>Gig list searchable by artist and filterable by month
+Gig details and a visit note for group, access or ticket questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J14" s="6" t="str">
+        <ns0:v>Help visitors find a relevant gig and organise the questions they need to ask.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K14" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Duffy's. it includes gig list searchable by artist and filterable by month and gig details and a visit note for group, access or ticket questions. the idea is to help visitors find a relevant gig and organise the questions they need to ask. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L14" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15" ht="150" customHeight="1">
       <ns0:c r="A15" s="6" t="n">
         <ns0:v>9</ns0:v>
       </ns0:c>
@@ -578,8 +702,22 @@
       <ns0:c r="H15" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/sams-beauty-den-in-butchers-salon-leicester-uk-10-allandale-road-o3llsgib</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="16" ht="66" customHeight="1">
+      <ns0:c r="I15" s="6" t="str">
+        <ns0:v>Service selector including Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J15" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K15" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Sam’s Beauty Den in Butchers Salon. visitors can compare options such as Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L15" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16" ht="150" customHeight="1">
       <ns0:c r="A16" s="6" t="n">
         <ns0:v>10</ns0:v>
       </ns0:c>
@@ -602,8 +740,21 @@
       <ns0:c r="H16" s="6" t="str">
         <ns0:v>https://visitleicester.info/point-of-interest/mitsuki/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="17" ht="66" customHeight="1">
+      <ns0:c r="I16" s="6" t="str">
+        <ns0:v>Sushi, bento and ramen category filters
+Dish detail views and a copyable favourites list</ns0:v>
+      </ns0:c>
+      <ns0:c r="J16" s="6" t="str">
+        <ns0:v>Help diners put a few Japanese dishes together before their visit.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K16" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Mitsuki. it includes sushi, bento and ramen category filters and dish detail views and a copyable favourites list. the idea is to help diners put a few Japanese dishes together before their visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L16" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17" ht="150" customHeight="1">
       <ns0:c r="A17" s="6" t="n">
         <ns0:v>11</ns0:v>
       </ns0:c>
@@ -626,8 +777,21 @@
       <ns0:c r="H17" s="6" t="str">
         <ns0:v>https://niche-eats.co.uk/restaurants/leicester/kurda-restaurant-leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="18" ht="66" customHeight="1">
+      <ns0:c r="I17" s="6" t="str">
+        <ns0:v>Sharing platter guide organised by group size
+Meal discussion note with food choice, guest count and preferred date</ns0:v>
+      </ns0:c>
+      <ns0:c r="J17" s="6" t="str">
+        <ns0:v>Help groups decide what to ask about before speaking to the restaurant.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K17" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Kurda Restaurant. it includes sharing platter guide organised by group size and meal discussion note with food choice, guest count and preferred date. the idea is to help groups decide what to ask about before speaking to the restaurant. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L17" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18" ht="150" customHeight="1">
       <ns0:c r="A18" s="6" t="n">
         <ns0:v>12</ns0:v>
       </ns0:c>
@@ -651,8 +815,21 @@
         <ns0:v>https://tatraleicester.co.uk/contact/
 https://www.bizseek.co.uk/tatra-eastern-corner-07883-518180</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="19" ht="66" customHeight="1">
+      <ns0:c r="I18" s="6" t="str">
+        <ns0:v>Menu sections with dish photographs
+Event enquiry outline covering occasion, guests, food and collection preferences</ns0:v>
+      </ns0:c>
+      <ns0:c r="J18" s="6" t="str">
+        <ns0:v>Make it easier to start a conversation about a celebration or catering enquiry.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K18" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Tatra Eastern Corner. it includes menu sections with dish photographs and event enquiry outline covering occasion, guests, food and collection preferences. the idea is to make it easier to start a conversation about a celebration or catering enquiry. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L18" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19" ht="150" customHeight="1">
       <ns0:c r="A19" s="6" t="n">
         <ns0:v>13</ns0:v>
       </ns0:c>
@@ -677,8 +854,21 @@
 https://img01.products.bt.co.uk/content/dam/bt/a-z-directory/leics-a-z-directory.pdf
 https://play.google.com/store/apps/details?id=com.palya_catering.mobile.app</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="20" ht="66" customHeight="1">
+      <ns0:c r="I19" s="6" t="str">
+        <ns0:v>Daily versus weekly and monthly meal sections
+Catering brief with occasion, date, guest count, location and dietary requests</ns0:v>
+      </ns0:c>
+      <ns0:c r="J19" s="6" t="str">
+        <ns0:v>Bring the important event details together before a catering conversation.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K19" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for PALYA'S Catering. it includes daily versus weekly and monthly meal sections and catering brief with occasion, date, guest count, location and dietary requests. the idea is to bring the important event details together before a catering conversation. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L19" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20" ht="150" customHeight="1">
       <ns0:c r="A20" s="6" t="n">
         <ns0:v>14</ns0:v>
       </ns0:c>
@@ -701,8 +891,21 @@
       <ns0:c r="H20" s="6" t="str">
         <ns0:v>https://www.yell.com/biz/piero-s-snack-bar-leicester-732656/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="21" ht="66" customHeight="1">
+      <ns0:c r="I20" s="6" t="str">
+        <ns0:v>Breakfast, lunch and drinks filters
+Café call outline with visit type, group size and questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J20" s="6" t="str">
+        <ns0:v>Help customers narrow down a café visit and explain what they need when calling.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K20" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Piero Snack Bar. it includes breakfast, lunch and drinks filters and café call outline with visit type, group size and questions. the idea is to help customers narrow down a café visit and explain what they need when calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L20" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21" ht="150" customHeight="1">
       <ns0:c r="A21" s="6" t="n">
         <ns0:v>15</ns0:v>
       </ns0:c>
@@ -726,8 +929,21 @@
         <ns0:v>https://www.countryfayreleicester.com/contact
 https://www.bizseek.co.uk/country-fayre_995-0116-253-1432</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="22" ht="66" customHeight="1">
+      <ns0:c r="I21" s="6" t="str">
+        <ns0:v>Product range explorer for cheese, meats, pastry and dairy
+Different enquiry paths for home shopping, trade supply and celebration cheese cakes</ns0:v>
+      </ns0:c>
+      <ns0:c r="J21" s="6" t="str">
+        <ns0:v>Separate everyday purchases from trade and celebration enquiries.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K21" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Country Fayre Foods. it includes product range explorer for cheese, meats, pastry and dairy and different enquiry paths for home shopping, trade supply and celebration cheese cakes. the idea is to separate everyday purchases from trade and celebration enquiries. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L21" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22" ht="150" customHeight="1">
       <ns0:c r="A22" s="6" t="n">
         <ns0:v>16</ns0:v>
       </ns0:c>
@@ -750,8 +966,21 @@
       <ns0:c r="H22" s="6" t="str">
         <ns0:v>https://www.restaurantji.co.uk/leicestershire/leicester/taste-of-china-restaurant-/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="23" ht="66" customHeight="1">
+      <ns0:c r="I22" s="6" t="str">
+        <ns0:v>Searchable rice and noodle menu selection
+Meal note with group size, visit type and questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J22" s="6" t="str">
+        <ns0:v>Help customers narrow down dishes and prepare a clear meal enquiry.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K22" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Taste of China. it includes searchable rice and noodle menu selection and meal note with group size, visit type and questions. the idea is to help customers narrow down dishes and prepare a clear meal enquiry. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L22" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23" ht="150" customHeight="1">
       <ns0:c r="A23" s="6" t="n">
         <ns0:v>17</ns0:v>
       </ns0:c>
@@ -776,8 +1005,21 @@
       <ns0:c r="H23" s="6" t="str">
         <ns0:v>https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d15705562-Reviews-Noodle_House-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="24" ht="66" customHeight="1">
+      <ns0:c r="I23" s="6" t="str">
+        <ns0:v>Box mix, noodle, rice and soup filters
+Group shortlist with quantities for each selected dish</ns0:v>
+      </ns0:c>
+      <ns0:c r="J23" s="6" t="str">
+        <ns0:v>Help people coordinate a group meal before checking the real ordering menu.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K23" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Noodle House. it includes box mix, noodle, rice and soup filters and group shortlist with quantities for each selected dish. the idea is to help people coordinate a group meal before checking the real ordering menu. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L23" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24" ht="150" customHeight="1">
       <ns0:c r="A24" s="6" t="n">
         <ns0:v>18</ns0:v>
       </ns0:c>
@@ -801,8 +1043,21 @@
         <ns0:v>https://eatoutmap.com/en/uk/leicester/paper-wings-cafe
 https://paperwingscafe.co.uk/pages/private-hire-events</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="25" ht="66" customHeight="1">
+      <ns0:c r="I24" s="6" t="str">
+        <ns0:v>Separate daytime upstairs and evening whole-space hire options
+Hire enquiry outline with event type, date, guests, duration and setup needs</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="6" t="str">
+        <ns0:v>Make a workshop, meetup or celebration enquiry easier to explain.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K24" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Paper Wings Café. it includes separate daytime upstairs and evening whole-space hire options and hire enquiry outline with event type, date, guests, duration and setup needs. the idea is to make a workshop, meetup or celebration enquiry easier to explain. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L24" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25" ht="150" customHeight="1">
       <ns0:c r="A25" s="6" t="n">
         <ns0:v>19</ns0:v>
       </ns0:c>
@@ -825,8 +1080,22 @@
       <ns0:c r="H25" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/oh-so-pretty-wigston-4-liskeard-house-telbdqpd</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="26" ht="66" customHeight="1">
+      <ns0:c r="I25" s="6" t="str">
+        <ns0:v>Service selector including Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J25" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K25" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Oh So Pretty. visitors can compare options such as Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L25" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26" ht="150" customHeight="1">
       <ns0:c r="A26" s="6" t="n">
         <ns0:v>20</ns0:v>
       </ns0:c>
@@ -849,8 +1118,21 @@
       <ns0:c r="H26" s="6" t="str">
         <ns0:v>https://foneplus.co.uk/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="27" ht="66" customHeight="1">
+      <ns0:c r="I26" s="6" t="str">
+        <ns0:v>Repair enquiry guide for phones, tablets, computers and consoles
+Device model and fault selection with a reviewable enquiry summary</ns0:v>
+      </ns0:c>
+      <ns0:c r="J26" s="6" t="str">
+        <ns0:v>Help customers describe their device problem before contacting the Leicester shop.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K26" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Fone Plus. it includes repair enquiry guide for phones, tablets, computers and consoles and device model and fault selection with a reviewable enquiry summary. the idea is to help customers describe their device problem before contacting the Leicester shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L26" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27" ht="150" customHeight="1">
       <ns0:c r="A27" s="6" t="n">
         <ns0:v>21</ns0:v>
       </ns0:c>
@@ -874,8 +1156,21 @@
         <ns0:v>https://romaleicester.co.uk/location/
 https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d1637479-Reviews-Cafe_Roma-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="28" ht="66" customHeight="1">
+      <ns0:c r="I27" s="6" t="str">
+        <ns0:v>Brunch, lunch and evening menu sections
+Dining enquiry notes with occasion and guests, plus the existing Dojo booking link</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="6" t="str">
+        <ns0:v>Help visitors choose the right service and prepare their dining questions.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K27" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Roma. it includes brunch, lunch and evening menu sections and dining enquiry notes with occasion and guests, plus the existing Dojo booking link. the idea is to help visitors choose the right service and prepare their dining questions. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L27" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28" ht="150" customHeight="1">
       <ns0:c r="A28" s="6" t="n">
         <ns0:v>22</ns0:v>
       </ns0:c>
@@ -894,8 +1189,22 @@
       <ns0:c r="F28" s="6" t="str"/>
       <ns0:c r="G28" s="6" t="str"/>
       <ns0:c r="H28" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="29" ht="66" customHeight="1">
+      <ns0:c r="I28" s="6" t="str">
+        <ns0:v>Service selector including Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J28" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K28" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Cabello Mens Hairsalon. visitors can compare options such as Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L28" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29" ht="150" customHeight="1">
       <ns0:c r="A29" s="6" t="n">
         <ns0:v>23</ns0:v>
       </ns0:c>
@@ -918,8 +1227,21 @@
       <ns0:c r="H29" s="6" t="str">
         <ns0:v>https://www.yell.com/biz/frank-lee-and-son-ltd-leicester-1578776/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="30" ht="66" customHeight="1">
+      <ns0:c r="I29" s="6" t="str">
+        <ns0:v>Range guide including beef, pork, lamb and alternative cuts
+Copyable butcher ask list based on cooking method, people and recipe questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J29" s="6" t="str">
+        <ns0:v>Help customers ask for a suitable cut without needing to know every product name.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K29" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Frank Lee And Son. it includes range guide including beef, pork, lamb and alternative cuts and copyable butcher ask list based on cooking method, people and recipe questions. the idea is to help customers ask for a suitable cut without needing to know every product name. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L29" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30" ht="150" customHeight="1">
       <ns0:c r="A30" s="6" t="n">
         <ns0:v>24</ns0:v>
       </ns0:c>
@@ -942,8 +1264,21 @@
       <ns0:c r="H30" s="6" t="str">
         <ns0:v>https://www.locaji.co.uk/leicestershire/leicester/guilin-street-food/431739/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="31" ht="66" customHeight="1">
+      <ns0:c r="I30" s="6" t="str">
+        <ns0:v>Regional noodle guide with English and Chinese dish names
+Counter checklist for a chosen dish, group size, spice and ingredient questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="6" t="str">
+        <ns0:v>Make unfamiliar dishes easier to explore before asking at the counter.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K30" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Guilin Street Food. it includes regional noodle guide with English and Chinese dish names and counter checklist for a chosen dish, group size, spice and ingredient questions. the idea is to make unfamiliar dishes easier to explore before asking at the counter. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L30" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31" ht="150" customHeight="1">
       <ns0:c r="A31" s="6" t="n">
         <ns0:v>25</ns0:v>
       </ns0:c>
@@ -966,8 +1301,21 @@
       <ns0:c r="H31" s="6" t="str">
         <ns0:v>https://www.leicestermarket.co.uk/outdoor-market/outdoor-market-directory/leicester-wholesale-fish-direct/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="32" ht="66" customHeight="1">
+      <ns0:c r="I31" s="6" t="str">
+        <ns0:v>Fish, shellfish and crustacean range guide
+Question list covering cooking plan, preparation, weight and handling</ns0:v>
+      </ns0:c>
+      <ns0:c r="J31" s="6" t="str">
+        <ns0:v>Help customers arrive with useful questions about choosing and preparing their fish.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K31" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Leicester Wholesale Fish Direct. it includes fish, shellfish and crustacean range guide and question list covering cooking plan, preparation, weight and handling. the idea is to help customers arrive with useful questions about choosing and preparing their fish. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L31" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32" ht="150" customHeight="1">
       <ns0:c r="A32" s="6" t="n">
         <ns0:v>26</ns0:v>
       </ns0:c>
@@ -990,8 +1338,22 @@
       <ns0:c r="H32" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/violets-leicester-mowmacre-sports-ground-j96u6szs</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="33" ht="66" customHeight="1">
+      <ns0:c r="I32" s="6" t="str">
+        <ns0:v>Service selector including Cut &amp; Blow Dry and Blow Dry
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J32" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K32" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Violet’s Hair Studio. visitors can compare options such as Cut &amp; Blow Dry and Blow Dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L32" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33" ht="150" customHeight="1">
       <ns0:c r="A33" s="6" t="n">
         <ns0:v>27</ns0:v>
       </ns0:c>
@@ -1014,8 +1376,22 @@
       <ns0:c r="H33" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/beauty-by-mel-glenfield-13-stamford-street-zk5d4485</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="34" ht="66" customHeight="1">
+      <ns0:c r="I33" s="6" t="str">
+        <ns0:v>Service selector including Back, Neck &amp; Shoulders and Gel Toes
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J33" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K33" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Beauty by Mel. visitors can compare options such as Back, Neck &amp; Shoulders and Gel Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L33" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34" ht="150" customHeight="1">
       <ns0:c r="A34" s="6" t="n">
         <ns0:v>28</ns0:v>
       </ns0:c>
@@ -1034,8 +1410,21 @@
       <ns0:c r="F34" s="6" t="str"/>
       <ns0:c r="G34" s="6" t="str"/>
       <ns0:c r="H34" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="35" ht="66" customHeight="1">
+      <ns0:c r="I34" s="6" t="str">
+        <ns0:v>Fruit tea finder for a chosen flavour
+Single flavour versus flavour pair matching</ns0:v>
+      </ns0:c>
+      <ns0:c r="J34" s="6" t="str">
+        <ns0:v>Help someone who likes a particular fruit find relevant drinks quickly.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K34" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Blossom Boba. it includes fruit tea finder for a chosen flavour and single flavour versus flavour pair matching. the idea is to help someone who likes a particular fruit find relevant drinks quickly. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L34" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35" ht="150" customHeight="1">
       <ns0:c r="A35" s="6" t="n">
         <ns0:v>29</ns0:v>
       </ns0:c>
@@ -1058,8 +1447,21 @@
       <ns0:c r="H35" s="6" t="str">
         <ns0:v>https://leicesterrestaurantweek.co.uk/restaurants/latin-kitchen/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="36" ht="66" customHeight="1">
+      <ns0:c r="I35" s="6" t="str">
+        <ns0:v>Plated food versus handheld food filters
+Dish planner with side choice, quantities and group questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J35" s="6" t="str">
+        <ns0:v>Help customers put their meal preferences into one clear discussion note.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K35" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Latin Kitchen. it includes plated food versus handheld food filters and dish planner with side choice, quantities and group questions. the idea is to help customers put their meal preferences into one clear discussion note. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L35" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36" ht="150" customHeight="1">
       <ns0:c r="A36" s="6" t="n">
         <ns0:v>30</ns0:v>
       </ns0:c>
@@ -1082,8 +1484,21 @@
       <ns0:c r="H36" s="6" t="str">
         <ns0:v>https://restaurantguru.com/sakura-Leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="37" ht="66" customHeight="1">
+      <ns0:c r="I36" s="6" t="str">
+        <ns0:v>Searchable sushi, bento, noodle and starter selection
+Copyable meal shortlist with a personal reminder</ns0:v>
+      </ns0:c>
+      <ns0:c r="J36" s="6" t="str">
+        <ns0:v>Help diners keep their favourite dishes together while choosing a meal.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K36" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Sakura. it includes searchable sushi, bento, noodle and starter selection and copyable meal shortlist with a personal reminder. the idea is to help diners keep their favourite dishes together while choosing a meal. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L36" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="37" ht="150" customHeight="1">
       <ns0:c r="A37" s="6" t="n">
         <ns0:v>31</ns0:v>
       </ns0:c>
@@ -1106,8 +1521,21 @@
       <ns0:c r="H37" s="6" t="str">
         <ns0:v>https://www.yell.com/biz/silver-street-cafe-leicester-734925/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="38" ht="66" customHeight="1">
+      <ns0:c r="I37" s="6" t="str">
+        <ns0:v>Search and filters for breakfast plates and hot cobs
+Copyable café shortlist with group size and beans or tomatoes preference</ns0:v>
+      </ns0:c>
+      <ns0:c r="J37" s="6" t="str">
+        <ns0:v>Help visitors organise a breakfast choice before checking it with the café.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K37" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Silver Street Cafe. it includes search and filters for breakfast plates and hot cobs and copyable café shortlist with group size and beans or tomatoes preference. the idea is to help visitors organise a breakfast choice before checking it with the café. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L37" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="38" ht="150" customHeight="1">
       <ns0:c r="A38" s="6" t="n">
         <ns0:v>32</ns0:v>
       </ns0:c>
@@ -1131,8 +1559,22 @@
         <ns0:v>https://www.fresha.com/a/the-beauty-lab-thurmaston-7-silverdale-drive-h5nuazbm
 https://www.sumupbookings.com/the-beauty-lab-6</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="39" ht="66" customHeight="1">
+      <ns0:c r="I38" s="6" t="str">
+        <ns0:v>Service selector including Brow wax and Brow wax &amp; tint
+Listed prices and appointment lengths update with the selected service
+Link to the existing SumUp Bookings booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J38" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K38" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for The Beauty Lab. visitors can compare options such as Brow wax and Brow wax &amp; tint, see the listed price and appointment length, then open your SumUp Bookings booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L38" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="39" ht="150" customHeight="1">
       <ns0:c r="A39" s="6" t="n">
         <ns0:v>33</ns0:v>
       </ns0:c>
@@ -1155,8 +1597,21 @@
       <ns0:c r="H39" s="6" t="str">
         <ns0:v>https://steaknlounge.co.uk/contact-us/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="40" ht="66" customHeight="1">
+      <ns0:c r="I39" s="6" t="str">
+        <ns0:v>Food category explorer across steaks, starters, sizzlers and more
+Food photograph viewer and links to the existing booking route</ns0:v>
+      </ns0:c>
+      <ns0:c r="J39" s="6" t="str">
+        <ns0:v>Help diners explore the type of evening they want before checking availability.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K39" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Steak &amp; Lounge. it includes food category explorer across steaks, starters, sizzlers and more and food photograph viewer and links to the existing booking route. the idea is to help diners explore the type of evening they want before checking availability. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L39" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="40" ht="150" customHeight="1">
       <ns0:c r="A40" s="6" t="n">
         <ns0:v>34</ns0:v>
       </ns0:c>
@@ -1181,8 +1636,21 @@
       <ns0:c r="H40" s="6" t="str">
         <ns0:v>https://explorereats.com/restaurants/raykdi/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="41" ht="66" customHeight="1">
+      <ns0:c r="I40" s="6" t="str">
+        <ns0:v>Menu category filters and item detail views
+Copyable dish shortlist</ns0:v>
+      </ns0:c>
+      <ns0:c r="J40" s="6" t="str">
+        <ns0:v>Help customers explore the chaat menu and keep the dishes they want to try together.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K40" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Raykdi. it includes menu category filters and item detail views and copyable dish shortlist. the idea is to help customers explore the chaat menu and keep the dishes they want to try together. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L40" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="41" ht="150" customHeight="1">
       <ns0:c r="A41" s="6" t="n">
         <ns0:v>35</ns0:v>
       </ns0:c>
@@ -1208,8 +1676,21 @@
         <ns0:v>https://www.leicestermarket.co.uk/outdoor-market/outdoor-market-directory/edwards-butchers-2/
 https://www.yell.com/biz/keith-ashmore-s-quality-butchers-leicester-3799801/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="42" ht="66" customHeight="1">
+      <ns0:c r="I41" s="6" t="str">
+        <ns0:v>Range guide covering beef, lamb, pork, poultry and offal
+Butcher question list shaped by meal type, people and preparation needs</ns0:v>
+      </ns0:c>
+      <ns0:c r="J41" s="6" t="str">
+        <ns0:v>Help customers explain what they are cooking and get advice at the counter.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K41" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Keith Ashmore. it includes range guide covering beef, lamb, pork, poultry and offal and butcher question list shaped by meal type, people and preparation needs. the idea is to help customers explain what they are cooking and get advice at the counter. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L41" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="42" ht="150" customHeight="1">
       <ns0:c r="A42" s="6" t="n">
         <ns0:v>36</ns0:v>
       </ns0:c>
@@ -1232,8 +1713,21 @@
       <ns0:c r="H42" s="6" t="str">
         <ns0:v>https://restaurantguru.com/La-Foret-Cafe-Leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="43" ht="66" customHeight="1">
+      <ns0:c r="I42" s="6" t="str">
+        <ns0:v>Brunch, lunch and drinks filters
+Café list for shortlisted dishes and drinks</ns0:v>
+      </ns0:c>
+      <ns0:c r="J42" s="6" t="str">
+        <ns0:v>Help visitors choose a few brunch and drink ideas before arriving.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K42" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for La Foret Cafe. it includes brunch, lunch and drinks filters and café list for shortlisted dishes and drinks. the idea is to help visitors choose a few brunch and drink ideas before arriving. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L42" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="43" ht="150" customHeight="1">
       <ns0:c r="A43" s="6" t="n">
         <ns0:v>37</ns0:v>
       </ns0:c>
@@ -1256,8 +1750,21 @@
       <ns0:c r="H43" s="6" t="str">
         <ns0:v>https://es.restaurantguru.com/LYNN-Leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="44" ht="66" customHeight="1">
+      <ns0:c r="I43" s="6" t="str">
+        <ns0:v>Separate brunch and bistro views with dish search
+Meal note that includes occasion, day and group size</ns0:v>
+      </ns0:c>
+      <ns0:c r="J43" s="6" t="str">
+        <ns0:v>Help visitors distinguish a brunch plan from an evening meal.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K43" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for LYNN. it includes separate brunch and bistro views with dish search and meal note that includes occasion, day and group size. the idea is to help visitors distinguish a brunch plan from an evening meal. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L43" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="44" ht="150" customHeight="1">
       <ns0:c r="A44" s="6" t="n">
         <ns0:v>38</ns0:v>
       </ns0:c>
@@ -1280,8 +1787,21 @@
       <ns0:c r="H44" s="6" t="str">
         <ns0:v>https://restaurantguru.com/Milan-Di-Damao-Leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="45" ht="66" customHeight="1">
+      <ns0:c r="I44" s="6" t="str">
+        <ns0:v>Searchable nasta, chai and Indo-Chinese dish references
+Copyable ask list with visit day, time of day and availability questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J44" s="6" t="str">
+        <ns0:v>Help visitors ask about the dishes they have seen without assuming they are available today.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K44" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Milan Di Damao. it includes searchable nasta, chai and Indo-Chinese dish references and copyable ask list with visit day, time of day and availability questions. the idea is to help visitors ask about the dishes they have seen without assuming they are available today. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L44" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="45" ht="150" customHeight="1">
       <ns0:c r="A45" s="6" t="n">
         <ns0:v>39</ns0:v>
       </ns0:c>
@@ -1304,8 +1824,22 @@
       <ns0:c r="H45" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/beautylicious-braunstone-town-edward-avenue-wkuhuibt</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="46" ht="66" customHeight="1">
+      <ns0:c r="I45" s="6" t="str">
+        <ns0:v>Service selector including Eyebrows · threading and Eyebrows · waxing
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J45" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K45" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Beautylicious. visitors can compare options such as Eyebrows · threading and Eyebrows · waxing, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L45" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="46" ht="150" customHeight="1">
       <ns0:c r="A46" s="6" t="n">
         <ns0:v>40</ns0:v>
       </ns0:c>
@@ -1328,8 +1862,22 @@
       <ns0:c r="H46" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/queen-lashes-leicester-70-burnham-drive-ed7gqg00</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="47" ht="66" customHeight="1">
+      <ns0:c r="I46" s="6" t="str">
+        <ns0:v>Service selector including Russian Infills and Classic Full Set
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J46" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K46" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Queen Lashes. visitors can compare options such as Russian Infills and Classic Full Set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L46" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="47" ht="150" customHeight="1">
       <ns0:c r="A47" s="6" t="n">
         <ns0:v>41</ns0:v>
       </ns0:c>
@@ -1348,8 +1896,21 @@
       <ns0:c r="F47" s="6" t="str"/>
       <ns0:c r="G47" s="6" t="str"/>
       <ns0:c r="H47" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="48" ht="66" customHeight="1">
+      <ns0:c r="I47" s="6" t="str">
+        <ns0:v>Menswear and womenswear browsing choices
+Casual or formal preferences with a copyable visit shortlist</ns0:v>
+      </ns0:c>
+      <ns0:c r="J47" s="6" t="str">
+        <ns0:v>Help shoppers describe the kind of outfit they are looking for.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K47" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for RKD. it includes menswear and womenswear browsing choices and casual or formal preferences with a copyable visit shortlist. the idea is to help shoppers describe the kind of outfit they are looking for. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L47" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="48" ht="150" customHeight="1">
       <ns0:c r="A48" s="6" t="n">
         <ns0:v>42</ns0:v>
       </ns0:c>
@@ -1372,8 +1933,21 @@
       <ns0:c r="H48" s="6" t="str">
         <ns0:v>https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d32682565-Reviews-Super_Game_Shack_Level_2-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="49" ht="66" customHeight="1">
+      <ns0:c r="I48" s="6" t="str">
+        <ns0:v>Arcade, café and shop visit guide
+Copyable list of activities to explore</ns0:v>
+      </ns0:c>
+      <ns0:c r="J48" s="6" t="str">
+        <ns0:v>Help visitors plan a trip that combines gaming, a café stop and browsing.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K48" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Super Game Shack Level 2. it includes arcade, café and shop visit guide and copyable list of activities to explore. the idea is to help visitors plan a trip that combines gaming, a café stop and browsing. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L48" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="49" ht="150" customHeight="1">
       <ns0:c r="A49" s="6" t="n">
         <ns0:v>43</ns0:v>
       </ns0:c>
@@ -1396,8 +1970,21 @@
       <ns0:c r="H49" s="6" t="str">
         <ns0:v>https://leicester.cylex-uk.co.uk/company/bradgate-lace-26489325.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="50" ht="66" customHeight="1">
+      <ns0:c r="I49" s="6" t="str">
+        <ns0:v>Window measurement notes with room labels and centimetre or inch units
+Multiple window entries with edit, copy and print controls</ns0:v>
+      </ns0:c>
+      <ns0:c r="J49" s="6" t="str">
+        <ns0:v>Help customers bring organised measurements and questions into the shop.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K49" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Bradgate Lace. it includes window measurement notes with room labels and centimetre or inch units and multiple window entries with edit, copy and print controls. the idea is to help customers bring organised measurements and questions into the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L49" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="50" ht="150" customHeight="1">
       <ns0:c r="A50" s="6" t="n">
         <ns0:v>44</ns0:v>
       </ns0:c>
@@ -1420,8 +2007,21 @@
       <ns0:c r="H50" s="6" t="str">
         <ns0:v>https://www.bizseek.co.uk/humberstone-mobile-satellite-tv-centre-07849-027337</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="51" ht="66" customHeight="1">
+      <ns0:c r="I50" s="6" t="str">
+        <ns0:v>Phone make, model and fault enquiry guide
+Copyable repair discussion notes</ns0:v>
+      </ns0:c>
+      <ns0:c r="J50" s="6" t="str">
+        <ns0:v>Help customers describe a screen, charging or camera problem before contacting the shop.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K50" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Humberstone Mobile. it includes phone make, model and fault enquiry guide and copyable repair discussion notes. the idea is to help customers describe a screen, charging or camera problem before contacting the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L50" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="51" ht="150" customHeight="1">
       <ns0:c r="A51" s="6" t="n">
         <ns0:v>45</ns0:v>
       </ns0:c>
@@ -1444,8 +2044,21 @@
       <ns0:c r="H51" s="6" t="str">
         <ns0:v>https://firmania.co.uk/leicester/kicheri-6475799</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="52" ht="66" customHeight="1">
+      <ns0:c r="I51" s="6" t="str">
+        <ns0:v>Searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks
+Food photograph views and an existing Uber Eats link</ns0:v>
+      </ns0:c>
+      <ns0:c r="J51" s="6" t="str">
+        <ns0:v>Help customers find a relevant lunch choice before visiting or opening the ordering provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K51" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Kicheri. it includes searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks and food photograph views and an existing Uber Eats link. the idea is to help customers find a relevant lunch choice before visiting or opening the ordering provider. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L51" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="52" ht="150" customHeight="1">
       <ns0:c r="A52" s="6" t="n">
         <ns0:v>46</ns0:v>
       </ns0:c>
@@ -1464,8 +2077,22 @@
       <ns0:c r="F52" s="6" t="str"/>
       <ns0:c r="G52" s="6" t="str"/>
       <ns0:c r="H52" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="53" ht="66" customHeight="1">
+      <ns0:c r="I52" s="6" t="str">
+        <ns0:v>Service selector including BIAB Manicure and Gel Manicure
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J52" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K52" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for By.meadowmae. visitors can compare options such as BIAB Manicure and Gel Manicure, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L52" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="53" ht="150" customHeight="1">
       <ns0:c r="A53" s="6" t="n">
         <ns0:v>47</ns0:v>
       </ns0:c>
@@ -1484,8 +2111,22 @@
       <ns0:c r="F53" s="6" t="str"/>
       <ns0:c r="G53" s="6" t="str"/>
       <ns0:c r="H53" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="54" ht="66" customHeight="1">
+      <ns0:c r="I53" s="6" t="str">
+        <ns0:v>Service selector including Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J53" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K53" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Cargo Male Grooming. visitors can compare options such as Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L53" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="54" ht="150" customHeight="1">
       <ns0:c r="A54" s="6" t="n">
         <ns0:v>48</ns0:v>
       </ns0:c>
@@ -1511,8 +2152,21 @@
         <ns0:v>https://wanderlog.com/place/details/1430416/cafe-dido
 https://www.yell.com/biz/cafe-dido-leicester-6484595/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="55" ht="66" customHeight="1">
+      <ns0:c r="I54" s="6" t="str">
+        <ns0:v>Visit planner for breakfast, lunch or a drink break
+Question list for dates, group size, outdoor seating and access</ns0:v>
+      </ns0:c>
+      <ns0:c r="J54" s="6" t="str">
+        <ns0:v>Help visitors organise their café questions before calling.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K54" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Cade Dido. it includes visit planner for breakfast, lunch or a drink break and question list for dates, group size, outdoor seating and access. the idea is to help visitors organise their café questions before calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L54" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="55" ht="150" customHeight="1">
       <ns0:c r="A55" s="6" t="n">
         <ns0:v>49</ns0:v>
       </ns0:c>
@@ -1535,8 +2189,22 @@
       <ns0:c r="H55" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/grace-hairstylist-leicester-browns-107-clarendon-park-road-w3ytcuxn</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="56" ht="66" customHeight="1">
+      <ns0:c r="I55" s="6" t="str">
+        <ns0:v>Service selector including Ladies Cut &amp; Finish and Blow dry
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J55" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K55" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Grace Hairstylist. visitors can compare options such as Ladies Cut &amp; Finish and Blow dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L55" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="56" ht="150" customHeight="1">
       <ns0:c r="A56" s="6" t="n">
         <ns0:v>50</ns0:v>
       </ns0:c>
@@ -1559,8 +2227,22 @@
       <ns0:c r="H56" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/joshs-hair-hideaway-leicester-uk-39-courtenay-road-r4zvys8z</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="57" ht="66" customHeight="1">
+      <ns0:c r="I56" s="6" t="str">
+        <ns0:v>Service selector including Cut &amp; Finish and Gents Cut &amp; Finish
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J56" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K56" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Josh’s Hair Hideaway. visitors can compare options such as Cut &amp; Finish and Gents Cut &amp; Finish, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L56" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="57" ht="150" customHeight="1">
       <ns0:c r="A57" s="6" t="n">
         <ns0:v>51</ns0:v>
       </ns0:c>
@@ -1583,8 +2265,22 @@
       <ns0:c r="H57" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/pretty-suite-by-abbie-leicester-hill-rise-tw0ac4s3</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="58" ht="66" customHeight="1">
+      <ns0:c r="I57" s="6" t="str">
+        <ns0:v>Service selector including 30 min Mini fill and Brow wax and tint
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J57" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K57" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Pretty Suite by Abbie. visitors can compare options such as 30 min Mini fill and Brow wax and tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L57" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="58" ht="150" customHeight="1">
       <ns0:c r="A58" s="6" t="n">
         <ns0:v>52</ns0:v>
       </ns0:c>
@@ -1607,8 +2303,21 @@
       <ns0:c r="H58" s="6" t="str">
         <ns0:v>https://haymarketshoppingcentre.com/stores/haymarket-kiosk.php</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="59" ht="66" customHeight="1">
+      <ns0:c r="I58" s="6" t="str">
+        <ns0:v>Guide to snacks, newspapers, mobile top-ups and bill services
+Visit checklist with questions for the selected services</ns0:v>
+      </ns0:c>
+      <ns0:c r="J58" s="6" t="str">
+        <ns0:v>Help shoppers check what they need from the kiosk before making a trip.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K58" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Haymarket Kiosk. it includes guide to snacks, newspapers, mobile top-ups and bill services and visit checklist with questions for the selected services. the idea is to help shoppers check what they need from the kiosk before making a trip. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L58" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="59" ht="150" customHeight="1">
       <ns0:c r="A59" s="6" t="n">
         <ns0:v>53</ns0:v>
       </ns0:c>
@@ -1631,8 +2340,22 @@
       <ns0:c r="H59" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/aimee-charlotte-beauty-anstey-megslashes-37-the-nook-c4dfe1bt</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="60" ht="66" customHeight="1">
+      <ns0:c r="I59" s="6" t="str">
+        <ns0:v>Service selector including Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J59" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K59" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Aimee Charlotte Beauty. visitors can compare options such as Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L59" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="60" ht="150" customHeight="1">
       <ns0:c r="A60" s="6" t="n">
         <ns0:v>54</ns0:v>
       </ns0:c>
@@ -1655,8 +2378,22 @@
       <ns0:c r="H60" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/anelita-beauty-leicester-30a-blaby-road-y1gkfn59</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="61" ht="66" customHeight="1">
+      <ns0:c r="I60" s="6" t="str">
+        <ns0:v>Service selector including LVL Lash Lift and Individual eyelash extensions - Full set
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J60" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K60" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Anelita Beauty. visitors can compare options such as LVL Lash Lift and Individual eyelash extensions - Full set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L60" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="61" ht="150" customHeight="1">
       <ns0:c r="A61" s="6" t="n">
         <ns0:v>55</ns0:v>
       </ns0:c>
@@ -1679,8 +2416,22 @@
       <ns0:c r="H61" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/hair-by-tia-leicester-uk-100-lorne-road-glbzje22</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="62" ht="66" customHeight="1">
+      <ns0:c r="I61" s="6" t="str">
+        <ns0:v>Service selector including Hair up and Tapes Half head Maintenance
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J61" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K61" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Hair by Tia. visitors can compare options such as Hair up and Tapes Half head Maintenance, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L61" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="62" ht="150" customHeight="1">
       <ns0:c r="A62" s="6" t="n">
         <ns0:v>56</ns0:v>
       </ns0:c>
@@ -1703,8 +2454,21 @@
       <ns0:c r="H62" s="6" t="str">
         <ns0:v>https://www.cybo.com/GB-biz/international-food-centre_24f</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="63" ht="66" customHeight="1">
+      <ns0:c r="I62" s="6" t="str">
+        <ns0:v>Produce, grocery and fresh bread category guide
+Copyable shopping interests list</ns0:v>
+      </ns0:c>
+      <ns0:c r="J62" s="6" t="str">
+        <ns0:v>Help customers organise the parts of their shop they want to ask about.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K62" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for International Food Centre. it includes produce, grocery and fresh bread category guide and copyable shopping interests list. the idea is to help customers organise the parts of their shop they want to ask about. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L62" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="63" ht="150" customHeight="1">
       <ns0:c r="A63" s="6" t="n">
         <ns0:v>57</ns0:v>
       </ns0:c>
@@ -1727,8 +2491,21 @@
       <ns0:c r="H63" s="6" t="str">
         <ns0:v>https://visitleicester.info/point-of-interest/the-good-earth/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="64" ht="66" customHeight="1">
+      <ns0:c r="I63" s="6" t="str">
+        <ns0:v>Vegetarian dish examples grouped by comfort food and soup
+Café photograph viewer and Free Lane visit information</ns0:v>
+      </ns0:c>
+      <ns0:c r="J63" s="6" t="str">
+        <ns0:v>Give visitors a feel for the cooking and help them recognise the café.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K63" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for The Good Earth. it includes vegetarian dish examples grouped by comfort food and soup and café photograph viewer and Free Lane visit information. the idea is to give visitors a feel for the cooking and help them recognise the café. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L63" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="64" ht="150" customHeight="1">
       <ns0:c r="A64" s="6" t="n">
         <ns0:v>58</ns0:v>
       </ns0:c>
@@ -1747,8 +2524,21 @@
       <ns0:c r="F64" s="6" t="str"/>
       <ns0:c r="G64" s="6" t="str"/>
       <ns0:c r="H64" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="65" ht="66" customHeight="1">
+      <ns0:c r="I64" s="6" t="str">
+        <ns0:v>Fruit, meat and chicken, and bread category choices
+Copyable shopping note</ns0:v>
+      </ns0:c>
+      <ns0:c r="J64" s="6" t="str">
+        <ns0:v>Help customers bring together the items they want to discuss in the shop.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K64" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Leicester Fresh Food. it includes fruit, meat and chicken, and bread category choices and copyable shopping note. the idea is to help customers bring together the items they want to discuss in the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L64" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="65" ht="150" customHeight="1">
       <ns0:c r="A65" s="6" t="n">
         <ns0:v>59</ns0:v>
       </ns0:c>
@@ -1771,8 +2561,21 @@
       <ns0:c r="H65" s="6" t="str">
         <ns0:v>https://firmania.co.uk/leicester/soi52-thai-therapy-5103243</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="66" ht="66" customHeight="1">
+      <ns0:c r="I65" s="6" t="str">
+        <ns0:v>Treatment information and Church Gate location details
+Links to the existing business website and directions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J65" s="6" t="str">
+        <ns0:v>Give people a clear starting point for asking about treatments and planning a visit.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K65" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Soi 52. it includes treatment information and Church Gate location details and links to the existing business website and directions. the idea is to give people a clear starting point for asking about treatments and planning a visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L65" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="66" ht="150" customHeight="1">
       <ns0:c r="A66" s="6" t="n">
         <ns0:v>60</ns0:v>
       </ns0:c>
@@ -1791,8 +2594,22 @@
       <ns0:c r="F66" s="6" t="str"/>
       <ns0:c r="G66" s="6" t="str"/>
       <ns0:c r="H66" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="67" ht="66" customHeight="1">
+      <ns0:c r="I66" s="6" t="str">
+        <ns0:v>Service selector including Wash Cut &amp; Blowdry and Signature Blowout
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J66" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K66" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Soie Hair. visitors can compare options such as Wash Cut &amp; Blowdry and Signature Blowout, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L66" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="67" ht="150" customHeight="1">
       <ns0:c r="A67" s="6" t="n">
         <ns0:v>61</ns0:v>
       </ns0:c>
@@ -1815,8 +2632,22 @@
       <ns0:c r="H67" s="6" t="str">
         <ns0:v>https://www.instagram.com/star_barbers_oadby/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="68" ht="66" customHeight="1">
+      <ns0:c r="I67" s="6" t="str">
+        <ns0:v>Service selector including Hair cut and Skin fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J67" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K67" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Star Barbers Oadby. visitors can compare options such as Hair cut and Skin fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L67" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="68" ht="150" customHeight="1">
       <ns0:c r="A68" s="6" t="n">
         <ns0:v>62</ns0:v>
       </ns0:c>
@@ -1835,8 +2666,22 @@
       <ns0:c r="F68" s="6" t="str"/>
       <ns0:c r="G68" s="6" t="str"/>
       <ns0:c r="H68" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="69" ht="66" customHeight="1">
+      <ns0:c r="I68" s="6" t="str">
+        <ns0:v>Service selector including Skin fade and Taper fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J68" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K68" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for M K BARBER. visitors can compare options such as Skin fade and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L68" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="69" ht="150" customHeight="1">
       <ns0:c r="A69" s="6" t="n">
         <ns0:v>63</ns0:v>
       </ns0:c>
@@ -1855,8 +2700,21 @@
       <ns0:c r="F69" s="6" t="str"/>
       <ns0:c r="G69" s="6" t="str"/>
       <ns0:c r="H69" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="70" ht="66" customHeight="1">
+      <ns0:c r="I69" s="6" t="str">
+        <ns0:v>Coffee, specials and açaí menu filters
+Four-topping açaí bowl outline builder</ns0:v>
+      </ns0:c>
+      <ns0:c r="J69" s="6" t="str">
+        <ns0:v>Let visitors explore a bowl combination before checking the existing ordering options.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K69" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Alcove. it includes coffee, specials and açaí menu filters and four-topping açaí bowl outline builder. the idea is to let visitors explore a bowl combination before checking the existing ordering options. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L69" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="70" ht="150" customHeight="1">
       <ns0:c r="A70" s="6" t="n">
         <ns0:v>64</ns0:v>
       </ns0:c>
@@ -1875,8 +2733,22 @@
       <ns0:c r="F70" s="6" t="str"/>
       <ns0:c r="G70" s="6" t="str"/>
       <ns0:c r="H70" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="71" ht="66" customHeight="1">
+      <ns0:c r="I70" s="6" t="str">
+        <ns0:v>Service selector including Gents Haircut and Skin Fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J70" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K70" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for The Mane Room Leicester. visitors can compare options such as Gents Haircut and Skin Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L70" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="71" ht="150" customHeight="1">
       <ns0:c r="A71" s="6" t="n">
         <ns0:v>65</ns0:v>
       </ns0:c>
@@ -1895,8 +2767,22 @@
       <ns0:c r="F71" s="6" t="str"/>
       <ns0:c r="G71" s="6" t="str"/>
       <ns0:c r="H71" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="72" ht="66" customHeight="1">
+      <ns0:c r="I71" s="6" t="str">
+        <ns0:v>Service selector including Gents Haircut and Skin or Zero Fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J71" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K71" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Mancave Barber Lounge. visitors can compare options such as Gents Haircut and Skin or Zero Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L71" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="72" ht="150" customHeight="1">
       <ns0:c r="A72" s="6" t="n">
         <ns0:v>66</ns0:v>
       </ns0:c>
@@ -1919,8 +2805,22 @@
       <ns0:c r="H72" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/11-11-studios-leicester-10-turville-road-d3i3gen7</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="73" ht="66" customHeight="1">
+      <ns0:c r="I72" s="6" t="str">
+        <ns0:v>Service selector including BIAB overlay and BIAB infill
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J72" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K72" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for 11:11 Studios. visitors can compare options such as BIAB overlay and BIAB infill, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L72" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="73" ht="150" customHeight="1">
       <ns0:c r="A73" s="6" t="n">
         <ns0:v>67</ns0:v>
       </ns0:c>
@@ -1943,8 +2843,22 @@
       <ns0:c r="H73" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/mphair-glenfield-102-dominion-road-dixl6g64</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="74" ht="66" customHeight="1">
+      <ns0:c r="I73" s="6" t="str">
+        <ns0:v>Service selector including Ladies Cut and Blow dry and Gents cut no wash
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J73" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K73" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for MPHair. visitors can compare options such as Ladies Cut and Blow dry and Gents cut no wash, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L73" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="74" ht="150" customHeight="1">
       <ns0:c r="A74" s="6" t="n">
         <ns0:v>68</ns0:v>
       </ns0:c>
@@ -1968,8 +2882,22 @@
         <ns0:v>https://www.fresha.com/a/be-beautiful-by-alex-glenfield-stamford-street-li3z5jdq
 https://www.facebook.com/p/Be-beautiful-by-Alex-100063692222493/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="75" ht="66" customHeight="1">
+      <ns0:c r="I74" s="6" t="str">
+        <ns0:v>Service selector including BIAB Infill and Eyebrow shape &amp; Tint
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J74" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K74" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Be beautiful by Alex. visitors can compare options such as BIAB Infill and Eyebrow shape &amp; Tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L74" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="75" ht="150" customHeight="1">
       <ns0:c r="A75" s="6" t="n">
         <ns0:v>69</ns0:v>
       </ns0:c>
@@ -1992,8 +2920,22 @@
       <ns0:c r="H75" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/graced-by-helen-leicester-aadams-apartments-uk-20-frog-island-b5u60lzv</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="76" ht="66" customHeight="1">
+      <ns0:c r="I75" s="6" t="str">
+        <ns0:v>Service selector including Knotless/Box Braids and Make-up (For Occasions)
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J75" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K75" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Graced by Helen. visitors can compare options such as Knotless/Box Braids and Make-up (For Occasions), see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L75" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="76" ht="150" customHeight="1">
       <ns0:c r="A76" s="6" t="n">
         <ns0:v>70</ns0:v>
       </ns0:c>
@@ -2019,8 +2961,21 @@
         <ns0:v>https://www.leicester.co.uk/listing/24804/
 https://wanderlog.com/place/details/3943590/the-pot-pourri-shop-leicester</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="77" ht="66" customHeight="1">
+      <ns0:c r="I76" s="6" t="str">
+        <ns0:v>Gift brief built around occasion and shopping interest
+Optional budget selection and a copyable summary</ns0:v>
+      </ns0:c>
+      <ns0:c r="J76" s="6" t="str">
+        <ns0:v>Help shoppers explain a birthday, thank-you or just-because gift idea.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K76" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Pot Pourri Shop. it includes gift brief built around occasion and shopping interest and optional budget selection and a copyable summary. the idea is to help shoppers explain a birthday, thank-you or just-because gift idea. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L76" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="77" ht="150" customHeight="1">
       <ns0:c r="A77" s="6" t="n">
         <ns0:v>71</ns0:v>
       </ns0:c>
@@ -2043,8 +2998,21 @@
       <ns0:c r="H77" s="6" t="str">
         <ns0:v>https://www.bestsalons.com/uk/leicester/nails</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="78" ht="66" customHeight="1">
+      <ns0:c r="I77" s="6" t="str">
+        <ns0:v>Nail inspiration choices from the salon gallery
+Call note combining the chosen look with preferred nail length</ns0:v>
+      </ns0:c>
+      <ns0:c r="J77" s="6" t="str">
+        <ns0:v>Help clients describe the finish they have in mind before speaking to the salon.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K77" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for London Nails. it includes nail inspiration choices from the salon gallery and call note combining the chosen look with preferred nail length. the idea is to help clients describe the finish they have in mind before speaking to the salon. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L77" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="78" ht="150" customHeight="1">
       <ns0:c r="A78" s="6" t="n">
         <ns0:v>72</ns0:v>
       </ns0:c>
@@ -2068,8 +3036,22 @@
         <ns0:v>https://www.fresha.com/a/tiegan-seaton-seats-hair-studio-anstey-4b-cropston-road-mozb3qoa
 https://www.facebook.com/people/Seats-Hair-Studio/61566781924188/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="79" ht="66" customHeight="1">
+      <ns0:c r="I78" s="6" t="str">
+        <ns0:v>Service selector including Restyle and Patch test &amp; consultation
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J78" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K78" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Tiegan Seaton (Seats Hair Studio). visitors can compare options such as Restyle and Patch test &amp; consultation, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L78" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="79" ht="150" customHeight="1">
       <ns0:c r="A79" s="6" t="n">
         <ns0:v>73</ns0:v>
       </ns0:c>
@@ -2092,8 +3074,22 @@
       <ns0:c r="H79" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/royalty-trimz-leicester-40-church-gate-xkxfpy1l</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="80" ht="66" customHeight="1">
+      <ns0:c r="I79" s="6" t="str">
+        <ns0:v>Service selector including Shape up and Haircut
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J79" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K79" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Royalty Trimz. visitors can compare options such as Shape up and Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L79" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="80" ht="150" customHeight="1">
       <ns0:c r="A80" s="6" t="n">
         <ns0:v>74</ns0:v>
       </ns0:c>
@@ -2116,8 +3112,22 @@
       <ns0:c r="H80" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/hair-muse-leicester-247-clarendon-park-road-lqtsyymq</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="81" ht="66" customHeight="1">
+      <ns0:c r="I80" s="6" t="str">
+        <ns0:v>Service selector including Ladies Cut &amp; Blowdry and Long Hair Blowdry
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J80" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K80" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Hair Muse. visitors can compare options such as Ladies Cut &amp; Blowdry and Long Hair Blowdry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L80" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="81" ht="150" customHeight="1">
       <ns0:c r="A81" s="6" t="n">
         <ns0:v>75</ns0:v>
       </ns0:c>
@@ -2140,8 +3150,22 @@
       <ns0:c r="H81" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/autofaders-ltd-where-style-meets-precision-leicester-8c-devana-road-nxj56jn6</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="82" ht="66" customHeight="1">
+      <ns0:c r="I81" s="6" t="str">
+        <ns0:v>Service selector including Haircut · Senior barber and Haircut &amp; Beard · Senior barber
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J81" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K81" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Autofaders. visitors can compare options such as Haircut · Senior barber and Haircut &amp; Beard · Senior barber, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L81" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="82" ht="150" customHeight="1">
       <ns0:c r="A82" s="6" t="n">
         <ns0:v>76</ns0:v>
       </ns0:c>
@@ -2165,8 +3189,22 @@
         <ns0:v>https://www.fresha.com/a/glamupwithester-leicester-airborne-rn00zt24
 https://www.instagram.com/glamupwithester/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="83" ht="66" customHeight="1">
+      <ns0:c r="I82" s="6" t="str">
+        <ns0:v>Service selector including Makeup and Prom makeup
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J82" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K82" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for GlamUpWithEster. visitors can compare options such as Makeup and Prom makeup, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L82" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="83" ht="150" customHeight="1">
       <ns0:c r="A83" s="6" t="n">
         <ns0:v>77</ns0:v>
       </ns0:c>
@@ -2185,8 +3223,22 @@
       <ns0:c r="F83" s="6" t="str"/>
       <ns0:c r="G83" s="6" t="str"/>
       <ns0:c r="H83" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="84" ht="66" customHeight="1">
+      <ns0:c r="I83" s="6" t="str">
+        <ns0:v>Service selector including Builder Gel Infills and Acrylic Nails
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J83" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K83" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Mercy Nails. visitors can compare options such as Builder Gel Infills and Acrylic Nails, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L83" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="84" ht="150" customHeight="1">
       <ns0:c r="A84" s="6" t="n">
         <ns0:v>78</ns0:v>
       </ns0:c>
@@ -2210,8 +3262,22 @@
         <ns0:v>https://www.fresha.com/a/sapphire-treatments-leicester-vsa5bzok
 https://www.facebook.com/sapphiretreatments/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="85" ht="66" customHeight="1">
+      <ns0:c r="I84" s="6" t="str">
+        <ns0:v>Service selector including Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J84" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K84" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Sapphire Treatments. visitors can compare options such as Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L84" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="85" ht="150" customHeight="1">
       <ns0:c r="A85" s="6" t="n">
         <ns0:v>79</ns0:v>
       </ns0:c>
@@ -2235,8 +3301,22 @@
         <ns0:v>https://www.fresha.com/a/sambrayhair-thurmaston-uk-church-hill-road-w5hi6pp2
 https://www.facebook.com/people/Sambrayhair/61550635373315/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="86" ht="66" customHeight="1">
+      <ns0:c r="I85" s="6" t="str">
+        <ns0:v>Service selector including Wash Cut &amp; Blowdry and Mens Haircut
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J85" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K85" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for SamBrayHair. visitors can compare options such as Wash Cut &amp; Blowdry and Mens Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L85" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="86" ht="150" customHeight="1">
       <ns0:c r="A86" s="6" t="n">
         <ns0:v>80</ns0:v>
       </ns0:c>
@@ -2259,8 +3339,22 @@
       <ns0:c r="H86" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/jennifer-audrey-nails-beauty-leicester-thurmaston-fa8uc05k</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="87" ht="66" customHeight="1">
+      <ns0:c r="I86" s="6" t="str">
+        <ns0:v>Service selector including BIAB and BIAB Toes
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J86" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K86" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Jennifer Audrey Nails &amp; Beauty. visitors can compare options such as BIAB and BIAB Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L86" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="87" ht="150" customHeight="1">
       <ns0:c r="A87" s="6" t="n">
         <ns0:v>81</ns0:v>
       </ns0:c>
@@ -2283,8 +3377,21 @@
       <ns0:c r="H87" s="6" t="str">
         <ns0:v>https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d17150858-Reviews-Oppa-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="88" ht="66" customHeight="1">
+      <ns0:c r="I87" s="6" t="str">
+        <ns0:v>Korean dish filters covering bibimbap, bulgogi, soups and more
+Meal shortlist with table BBQ, spice and allergy questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J87" s="6" t="str">
+        <ns0:v>Help a group organise dishes and the questions they want to discuss.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K87" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Oppa Korean Restaurant. it includes korean dish filters covering bibimbap, bulgogi, soups and more and meal shortlist with table BBQ, spice and allergy questions. the idea is to help a group organise dishes and the questions they want to discuss. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L87" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="88" ht="150" customHeight="1">
       <ns0:c r="A88" s="6" t="n">
         <ns0:v>82</ns0:v>
       </ns0:c>
@@ -2308,8 +3415,21 @@
         <ns0:v>https://visitleicester.info/point-of-interest/sherwins-cheese-co/
 https://www.charlesmartell.com/retailers/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="89" ht="66" customHeight="1">
+      <ns0:c r="I88" s="6" t="str">
+        <ns0:v>Cheese and deli guide with accompaniment ideas
+Gathering question list covering guest count, flavour preferences and serving questions</ns0:v>
+      </ns0:c>
+      <ns0:c r="J88" s="6" t="str">
+        <ns0:v>Help customers ask for a cheese selection suited to their gathering.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K88" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Sherwin's Cheese Company. it includes cheese and deli guide with accompaniment ideas and gathering question list covering guest count, flavour preferences and serving questions. the idea is to help customers ask for a cheese selection suited to their gathering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L88" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="89" ht="150" customHeight="1">
       <ns0:c r="A89" s="6" t="n">
         <ns0:v>83</ns0:v>
       </ns0:c>
@@ -2332,8 +3452,21 @@
       <ns0:c r="H89" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/amic-studios-birstall-2b-stonehill-avenue-ekar337w</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="90" ht="66" customHeight="1">
+      <ns0:c r="I89" s="6" t="str">
+        <ns0:v>Service search and filters for Dan, Tate, Dom and Alfie
+Named barber service listings with the existing Fresha route</ns0:v>
+      </ns0:c>
+      <ns0:c r="J89" s="6" t="str">
+        <ns0:v>Help clients find the barber and service they want before opening the booking page.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K89" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Amic Studios. it includes service search and filters for Dan, Tate, Dom and Alfie and named barber service listings with the existing Fresha route. the idea is to help clients find the barber and service they want before opening the booking page. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L89" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="90" ht="150" customHeight="1">
       <ns0:c r="A90" s="6" t="n">
         <ns0:v>84</ns0:v>
       </ns0:c>
@@ -2356,8 +3489,22 @@
       <ns0:c r="H90" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/irl-nails-and-beauty-leicester-naver-road-mumgjpxd</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="91" ht="66" customHeight="1">
+      <ns0:c r="I90" s="6" t="str">
+        <ns0:v>Service selector including Gel polish - one colour and Removals with new set
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J90" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K90" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for IRL Nails and Beauty. visitors can compare options such as Gel polish - one colour and Removals with new set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L90" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="91" ht="150" customHeight="1">
       <ns0:c r="A91" s="6" t="n">
         <ns0:v>85</ns0:v>
       </ns0:c>
@@ -2380,8 +3527,22 @@
       <ns0:c r="H91" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/hair-by-wikki-leicester-50a-hinckley-road-mtq61cm7</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="92" ht="66" customHeight="1">
+      <ns0:c r="I91" s="6" t="str">
+        <ns0:v>Service selector including Ladies Cut &amp; Blow Dry and Gents Cut
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J91" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K91" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Hair By Wikki. visitors can compare options such as Ladies Cut &amp; Blow Dry and Gents Cut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L91" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="92" ht="150" customHeight="1">
       <ns0:c r="A92" s="6" t="n">
         <ns0:v>86</ns0:v>
       </ns0:c>
@@ -2400,8 +3561,21 @@
       <ns0:c r="F92" s="6" t="str"/>
       <ns0:c r="G92" s="6" t="str"/>
       <ns0:c r="H92" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="93" ht="66" customHeight="1">
+      <ns0:c r="I92" s="6" t="str">
+        <ns0:v>Searchable menu selection with burger, wrap, pizza and grill filters
+Existing Deliveroo link alongside location information</ns0:v>
+      </ns0:c>
+      <ns0:c r="J92" s="6" t="str">
+        <ns0:v>Help customers find a meal category quickly before checking the ordering menu.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K92" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for LALA’S Restaurant. it includes searchable menu selection with burger, wrap, pizza and grill filters and existing Deliveroo link alongside location information. the idea is to help customers find a meal category quickly before checking the ordering menu. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L92" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="93" ht="150" customHeight="1">
       <ns0:c r="A93" s="6" t="n">
         <ns0:v>87</ns0:v>
       </ns0:c>
@@ -2420,8 +3594,22 @@
       <ns0:c r="F93" s="6" t="str"/>
       <ns0:c r="G93" s="6" t="str"/>
       <ns0:c r="H93" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="94" ht="66" customHeight="1">
+      <ns0:c r="I93" s="6" t="str">
+        <ns0:v>Service selector including Cut and Finish and Cut and Finish w/ Beard Trim
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J93" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K93" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for VOSS. Barbering and Men’s Hair Specialist. visitors can compare options such as Cut and Finish and Cut and Finish w/ Beard Trim, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L93" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="94" ht="150" customHeight="1">
       <ns0:c r="A94" s="6" t="n">
         <ns0:v>88</ns0:v>
       </ns0:c>
@@ -2440,8 +3628,21 @@
       <ns0:c r="F94" s="6" t="str"/>
       <ns0:c r="G94" s="6" t="str"/>
       <ns0:c r="H94" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="95" ht="66" customHeight="1">
+      <ns0:c r="I94" s="6" t="str">
+        <ns0:v>Searchable hot and cold mezze selection
+Existing Uber Eats link and Gallowtree Gate visit information</ns0:v>
+      </ns0:c>
+      <ns0:c r="J94" s="6" t="str">
+        <ns0:v>Help visitors explore mezze choices before ordering or visiting.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K94" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Falafelland. it includes searchable hot and cold mezze selection and existing Uber Eats link and Gallowtree Gate visit information. the idea is to help visitors explore mezze choices before ordering or visiting. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L94" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="95" ht="150" customHeight="1">
       <ns0:c r="A95" s="6" t="n">
         <ns0:v>89</ns0:v>
       </ns0:c>
@@ -2460,8 +3661,22 @@
       <ns0:c r="F95" s="6" t="str"/>
       <ns0:c r="G95" s="6" t="str"/>
       <ns0:c r="H95" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="96" ht="66" customHeight="1">
+      <ns0:c r="I95" s="6" t="str">
+        <ns0:v>Service selector including Beard Trim and Condition and Taper fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J95" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K95" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Amo’s Cutthroat. visitors can compare options such as Beard Trim and Condition and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L95" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="96" ht="150" customHeight="1">
       <ns0:c r="A96" s="6" t="n">
         <ns0:v>90</ns0:v>
       </ns0:c>
@@ -2480,8 +3695,22 @@
       <ns0:c r="F96" s="6" t="str"/>
       <ns0:c r="G96" s="6" t="str"/>
       <ns0:c r="H96" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="97" ht="66" customHeight="1">
+      <ns0:c r="I96" s="6" t="str">
+        <ns0:v>Service selector including Haircut with Martin and Haircut with Alex
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J96" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K96" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Til Next Time Barbershop. visitors can compare options such as Haircut with Martin and Haircut with Alex, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L96" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="97" ht="150" customHeight="1">
       <ns0:c r="A97" s="6" t="n">
         <ns0:v>91</ns0:v>
       </ns0:c>
@@ -2504,8 +3733,21 @@
       <ns0:c r="H97" s="6" t="str">
         <ns0:v>https://visitleicester.info/point-of-interest/karamay/</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="98" ht="66" customHeight="1">
+      <ns0:c r="I97" s="6" t="str">
+        <ns0:v>Searchable Uyghur menu across noodles, dumplings, skewers and vegetables
+Links to the existing business and ordering pages</ns0:v>
+      </ns0:c>
+      <ns0:c r="J97" s="6" t="str">
+        <ns0:v>Help diners explore unfamiliar dishes and find the next step for a visit or order.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K97" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Karamay Hot Pot. it includes searchable Uyghur menu across noodles, dumplings, skewers and vegetables and links to the existing business and ordering pages. the idea is to help diners explore unfamiliar dishes and find the next step for a visit or order. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L97" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="98" ht="150" customHeight="1">
       <ns0:c r="A98" s="6" t="n">
         <ns0:v>92</ns0:v>
       </ns0:c>
@@ -2528,8 +3770,22 @@
       <ns0:c r="H98" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/by-nancy-south-wigston-2-orange-street-vpssmvw9</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="99" ht="66" customHeight="1">
+      <ns0:c r="I98" s="6" t="str">
+        <ns0:v>Service selector including BIAB Manicure and BIAB Manicure &amp; Simple Nail Art
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J98" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K98" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for By Nancy. visitors can compare options such as BIAB Manicure and BIAB Manicure &amp; Simple Nail Art, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L98" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="99" ht="150" customHeight="1">
       <ns0:c r="A99" s="6" t="n">
         <ns0:v>93</ns0:v>
       </ns0:c>
@@ -2552,8 +3808,22 @@
       <ns0:c r="H99" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/elmaybeauty-x-wigston-hazelwood-road-suc2o819</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="100" ht="66" customHeight="1">
+      <ns0:c r="I99" s="6" t="str">
+        <ns0:v>Service selector including Double classic infill and Korean lash lift
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J99" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K99" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for elmaybeauty.x. visitors can compare options such as Double classic infill and Korean lash lift, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L99" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="100" ht="150" customHeight="1">
       <ns0:c r="A100" s="6" t="n">
         <ns0:v>94</ns0:v>
       </ns0:c>
@@ -2578,8 +3848,21 @@
       <ns0:c r="H100" s="6" t="str">
         <ns0:v>https://www.bizseek.co.uk/cafe-bruxelles-0116-253-1325</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="101" ht="66" customHeight="1">
+      <ns0:c r="I100" s="6" t="str">
+        <ns0:v>Visit checklist for a chosen date and group size
+Questions covering Belgian beers, weekend plans, access and arrival</ns0:v>
+      </ns0:c>
+      <ns0:c r="J100" s="6" t="str">
+        <ns0:v>Help groups organise what to check with the venue before a visit.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K100" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Café Bruxelles. it includes visit checklist for a chosen date and group size and questions covering Belgian beers, weekend plans, access and arrival. the idea is to help groups organise what to check with the venue before a visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L100" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="101" ht="150" customHeight="1">
       <ns0:c r="A101" s="6" t="n">
         <ns0:v>95</ns0:v>
       </ns0:c>
@@ -2603,8 +3886,21 @@
         <ns0:v>https://visitleicester.info/wp-content/uploads/2025/04/Leicester-Cafe-Directory.pdf
 https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d3485785-Reviews-Deli_Ish-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="102" ht="66" customHeight="1">
+      <ns0:c r="I101" s="6" t="str">
+        <ns0:v>Filter for vegetarian menu listings
+Item detail views across breakfast, paninis, wraps and salads</ns0:v>
+      </ns0:c>
+      <ns0:c r="J101" s="6" t="str">
+        <ns0:v>Help customers narrow down lunch options before checking ingredients and ordering.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K101" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Deliish. it includes filter for vegetarian menu listings and item detail views across breakfast, paninis, wraps and salads. the idea is to help customers narrow down lunch options before checking ingredients and ordering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L101" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="102" ht="150" customHeight="1">
       <ns0:c r="A102" s="6" t="n">
         <ns0:v>96</ns0:v>
       </ns0:c>
@@ -2623,8 +3919,22 @@
       <ns0:c r="F102" s="6" t="str"/>
       <ns0:c r="G102" s="6" t="str"/>
       <ns0:c r="H102" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="103" ht="66" customHeight="1">
+      <ns0:c r="I102" s="6" t="str">
+        <ns0:v>Service selector including Brow architecture · mapping and shaping and Lash Removal
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J102" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K102" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Ink&amp;Beauty Factory. visitors can compare options such as Brow architecture · mapping and shaping and Lash Removal, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L102" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="103" ht="150" customHeight="1">
       <ns0:c r="A103" s="6" t="n">
         <ns0:v>97</ns0:v>
       </ns0:c>
@@ -2647,8 +3957,22 @@
       <ns0:c r="H103" s="6" t="str">
         <ns0:v>https://www.fresha.com/a/shortys-leicester-leicester-hair-1rd-42-44-rutland-street-jq5wg2jp</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="104" ht="66" customHeight="1">
+      <ns0:c r="I103" s="6" t="str">
+        <ns0:v>Service selector including Haircut (Leicester) and Haircut and beard trim
+Listed prices and appointment lengths update with the selected service
+Link to the existing Fresha booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J103" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K103" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Shortys - Leicester. visitors can compare options such as Haircut (Leicester) and Haircut and beard trim, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L103" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="104" ht="150" customHeight="1">
       <ns0:c r="A104" s="6" t="n">
         <ns0:v>98</ns0:v>
       </ns0:c>
@@ -2671,8 +3995,22 @@
       <ns0:c r="H104" s="6" t="str">
         <ns0:v>https://www.visitleicester.info/dbimgs/5007%20LCC%20-%20Beauty-guide_WEB.pdf</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="105" ht="66" customHeight="1">
+      <ns0:c r="I104" s="6" t="str">
+        <ns0:v>Service selector including SkinFade and Classic Haircut
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J104" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K104" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Taurus barbers. visitors can compare options such as SkinFade and Classic Haircut, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L104" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="105" ht="150" customHeight="1">
       <ns0:c r="A105" s="6" t="n">
         <ns0:v>99</ns0:v>
       </ns0:c>
@@ -2691,8 +4029,22 @@
       <ns0:c r="F105" s="6" t="str"/>
       <ns0:c r="G105" s="6" t="str"/>
       <ns0:c r="H105" s="6" t="str"/>
-    </ns0:row>
-    <ns0:row r="106" ht="66" customHeight="1">
+      <ns0:c r="I105" s="6" t="str">
+        <ns0:v>Service selector including Haircut and Skin-Fade/Taper fade
+Listed prices and appointment lengths update with the selected service
+Link to the existing Booksy booking page</ns0:v>
+      </ns0:c>
+      <ns0:c r="J105" s="6" t="str">
+        <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K105" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Hair Roots &amp; Co. visitors can compare options such as Haircut and Skin-Fade/Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L105" s="6" t="str">
+        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="106" ht="150" customHeight="1">
       <ns0:c r="A106" s="6" t="n">
         <ns0:v>100</ns0:v>
       </ns0:c>
@@ -2711,6 +4063,19 @@
       <ns0:c r="F106" s="6" t="str"/>
       <ns0:c r="G106" s="6" t="str"/>
       <ns0:c r="H106" s="6" t="str"/>
+      <ns0:c r="I106" s="6" t="str">
+        <ns0:v>Searchable brunch selection grouped into bowls, toast, brunch and bread
+Existing ordering route and Braunstone Gate visit information</ns0:v>
+      </ns0:c>
+      <ns0:c r="J106" s="6" t="str">
+        <ns0:v>Help visitors find the kind of brunch they fancy before visiting or ordering.</ns0:v>
+      </ns0:c>
+      <ns0:c r="K106" s="6" t="str">
+        <ns0:v>i’ve put together a website preview for Ninety Six Degrees. it includes searchable brunch selection grouped into bowls, toast, brunch and bread and existing ordering route and Braunstone Gate visit information. the idea is to help visitors find the kind of brunch they fancy before visiting or ordering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+      </ns0:c>
+      <ns0:c r="L106" s="6" t="str">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+      </ns0:c>
     </ns0:row>
   </ns0:sheetData>
   <ns0:hyperlinks>
@@ -2817,7 +4182,7 @@
   </ns0:hyperlinks>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ns0:tableParts count="1">
-    <ns0:tablePart ns1:id="R00c6e047b90a459b"/>
+    <ns0:tablePart ns1:id="Ra09ae118ee1f481b"/>
   </ns0:tableParts>
 </ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
Describe actual booking, ordering and contact links in email features
</commit_message>
<xml_diff>
--- a/website-demos/business-contacts.xlsx
+++ b/website-demos/business-contacts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="R2d439c0b0b304bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="R50a44b484bd14a19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,8 +97,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BusinessContacts" displayName="BusinessContacts" ref="A6:L106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="12">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BusinessContacts" displayName="BusinessContacts" ref="A6:M106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
     <x:tableColumn id="1" name="No."/>
     <x:tableColumn id="2" name="Business name"/>
     <x:tableColumn id="3" name="Contact phone number"/>
@@ -111,6 +111,7 @@
     <x:tableColumn id="10" name="Customer benefit"/>
     <x:tableColumn id="11" name="Email paragraph"/>
     <x:tableColumn id="12" name="Demo limitations"/>
+    <x:tableColumn id="13" name="Booking and contact destinations"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -323,6 +324,7 @@
     <ns0:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
     <ns0:col min="11" max="11" width="100" hidden="0" customWidth="1"/>
     <ns0:col min="12" max="12" width="72" hidden="0" customWidth="1"/>
+    <ns0:col min="13" max="13" width="95" hidden="0" customWidth="1"/>
   </ns0:cols>
   <ns0:sheetData>
     <ns0:row r="2">
@@ -377,8 +379,11 @@
       <ns0:c r="L6" s="5" t="str">
         <ns0:v>Demo limitations</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="7" ht="150" customHeight="1">
+      <ns0:c r="M6" s="5" t="str">
+        <ns0:v>Booking and contact destinations</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7" ht="210" customHeight="1">
       <ns0:c r="A7" s="6" t="n">
         <ns0:v>1</ns0:v>
       </ns0:c>
@@ -403,19 +408,23 @@
       </ns0:c>
       <ns0:c r="I7" s="6" t="str">
         <ns0:v>Service guide for cuts, colour and occasions
-Appointment discussion notes with a preferred date</ns0:v>
+Appointment discussion notes with a preferred date
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J7" s="6" t="str">
         <ns0:v>Help visitors explain the look and appointment they have in mind before calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K7" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Andrew Leonards Hairdressing. it includes service guide for cuts, colour and occasions and appointment discussion notes with a preferred date. the idea is to help visitors explain the look and appointment they have in mind before calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Andrew Leonards Hairdressing. it includes service guide for cuts, colour and occasions and appointment discussion notes with a preferred date. the idea is to help visitors explain the look and appointment they have in mind before calling. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L7" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="8" ht="150" customHeight="1">
+      <ns0:c r="M7" s="6" t="str">
+        <ns0:v>Tap to call 01162621675: tel:01162621675</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" ht="210" customHeight="1">
       <ns0:c r="A8" s="6" t="n">
         <ns0:v>2</ns0:v>
       </ns0:c>
@@ -440,19 +449,23 @@
       </ns0:c>
       <ns0:c r="I8" s="6" t="str">
         <ns0:v>Lunch categories for sandwiches, soup and buffets
-Group lunch planner with headcount, date and dietary questions</ns0:v>
+Group lunch planner with headcount, date and dietary questions
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J8" s="6" t="str">
         <ns0:v>Make a catering conversation easier to start with the key details already together.</ns0:v>
       </ns0:c>
       <ns0:c r="K8" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Bar Sandwich. it includes lunch categories for sandwiches, soup and buffets and group lunch planner with headcount, date and dietary questions. the idea is to make a catering conversation easier to start with the key details already together. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Bar Sandwich. it includes lunch categories for sandwiches, soup and buffets and group lunch planner with headcount, date and dietary questions. the idea is to make a catering conversation easier to start with the key details already together. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L8" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="9" ht="150" customHeight="1">
+      <ns0:c r="M8" s="6" t="str">
+        <ns0:v>Tap to call 01162519770: tel:01162519770</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" ht="210" customHeight="1">
       <ns0:c r="A9" s="6" t="n">
         <ns0:v>3</ns0:v>
       </ns0:c>
@@ -480,19 +493,23 @@
       </ns0:c>
       <ns0:c r="I9" s="6" t="str">
         <ns0:v>Lunch, cake and drink category filters
-Café shortlist with item details and a copyable visit note</ns0:v>
+Café shortlist with item details and a copyable visit note
+Direct link to Deliveroo ordering menu</ns0:v>
       </ns0:c>
       <ns0:c r="J9" s="6" t="str">
         <ns0:v>Let people pick out a lunch or cake idea before visiting High Street.</ns0:v>
       </ns0:c>
       <ns0:c r="K9" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for 5 Coats. it includes lunch, cake and drink category filters and café shortlist with item details and a copyable visit note. the idea is to let people pick out a lunch or cake idea before visiting High Street. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for 5 Coats. it includes lunch, cake and drink category filters and café shortlist with item details and a copyable visit note. the idea is to let people pick out a lunch or cake idea before visiting High Street. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L9" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M9" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/5-coats-cafe-19-high-street</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10" ht="210" customHeight="1">
       <ns0:c r="A10" s="6" t="n">
         <ns0:v>4</ns0:v>
       </ns0:c>
@@ -519,19 +536,23 @@
       </ns0:c>
       <ns0:c r="I10" s="6" t="str">
         <ns0:v>Acrylic, BIAB, gel and pedicure treatment guide
-Existing product guidance, nail inspiration gallery and Booksy links</ns0:v>
+Existing product guidance, nail inspiration gallery and Booksy links
+Booking buttons open Chloe's Nails’s existing Booksy booking profile</ns0:v>
       </ns0:c>
       <ns0:c r="J10" s="6" t="str">
         <ns0:v>Help clients think through their treatment and removal questions before opening Booksy.</ns0:v>
       </ns0:c>
       <ns0:c r="K10" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Chloe's Nails. it includes acrylic, BIAB, gel and pedicure treatment guide and existing product guidance, nail inspiration gallery and Booksy links. the idea is to help clients think through their treatment and removal questions before opening Booksy. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Chloe's Nails. it includes acrylic, BIAB, gel and pedicure treatment guide and existing product guidance, nail inspiration gallery and Booksy links. the idea is to help clients think through their treatment and removal questions before opening Booksy. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L10" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M10" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/178374_chloe-nails-leicester_nail-salon_31021_leicester</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11" ht="210" customHeight="1">
       <ns0:c r="A11" s="6" t="n">
         <ns0:v>5</ns0:v>
       </ns0:c>
@@ -556,19 +577,23 @@
       </ns0:c>
       <ns0:c r="I11" s="6" t="str">
         <ns0:v>Product enquiry list with quantities across Polish deli categories
-English or Polish enquiry summaries with collection and delivery questions</ns0:v>
+English or Polish enquiry summaries with collection and delivery questions
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J11" s="6" t="str">
         <ns0:v>Help customers explain the products and quantities they want to ask the counter about.</ns0:v>
       </ns0:c>
       <ns0:c r="K11" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Tomasz Kotula Butcher. it includes product enquiry list with quantities across Polish deli categories and english or Polish enquiry summaries with collection and delivery questions. the idea is to help customers explain the products and quantities they want to ask the counter about. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Tomasz Kotula Butcher. it includes product enquiry list with quantities across Polish deli categories and english or Polish enquiry summaries with collection and delivery questions. the idea is to help customers explain the products and quantities they want to ask the counter about. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L11" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="12" ht="150" customHeight="1">
+      <ns0:c r="M11" s="6" t="str">
+        <ns0:v>Tap to call 07739709241: tel:07739709241</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="210" customHeight="1">
       <ns0:c r="A12" s="6" t="n">
         <ns0:v>6</ns0:v>
       </ns0:c>
@@ -593,19 +618,23 @@
       </ns0:c>
       <ns0:c r="I12" s="6" t="str">
         <ns0:v>Discovery guide across jewellery, crystals, clothing, gifts and incense
-Personal shopping or gift choice with a copyable visit list</ns0:v>
+Personal shopping or gift choice with a copyable visit list
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J12" s="6" t="str">
         <ns0:v>Give visitors a starting point for browsing the shop or finding a gift.</ns0:v>
       </ns0:c>
       <ns0:c r="K12" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for The Very Bazaar. it includes discovery guide across jewellery, crystals, clothing, gifts and incense and personal shopping or gift choice with a copyable visit list. the idea is to give visitors a starting point for browsing the shop or finding a gift. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for The Very Bazaar. it includes discovery guide across jewellery, crystals, clothing, gifts and incense and personal shopping or gift choice with a copyable visit list. the idea is to give visitors a starting point for browsing the shop or finding a gift. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L12" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="13" ht="150" customHeight="1">
+      <ns0:c r="M12" s="6" t="str">
+        <ns0:v>Tap to call 01162621568: tel:01162621568</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13" ht="210" customHeight="1">
       <ns0:c r="A13" s="6" t="n">
         <ns0:v>7</ns0:v>
       </ns0:c>
@@ -630,19 +659,25 @@
       </ns0:c>
       <ns0:c r="I13" s="6" t="str">
         <ns0:v>Room search and filters for single, twin, double and family options
-Bed arrangements beside links to the existing Booking.com profile</ns0:v>
+Bed arrangements beside links to the existing Booking.com profile
+Direct link to Booking.com hotel page
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J13" s="6" t="str">
         <ns0:v>Help guests compare room types before checking current dates and rates.</ns0:v>
       </ns0:c>
       <ns0:c r="K13" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Croft Hotel. it includes room search and filters for single, twin, double and family options and bed arrangements beside links to the existing Booking.com profile. the idea is to help guests compare room types before checking current dates and rates. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Croft Hotel. it includes room search and filters for single, twin, double and family options and bed arrangements beside links to the existing Booking.com profile. the idea is to help guests compare room types before checking current dates and rates. the site also links to your Booking.com page to check room availability. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L13" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M13" s="6" t="str">
+        <ns0:v>Booking.com hotel page: https://www.booking.com/hotel/gb/croft.en-gb.html
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Croft%20Hotel%203%20Stanley%20Road%20Leicester%20LE2%201RF</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="210" customHeight="1">
       <ns0:c r="A14" s="6" t="n">
         <ns0:v>8</ns0:v>
       </ns0:c>
@@ -667,19 +702,23 @@
       </ns0:c>
       <ns0:c r="I14" s="6" t="str">
         <ns0:v>Gig list searchable by artist and filterable by month
-Gig details and a visit note for group, access or ticket questions</ns0:v>
+Gig details and a visit note for group, access or ticket questions
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J14" s="6" t="str">
         <ns0:v>Help visitors find a relevant gig and organise the questions they need to ask.</ns0:v>
       </ns0:c>
       <ns0:c r="K14" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Duffy's. it includes gig list searchable by artist and filterable by month and gig details and a visit note for group, access or ticket questions. the idea is to help visitors find a relevant gig and organise the questions they need to ask. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Duffy's. it includes gig list searchable by artist and filterable by month and gig details and a visit note for group, access or ticket questions. the idea is to help visitors find a relevant gig and organise the questions they need to ask. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L14" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="15" ht="150" customHeight="1">
+      <ns0:c r="M14" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Duffys+Bar+18+Pocklingtons+Walk+Leicester+LE1+6BU</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15" ht="210" customHeight="1">
       <ns0:c r="A15" s="6" t="n">
         <ns0:v>9</ns0:v>
       </ns0:c>
@@ -705,19 +744,24 @@
       <ns0:c r="I15" s="6" t="str">
         <ns0:v>Service selector including Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Sam’s Beauty Den in Butchers Salon’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J15" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K15" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Sam’s Beauty Den in Butchers Salon. visitors can compare options such as Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Sam’s Beauty Den in Butchers Salon. visitors can compare options such as Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L15" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M15" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/sams-beauty-den-in-butchers-salon-leicester-uk-10-allandale-road-o3llsgib
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=10%20Allandale%20Road%2C%20Leicester%20LE2%202DA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16" ht="210" customHeight="1">
       <ns0:c r="A16" s="6" t="n">
         <ns0:v>10</ns0:v>
       </ns0:c>
@@ -742,19 +786,23 @@
       </ns0:c>
       <ns0:c r="I16" s="6" t="str">
         <ns0:v>Sushi, bento and ramen category filters
-Dish detail views and a copyable favourites list</ns0:v>
+Dish detail views and a copyable favourites list
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J16" s="6" t="str">
         <ns0:v>Help diners put a few Japanese dishes together before their visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K16" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Mitsuki. it includes sushi, bento and ramen category filters and dish detail views and a copyable favourites list. the idea is to help diners put a few Japanese dishes together before their visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Mitsuki. it includes sushi, bento and ramen category filters and dish detail views and a copyable favourites list. the idea is to help diners put a few Japanese dishes together before their visit. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L16" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="17" ht="150" customHeight="1">
+      <ns0:c r="M16" s="6" t="str">
+        <ns0:v>Tap to call 01162554805: tel:01162554805</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17" ht="210" customHeight="1">
       <ns0:c r="A17" s="6" t="n">
         <ns0:v>11</ns0:v>
       </ns0:c>
@@ -779,19 +827,27 @@
       </ns0:c>
       <ns0:c r="I17" s="6" t="str">
         <ns0:v>Sharing platter guide organised by group size
-Meal discussion note with food choice, guest count and preferred date</ns0:v>
+Meal discussion note with food choice, guest count and preferred date
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J17" s="6" t="str">
         <ns0:v>Help groups decide what to ask about before speaking to the restaurant.</ns0:v>
       </ns0:c>
       <ns0:c r="K17" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Kurda Restaurant. it includes sharing platter guide organised by group size and meal discussion note with food choice, guest count and preferred date. the idea is to help groups decide what to ask about before speaking to the restaurant. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Kurda Restaurant. it includes sharing platter guide organised by group size and meal discussion note with food choice, guest count and preferred date. the idea is to help groups decide what to ask about before speaking to the restaurant. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L17" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M17" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/kurda-restaurant-10-12-humberstone-road
+Tap to call +447459948776: tel:+447459948776
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Kurda+Restaurant+10-12+Humberstone+Road+Leicester+LE5+0AR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18" ht="210" customHeight="1">
       <ns0:c r="A18" s="6" t="n">
         <ns0:v>12</ns0:v>
       </ns0:c>
@@ -817,19 +873,27 @@
       </ns0:c>
       <ns0:c r="I18" s="6" t="str">
         <ns0:v>Menu sections with dish photographs
-Event enquiry outline covering occasion, guests, food and collection preferences</ns0:v>
+Event enquiry outline covering occasion, guests, food and collection preferences
+Direct link to Tatra table request page
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J18" s="6" t="str">
         <ns0:v>Make it easier to start a conversation about a celebration or catering enquiry.</ns0:v>
       </ns0:c>
       <ns0:c r="K18" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Tatra Eastern Corner. it includes menu sections with dish photographs and event enquiry outline covering occasion, guests, food and collection preferences. the idea is to make it easier to start a conversation about a celebration or catering enquiry. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Tatra Eastern Corner. it includes menu sections with dish photographs and event enquiry outline covering occasion, guests, food and collection preferences. the idea is to make it easier to start a conversation about a celebration or catering enquiry. the site also links to your existing table request page. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L18" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M18" s="6" t="str">
+        <ns0:v>Tatra table request page: https://tatraleicester.co.uk/reservations/
+Tap to call +447883518180: tel:+447883518180
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Tatra+Eastern+Corner+1+Newport+Place+Leicester+LE1+1DL</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19" ht="210" customHeight="1">
       <ns0:c r="A19" s="6" t="n">
         <ns0:v>13</ns0:v>
       </ns0:c>
@@ -856,19 +920,25 @@
       </ns0:c>
       <ns0:c r="I19" s="6" t="str">
         <ns0:v>Daily versus weekly and monthly meal sections
-Catering brief with occasion, date, guest count, location and dietary requests</ns0:v>
+Catering brief with occasion, date, guest count, location and dietary requests
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J19" s="6" t="str">
         <ns0:v>Bring the important event details together before a catering conversation.</ns0:v>
       </ns0:c>
       <ns0:c r="K19" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for PALYA'S Catering. it includes daily versus weekly and monthly meal sections and catering brief with occasion, date, guest count, location and dietary requests. the idea is to bring the important event details together before a catering conversation. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for PALYA'S Catering. it includes daily versus weekly and monthly meal sections and catering brief with occasion, date, guest count, location and dietary requests. the idea is to bring the important event details together before a catering conversation. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L19" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M19" s="6" t="str">
+        <ns0:v>Tap to call +447955266135: tel:+447955266135
+Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/evington-valley/palyas-catering-74-conduit-street</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20" ht="210" customHeight="1">
       <ns0:c r="A20" s="6" t="n">
         <ns0:v>14</ns0:v>
       </ns0:c>
@@ -893,19 +963,27 @@
       </ns0:c>
       <ns0:c r="I20" s="6" t="str">
         <ns0:v>Breakfast, lunch and drinks filters
-Café call outline with visit type, group size and questions</ns0:v>
+Café call outline with visit type, group size and questions
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J20" s="6" t="str">
         <ns0:v>Help customers narrow down a café visit and explain what they need when calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K20" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Piero Snack Bar. it includes breakfast, lunch and drinks filters and café call outline with visit type, group size and questions. the idea is to help customers narrow down a café visit and explain what they need when calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Piero Snack Bar. it includes breakfast, lunch and drinks filters and café call outline with visit type, group size and questions. the idea is to help customers narrow down a café visit and explain what they need when calling. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L20" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M20" s="6" t="str">
+        <ns0:v>Tap to call +441162515322: tel:+441162515322
+Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/pieros-snack-bar-8-loseby-lane
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Piero+Snack+Bar+8+Loseby+Lane+Leicester+LE1+5DR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21" ht="210" customHeight="1">
       <ns0:c r="A21" s="6" t="n">
         <ns0:v>15</ns0:v>
       </ns0:c>
@@ -931,19 +1009,25 @@
       </ns0:c>
       <ns0:c r="I21" s="6" t="str">
         <ns0:v>Product range explorer for cheese, meats, pastry and dairy
-Different enquiry paths for home shopping, trade supply and celebration cheese cakes</ns0:v>
+Different enquiry paths for home shopping, trade supply and celebration cheese cakes
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J21" s="6" t="str">
         <ns0:v>Separate everyday purchases from trade and celebration enquiries.</ns0:v>
       </ns0:c>
       <ns0:c r="K21" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Country Fayre Foods. it includes product range explorer for cheese, meats, pastry and dairy and different enquiry paths for home shopping, trade supply and celebration cheese cakes. the idea is to separate everyday purchases from trade and celebration enquiries. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Country Fayre Foods. it includes product range explorer for cheese, meats, pastry and dairy and different enquiry paths for home shopping, trade supply and celebration cheese cakes. the idea is to separate everyday purchases from trade and celebration enquiries. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L21" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="22" ht="150" customHeight="1">
+      <ns0:c r="M21" s="6" t="str">
+        <ns0:v>Tap to call 01162531432: tel:01162531432
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Country+Fayre+33+Market+Place+Leicester+LE1+5GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22" ht="210" customHeight="1">
       <ns0:c r="A22" s="6" t="n">
         <ns0:v>16</ns0:v>
       </ns0:c>
@@ -968,19 +1052,27 @@
       </ns0:c>
       <ns0:c r="I22" s="6" t="str">
         <ns0:v>Searchable rice and noodle menu selection
-Meal note with group size, visit type and questions</ns0:v>
+Meal note with group size, visit type and questions
+Direct link to Uber Eats ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J22" s="6" t="str">
         <ns0:v>Help customers narrow down dishes and prepare a clear meal enquiry.</ns0:v>
       </ns0:c>
       <ns0:c r="K22" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Taste of China. it includes searchable rice and noodle menu selection and meal note with group size, visit type and questions. the idea is to help customers narrow down dishes and prepare a clear meal enquiry. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Taste of China. it includes searchable rice and noodle menu selection and meal note with group size, visit type and questions. the idea is to help customers narrow down dishes and prepare a clear meal enquiry. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L22" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M22" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/taste-of-china-restaurant-leicester/rtCoA9kTX52dNSgg4eBzpw
+Tap to call +441162517878: tel:+441162517878
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Taste+of+China+25+High+Street+Leicester+LE1+4FP</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23" ht="210" customHeight="1">
       <ns0:c r="A23" s="6" t="n">
         <ns0:v>17</ns0:v>
       </ns0:c>
@@ -1007,19 +1099,25 @@
       </ns0:c>
       <ns0:c r="I23" s="6" t="str">
         <ns0:v>Box mix, noodle, rice and soup filters
-Group shortlist with quantities for each selected dish</ns0:v>
+Group shortlist with quantities for each selected dish
+Direct link to Uber Eats ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J23" s="6" t="str">
         <ns0:v>Help people coordinate a group meal before checking the real ordering menu.</ns0:v>
       </ns0:c>
       <ns0:c r="K23" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Noodle House. it includes box mix, noodle, rice and soup filters and group shortlist with quantities for each selected dish. the idea is to help people coordinate a group meal before checking the real ordering menu. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Noodle House. it includes box mix, noodle, rice and soup filters and group shortlist with quantities for each selected dish. the idea is to help people coordinate a group meal before checking the real ordering menu. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L23" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M23" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/noodle-house-narborough-road/WXgPuVsIUB2oSg39P31_NA
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Noodle+House+78+Narborough+Road+Leicester+LE3+0BS</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24" ht="210" customHeight="1">
       <ns0:c r="A24" s="6" t="n">
         <ns0:v>18</ns0:v>
       </ns0:c>
@@ -1045,19 +1143,23 @@
       </ns0:c>
       <ns0:c r="I24" s="6" t="str">
         <ns0:v>Separate daytime upstairs and evening whole-space hire options
-Hire enquiry outline with event type, date, guests, duration and setup needs</ns0:v>
+Hire enquiry outline with event type, date, guests, duration and setup needs
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J24" s="6" t="str">
         <ns0:v>Make a workshop, meetup or celebration enquiry easier to explain.</ns0:v>
       </ns0:c>
       <ns0:c r="K24" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Paper Wings Café. it includes separate daytime upstairs and evening whole-space hire options and hire enquiry outline with event type, date, guests, duration and setup needs. the idea is to make a workshop, meetup or celebration enquiry easier to explain. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Paper Wings Café. it includes separate daytime upstairs and evening whole-space hire options and hire enquiry outline with event type, date, guests, duration and setup needs. the idea is to make a workshop, meetup or celebration enquiry easier to explain. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L24" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="25" ht="150" customHeight="1">
+      <ns0:c r="M24" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://maps.app.goo.gl/jPqpp4EJdPvjpgpm8</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25" ht="210" customHeight="1">
       <ns0:c r="A25" s="6" t="n">
         <ns0:v>19</ns0:v>
       </ns0:c>
@@ -1083,19 +1185,24 @@
       <ns0:c r="I25" s="6" t="str">
         <ns0:v>Service selector including Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Oh So Pretty’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J25" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K25" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Oh So Pretty. visitors can compare options such as Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Oh So Pretty. visitors can compare options such as Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L25" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M25" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/oh-so-pretty-wigston-4-liskeard-house-telbdqpd
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=4%20Liskeard%20House%2C%20Wigston%20LE18%202GL</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26" ht="210" customHeight="1">
       <ns0:c r="A26" s="6" t="n">
         <ns0:v>20</ns0:v>
       </ns0:c>
@@ -1120,19 +1227,26 @@
       </ns0:c>
       <ns0:c r="I26" s="6" t="str">
         <ns0:v>Repair enquiry guide for phones, tablets, computers and consoles
-Device model and fault selection with a reviewable enquiry summary</ns0:v>
+Device model and fault selection with a reviewable enquiry summary
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J26" s="6" t="str">
         <ns0:v>Help customers describe their device problem before contacting the Leicester shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K26" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Fone Plus. it includes repair enquiry guide for phones, tablets, computers and consoles and device model and fault selection with a reviewable enquiry summary. the idea is to help customers describe their device problem before contacting the Leicester shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Fone Plus. it includes repair enquiry guide for phones, tablets, computers and consoles and device model and fault selection with a reviewable enquiry summary. the idea is to help customers describe their device problem before contacting the Leicester shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L26" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="27" ht="150" customHeight="1">
+      <ns0:c r="M26" s="6" t="str">
+        <ns0:v>Tap to call +447881906500: tel:+447881906500
+Tap to call +447447425001: tel:+447447425001
+Open directions in Google Maps: https://www.google.com/maps/place/Fone+Plus/@52.6368432,-1.1356291,17z/data=!3m1!4b1!4m6!3m5!1s0x4877610019cdd6f9:0xf850f2933751f558!8m2!3d52.6368432!4d-1.1330542!16s%2Fg%2F11ss35ryzr</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27" ht="210" customHeight="1">
       <ns0:c r="A27" s="6" t="n">
         <ns0:v>21</ns0:v>
       </ns0:c>
@@ -1158,19 +1272,27 @@
       </ns0:c>
       <ns0:c r="I27" s="6" t="str">
         <ns0:v>Brunch, lunch and evening menu sections
-Dining enquiry notes with occasion and guests, plus the existing Dojo booking link</ns0:v>
+Dining enquiry notes with occasion and guests, plus the existing Dojo booking link
+Direct link to Dojo table booking page
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J27" s="6" t="str">
         <ns0:v>Help visitors choose the right service and prepare their dining questions.</ns0:v>
       </ns0:c>
       <ns0:c r="K27" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Roma. it includes brunch, lunch and evening menu sections and dining enquiry notes with occasion and guests, plus the existing Dojo booking link. the idea is to help visitors choose the right service and prepare their dining questions. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Roma. it includes brunch, lunch and evening menu sections and dining enquiry notes with occasion and guests, plus the existing Dojo booking link. the idea is to help visitors choose the right service and prepare their dining questions. the site also links to your Dojo page for table bookings. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L27" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M27" s="6" t="str">
+        <ns0:v>Dojo table booking page: https://web.dojo.app/create_booking/vendor/Y65t9Q_MVtKVDzieR2yaN2Kkc9YfRctKlh_60fyZPSY_restaurant
+Tap to call 01162515959: tel:01162515959
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Roma+11+Halford+Street+Leicester+LE1+1JA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28" ht="210" customHeight="1">
       <ns0:c r="A28" s="6" t="n">
         <ns0:v>22</ns0:v>
       </ns0:c>
@@ -1192,19 +1314,24 @@
       <ns0:c r="I28" s="6" t="str">
         <ns0:v>Service selector including Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Cabello Mens Hairsalon’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J28" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K28" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Cabello Mens Hairsalon. visitors can compare options such as Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Cabello Mens Hairsalon. visitors can compare options such as Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L28" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M28" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/102764_cabello-mens-hairsalon_barber_64623_blaby
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=19a%20Leicester%20Road%20Blaby%20Leicester%20LE8%204GR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29" ht="210" customHeight="1">
       <ns0:c r="A29" s="6" t="n">
         <ns0:v>23</ns0:v>
       </ns0:c>
@@ -1229,19 +1356,23 @@
       </ns0:c>
       <ns0:c r="I29" s="6" t="str">
         <ns0:v>Range guide including beef, pork, lamb and alternative cuts
-Copyable butcher ask list based on cooking method, people and recipe questions</ns0:v>
+Copyable butcher ask list based on cooking method, people and recipe questions
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J29" s="6" t="str">
         <ns0:v>Help customers ask for a suitable cut without needing to know every product name.</ns0:v>
       </ns0:c>
       <ns0:c r="K29" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Frank Lee And Son. it includes range guide including beef, pork, lamb and alternative cuts and copyable butcher ask list based on cooking method, people and recipe questions. the idea is to help customers ask for a suitable cut without needing to know every product name. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Frank Lee And Son. it includes range guide including beef, pork, lamb and alternative cuts and copyable butcher ask list based on cooking method, people and recipe questions. the idea is to help customers ask for a suitable cut without needing to know every product name. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L29" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="30" ht="150" customHeight="1">
+      <ns0:c r="M29" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Frank%20Lee%20and%20Son%20Leicester%20Market%20Food%20Hall%20LE1%205GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30" ht="210" customHeight="1">
       <ns0:c r="A30" s="6" t="n">
         <ns0:v>24</ns0:v>
       </ns0:c>
@@ -1266,19 +1397,25 @@
       </ns0:c>
       <ns0:c r="I30" s="6" t="str">
         <ns0:v>Regional noodle guide with English and Chinese dish names
-Counter checklist for a chosen dish, group size, spice and ingredient questions</ns0:v>
+Counter checklist for a chosen dish, group size, spice and ingredient questions
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J30" s="6" t="str">
         <ns0:v>Make unfamiliar dishes easier to explore before asking at the counter.</ns0:v>
       </ns0:c>
       <ns0:c r="K30" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Guilin Street Food. it includes regional noodle guide with English and Chinese dish names and counter checklist for a chosen dish, group size, spice and ingredient questions. the idea is to make unfamiliar dishes easier to explore before asking at the counter. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Guilin Street Food. it includes regional noodle guide with English and Chinese dish names and counter checklist for a chosen dish, group size, spice and ingredient questions. the idea is to make unfamiliar dishes easier to explore before asking at the counter. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L30" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="31" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M30" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/guilin-street-food
+Tap to call +447550391293: tel:+447550391293</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31" ht="210" customHeight="1">
       <ns0:c r="A31" s="6" t="n">
         <ns0:v>25</ns0:v>
       </ns0:c>
@@ -1303,19 +1440,25 @@
       </ns0:c>
       <ns0:c r="I31" s="6" t="str">
         <ns0:v>Fish, shellfish and crustacean range guide
-Question list covering cooking plan, preparation, weight and handling</ns0:v>
+Question list covering cooking plan, preparation, weight and handling
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J31" s="6" t="str">
         <ns0:v>Help customers arrive with useful questions about choosing and preparing their fish.</ns0:v>
       </ns0:c>
       <ns0:c r="K31" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Leicester Wholesale Fish Direct. it includes fish, shellfish and crustacean range guide and question list covering cooking plan, preparation, weight and handling. the idea is to help customers arrive with useful questions about choosing and preparing their fish. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Leicester Wholesale Fish Direct. it includes fish, shellfish and crustacean range guide and question list covering cooking plan, preparation, weight and handling. the idea is to help customers arrive with useful questions about choosing and preparing their fish. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L31" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="32" ht="150" customHeight="1">
+      <ns0:c r="M31" s="6" t="str">
+        <ns0:v>Tap to call +441162165666: tel:+441162165666
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Leicester+Wholesale+Fish+Direct+Leicester+Market+Food+Hall+33+Market+Place+LE1+5GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32" ht="210" customHeight="1">
       <ns0:c r="A32" s="6" t="n">
         <ns0:v>26</ns0:v>
       </ns0:c>
@@ -1341,19 +1484,24 @@
       <ns0:c r="I32" s="6" t="str">
         <ns0:v>Service selector including Cut &amp; Blow Dry and Blow Dry
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Violet’s Hair Studio’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J32" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K32" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Violet’s Hair Studio. visitors can compare options such as Cut &amp; Blow Dry and Blow Dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Violet’s Hair Studio. visitors can compare options such as Cut &amp; Blow Dry and Blow Dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L32" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="33" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M32" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/violets-leicester-mowmacre-sports-ground-j96u6szs
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Mowmacre%20sports%20ground%2C%20Leicester%20LE4%202RG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33" ht="210" customHeight="1">
       <ns0:c r="A33" s="6" t="n">
         <ns0:v>27</ns0:v>
       </ns0:c>
@@ -1379,19 +1527,24 @@
       <ns0:c r="I33" s="6" t="str">
         <ns0:v>Service selector including Back, Neck &amp; Shoulders and Gel Toes
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Beauty by Mel’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J33" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K33" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Beauty by Mel. visitors can compare options such as Back, Neck &amp; Shoulders and Gel Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Beauty by Mel. visitors can compare options such as Back, Neck &amp; Shoulders and Gel Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L33" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="34" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M33" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/beauty-by-mel-glenfield-13-stamford-street-zk5d4485
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=13%20Stamford%20Street%2C%20Glenfield%20LE3%208DL</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34" ht="210" customHeight="1">
       <ns0:c r="A34" s="6" t="n">
         <ns0:v>28</ns0:v>
       </ns0:c>
@@ -1412,19 +1565,23 @@
       <ns0:c r="H34" s="6" t="str"/>
       <ns0:c r="I34" s="6" t="str">
         <ns0:v>Fruit tea finder for a chosen flavour
-Single flavour versus flavour pair matching</ns0:v>
+Single flavour versus flavour pair matching
+Direct link to Just Eat ordering menu</ns0:v>
       </ns0:c>
       <ns0:c r="J34" s="6" t="str">
         <ns0:v>Help someone who likes a particular fruit find relevant drinks quickly.</ns0:v>
       </ns0:c>
       <ns0:c r="K34" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Blossom Boba. it includes fruit tea finder for a chosen flavour and single flavour versus flavour pair matching. the idea is to help someone who likes a particular fruit find relevant drinks quickly. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Blossom Boba. it includes fruit tea finder for a chosen flavour and single flavour versus flavour pair matching. the idea is to help someone who likes a particular fruit find relevant drinks quickly. the site also links to your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L34" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="35" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M34" s="6" t="str">
+        <ns0:v>Just Eat ordering menu: https://www.just-eat.co.uk/restaurants-blossom-boba-leicester/menu</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35" ht="210" customHeight="1">
       <ns0:c r="A35" s="6" t="n">
         <ns0:v>29</ns0:v>
       </ns0:c>
@@ -1449,19 +1606,27 @@
       </ns0:c>
       <ns0:c r="I35" s="6" t="str">
         <ns0:v>Plated food versus handheld food filters
-Dish planner with side choice, quantities and group questions</ns0:v>
+Dish planner with side choice, quantities and group questions
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J35" s="6" t="str">
         <ns0:v>Help customers put their meal preferences into one clear discussion note.</ns0:v>
       </ns0:c>
       <ns0:c r="K35" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Latin Kitchen. it includes plated food versus handheld food filters and dish planner with side choice, quantities and group questions. the idea is to help customers put their meal preferences into one clear discussion note. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Latin Kitchen. it includes plated food versus handheld food filters and dish planner with side choice, quantities and group questions. the idea is to help customers put their meal preferences into one clear discussion note. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L35" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="36" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M35" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/latin-kitchen-uk
+Tap to call +447948758037: tel:+447948758037
+Open directions in Google Maps: https://maps.google.com/maps/place//data=!4m2!3m1!1s0x48776118b54332f9:0x4f87fe72148b6d79?entry=s</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36" ht="210" customHeight="1">
       <ns0:c r="A36" s="6" t="n">
         <ns0:v>30</ns0:v>
       </ns0:c>
@@ -1486,19 +1651,27 @@
       </ns0:c>
       <ns0:c r="I36" s="6" t="str">
         <ns0:v>Searchable sushi, bento, noodle and starter selection
-Copyable meal shortlist with a personal reminder</ns0:v>
+Copyable meal shortlist with a personal reminder
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J36" s="6" t="str">
         <ns0:v>Help diners keep their favourite dishes together while choosing a meal.</ns0:v>
       </ns0:c>
       <ns0:c r="K36" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Sakura. it includes searchable sushi, bento, noodle and starter selection and copyable meal shortlist with a personal reminder. the idea is to help diners keep their favourite dishes together while choosing a meal. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Sakura. it includes searchable sushi, bento, noodle and starter selection and copyable meal shortlist with a personal reminder. the idea is to help diners keep their favourite dishes together while choosing a meal. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L36" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="37" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M36" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/sakura-leicester
+Tap to call 01163481917: tel:01163481917
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Sakura%2080-84%20High%20Street%20Leicester%20LE1%205YP</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="37" ht="210" customHeight="1">
       <ns0:c r="A37" s="6" t="n">
         <ns0:v>31</ns0:v>
       </ns0:c>
@@ -1523,19 +1696,23 @@
       </ns0:c>
       <ns0:c r="I37" s="6" t="str">
         <ns0:v>Search and filters for breakfast plates and hot cobs
-Copyable café shortlist with group size and beans or tomatoes preference</ns0:v>
+Copyable café shortlist with group size and beans or tomatoes preference
+Direct link to Just Eat ordering menu</ns0:v>
       </ns0:c>
       <ns0:c r="J37" s="6" t="str">
         <ns0:v>Help visitors organise a breakfast choice before checking it with the café.</ns0:v>
       </ns0:c>
       <ns0:c r="K37" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Silver Street Cafe. it includes search and filters for breakfast plates and hot cobs and copyable café shortlist with group size and beans or tomatoes preference. the idea is to help visitors organise a breakfast choice before checking it with the café. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Silver Street Cafe. it includes search and filters for breakfast plates and hot cobs and copyable café shortlist with group size and beans or tomatoes preference. the idea is to help visitors organise a breakfast choice before checking it with the café. the site also links to your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L37" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="38" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M37" s="6" t="str">
+        <ns0:v>Just Eat ordering menu: https://www.just-eat.co.uk/restaurants-silver-street-cafe-leicester-le1/menu</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="38" ht="210" customHeight="1">
       <ns0:c r="A38" s="6" t="n">
         <ns0:v>32</ns0:v>
       </ns0:c>
@@ -1562,19 +1739,24 @@
       <ns0:c r="I38" s="6" t="str">
         <ns0:v>Service selector including Brow wax and Brow wax &amp; tint
 Listed prices and appointment lengths update with the selected service
-Link to the existing SumUp Bookings booking page</ns0:v>
+Booking buttons open The Beauty Lab’s existing SumUp Bookings booking page
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J38" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K38" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for The Beauty Lab. visitors can compare options such as Brow wax and Brow wax &amp; tint, see the listed price and appointment length, then open your SumUp Bookings booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for The Beauty Lab. visitors can compare options such as Brow wax and Brow wax &amp; tint, see the listed price and appointment length, then open your SumUp Bookings booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing SumUp Bookings page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L38" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="39" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M38" s="6" t="str">
+        <ns0:v>SumUp Bookings booking page: https://www.sumupbookings.com/the-beauty-lab-6
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=7%20Silverdale%20Drive%2C%20Thurmaston%20LE4%208NJ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="39" ht="210" customHeight="1">
       <ns0:c r="A39" s="6" t="n">
         <ns0:v>33</ns0:v>
       </ns0:c>
@@ -1599,19 +1781,25 @@
       </ns0:c>
       <ns0:c r="I39" s="6" t="str">
         <ns0:v>Food category explorer across steaks, starters, sizzlers and more
-Food photograph viewer and links to the existing booking route</ns0:v>
+Food photograph viewer and links to the existing booking route
+Direct link to OpenTable table booking page
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J39" s="6" t="str">
         <ns0:v>Help diners explore the type of evening they want before checking availability.</ns0:v>
       </ns0:c>
       <ns0:c r="K39" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Steak &amp; Lounge. it includes food category explorer across steaks, starters, sizzlers and more and food photograph viewer and links to the existing booking route. the idea is to help diners explore the type of evening they want before checking availability. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Steak &amp; Lounge. it includes food category explorer across steaks, starters, sizzlers and more and food photograph viewer and links to the existing booking route. the idea is to help diners explore the type of evening they want before checking availability. the site also links to your OpenTable page for table bookings. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L39" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="40" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M39" s="6" t="str">
+        <ns0:v>OpenTable table booking page: https://www.opentable.co.uk/r/steak-and-lounge-leicester
+Tap to call +441162622666: tel:+441162622666</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="40" ht="210" customHeight="1">
       <ns0:c r="A40" s="6" t="n">
         <ns0:v>34</ns0:v>
       </ns0:c>
@@ -1638,19 +1826,27 @@
       </ns0:c>
       <ns0:c r="I40" s="6" t="str">
         <ns0:v>Menu category filters and item detail views
-Copyable dish shortlist</ns0:v>
+Copyable dish shortlist
+Direct link to Uber Eats ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J40" s="6" t="str">
         <ns0:v>Help customers explore the chaat menu and keep the dishes they want to try together.</ns0:v>
       </ns0:c>
       <ns0:c r="K40" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Raykdi. it includes menu category filters and item detail views and copyable dish shortlist. the idea is to help customers explore the chaat menu and keep the dishes they want to try together. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Raykdi. it includes menu category filters and item detail views and copyable dish shortlist. the idea is to help customers explore the chaat menu and keep the dishes they want to try together. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L40" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="41" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M40" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/raykdi/vvkyVEY1U9m7DtpMCssIpQ
+Tap to call +447707181303: tel:+447707181303
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Raykdi%209%20Bath%20House%20Lane%20Leicester%20LE1%204SA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="41" ht="210" customHeight="1">
       <ns0:c r="A41" s="6" t="n">
         <ns0:v>35</ns0:v>
       </ns0:c>
@@ -1678,19 +1874,25 @@
       </ns0:c>
       <ns0:c r="I41" s="6" t="str">
         <ns0:v>Range guide covering beef, lamb, pork, poultry and offal
-Butcher question list shaped by meal type, people and preparation needs</ns0:v>
+Butcher question list shaped by meal type, people and preparation needs
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J41" s="6" t="str">
         <ns0:v>Help customers explain what they are cooking and get advice at the counter.</ns0:v>
       </ns0:c>
       <ns0:c r="K41" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Keith Ashmore. it includes range guide covering beef, lamb, pork, poultry and offal and butcher question list shaped by meal type, people and preparation needs. the idea is to help customers explain what they are cooking and get advice at the counter. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Keith Ashmore. it includes range guide covering beef, lamb, pork, poultry and offal and butcher question list shaped by meal type, people and preparation needs. the idea is to help customers explain what they are cooking and get advice at the counter. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L41" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="42" ht="150" customHeight="1">
+      <ns0:c r="M41" s="6" t="str">
+        <ns0:v>Tap to call +447710434752: tel:+447710434752
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Keith+Ashmore+Leicester+Market+Food+Hall+33+Market+Place+LE1+5GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="42" ht="210" customHeight="1">
       <ns0:c r="A42" s="6" t="n">
         <ns0:v>36</ns0:v>
       </ns0:c>
@@ -1715,19 +1917,25 @@
       </ns0:c>
       <ns0:c r="I42" s="6" t="str">
         <ns0:v>Brunch, lunch and drinks filters
-Café list for shortlisted dishes and drinks</ns0:v>
+Café list for shortlisted dishes and drinks
+Direct link to Deliveroo ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J42" s="6" t="str">
         <ns0:v>Help visitors choose a few brunch and drink ideas before arriving.</ns0:v>
       </ns0:c>
       <ns0:c r="K42" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for La Foret Cafe. it includes brunch, lunch and drinks filters and café list for shortlisted dishes and drinks. the idea is to help visitors choose a few brunch and drink ideas before arriving. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for La Foret Cafe. it includes brunch, lunch and drinks filters and café list for shortlisted dishes and drinks. the idea is to help visitors choose a few brunch and drink ideas before arriving. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L42" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="43" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M42" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/la-foret-cafe
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=11+King+Street%2C+Leicester</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="43" ht="210" customHeight="1">
       <ns0:c r="A43" s="6" t="n">
         <ns0:v>37</ns0:v>
       </ns0:c>
@@ -1752,19 +1960,29 @@
       </ns0:c>
       <ns0:c r="I43" s="6" t="str">
         <ns0:v>Separate brunch and bistro views with dish search
-Meal note that includes occasion, day and group size</ns0:v>
+Meal note that includes occasion, day and group size
+Direct link to SevenRooms table booking page
+Direct link to Just Eat ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J43" s="6" t="str">
         <ns0:v>Help visitors distinguish a brunch plan from an evening meal.</ns0:v>
       </ns0:c>
       <ns0:c r="K43" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for LYNN. it includes separate brunch and bistro views with dish search and meal note that includes occasion, day and group size. the idea is to help visitors distinguish a brunch plan from an evening meal. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for LYNN. it includes separate brunch and bistro views with dish search and meal note that includes occasion, day and group size. the idea is to help visitors distinguish a brunch plan from an evening meal. the site also links to your SevenRooms page for table bookings, and your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L43" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="44" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M43" s="6" t="str">
+        <ns0:v>SevenRooms table booking page: https://www.sevenrooms.com/explore/lynnleicester/reservations/create/search/
+Just Eat ordering menu: https://www.just-eat.co.uk/restaurants-lynn-leicester/menu
+Tap to call +447342375899: tel:+447342375899
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=LYNN%2014%20St%20Martins%20Square%20Leicester%20LE1%205DF</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="44" ht="210" customHeight="1">
       <ns0:c r="A44" s="6" t="n">
         <ns0:v>38</ns0:v>
       </ns0:c>
@@ -1789,19 +2007,23 @@
       </ns0:c>
       <ns0:c r="I44" s="6" t="str">
         <ns0:v>Searchable nasta, chai and Indo-Chinese dish references
-Copyable ask list with visit day, time of day and availability questions</ns0:v>
+Copyable ask list with visit day, time of day and availability questions
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J44" s="6" t="str">
         <ns0:v>Help visitors ask about the dishes they have seen without assuming they are available today.</ns0:v>
       </ns0:c>
       <ns0:c r="K44" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Milan Di Damao. it includes searchable nasta, chai and Indo-Chinese dish references and copyable ask list with visit day, time of day and availability questions. the idea is to help visitors ask about the dishes they have seen without assuming they are available today. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Milan Di Damao. it includes searchable nasta, chai and Indo-Chinese dish references and copyable ask list with visit day, time of day and availability questions. the idea is to help visitors ask about the dishes they have seen without assuming they are available today. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L44" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="45" ht="150" customHeight="1">
+      <ns0:c r="M44" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Milan%20Di%20Damao%2032%20Belgrave%20Road%20Leicester%20LE4%205AS</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="45" ht="210" customHeight="1">
       <ns0:c r="A45" s="6" t="n">
         <ns0:v>39</ns0:v>
       </ns0:c>
@@ -1827,19 +2049,24 @@
       <ns0:c r="I45" s="6" t="str">
         <ns0:v>Service selector including Eyebrows · threading and Eyebrows · waxing
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Beautylicious’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J45" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K45" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Beautylicious. visitors can compare options such as Eyebrows · threading and Eyebrows · waxing, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Beautylicious. visitors can compare options such as Eyebrows · threading and Eyebrows · waxing, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L45" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="46" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M45" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/beautylicious-braunstone-town-edward-avenue-wkuhuibt
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Edward%20Avenue%2C%20Braunstone%20Town%20LE3</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="46" ht="210" customHeight="1">
       <ns0:c r="A46" s="6" t="n">
         <ns0:v>40</ns0:v>
       </ns0:c>
@@ -1865,19 +2092,24 @@
       <ns0:c r="I46" s="6" t="str">
         <ns0:v>Service selector including Russian Infills and Classic Full Set
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Queen Lashes’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J46" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K46" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Queen Lashes. visitors can compare options such as Russian Infills and Classic Full Set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Queen Lashes. visitors can compare options such as Russian Infills and Classic Full Set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L46" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="47" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M46" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/queen-lashes-leicester-70-burnham-drive-ed7gqg00
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=70%20Burnham%20Drive%2C%20Leicester%20LE4%200HP</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="47" ht="210" customHeight="1">
       <ns0:c r="A47" s="6" t="n">
         <ns0:v>41</ns0:v>
       </ns0:c>
@@ -1904,13 +2136,14 @@
         <ns0:v>Help shoppers describe the kind of outfit they are looking for.</ns0:v>
       </ns0:c>
       <ns0:c r="K47" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for RKD. it includes menswear and womenswear browsing choices and casual or formal preferences with a copyable visit shortlist. the idea is to help shoppers describe the kind of outfit they are looking for. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for RKD. it includes menswear and womenswear browsing choices and casual or formal preferences with a copyable visit shortlist. the idea is to help shoppers describe the kind of outfit they are looking for. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L47" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="48" ht="150" customHeight="1">
+      <ns0:c r="M47" s="6" t="str"/>
+    </ns0:row>
+    <ns0:row r="48" ht="210" customHeight="1">
       <ns0:c r="A48" s="6" t="n">
         <ns0:v>42</ns0:v>
       </ns0:c>
@@ -1935,19 +2168,23 @@
       </ns0:c>
       <ns0:c r="I48" s="6" t="str">
         <ns0:v>Arcade, café and shop visit guide
-Copyable list of activities to explore</ns0:v>
+Copyable list of activities to explore
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J48" s="6" t="str">
         <ns0:v>Help visitors plan a trip that combines gaming, a café stop and browsing.</ns0:v>
       </ns0:c>
       <ns0:c r="K48" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Super Game Shack Level 2. it includes arcade, café and shop visit guide and copyable list of activities to explore. the idea is to help visitors plan a trip that combines gaming, a café stop and browsing. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Super Game Shack Level 2. it includes arcade, café and shop visit guide and copyable list of activities to explore. the idea is to help visitors plan a trip that combines gaming, a café stop and browsing. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L48" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="49" ht="150" customHeight="1">
+      <ns0:c r="M48" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Silver+Arcade+Leicester+LE1+5FA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="49" ht="210" customHeight="1">
       <ns0:c r="A49" s="6" t="n">
         <ns0:v>43</ns0:v>
       </ns0:c>
@@ -1972,19 +2209,27 @@
       </ns0:c>
       <ns0:c r="I49" s="6" t="str">
         <ns0:v>Window measurement notes with room labels and centimetre or inch units
-Multiple window entries with edit, copy and print controls</ns0:v>
+Multiple window entries with edit, copy and print controls
+Direct link to WhatsApp chat
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J49" s="6" t="str">
         <ns0:v>Help customers bring organised measurements and questions into the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K49" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Bradgate Lace. it includes window measurement notes with room labels and centimetre or inch units and multiple window entries with edit, copy and print controls. the idea is to help customers bring organised measurements and questions into the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Bradgate Lace. it includes window measurement notes with room labels and centimetre or inch units and multiple window entries with edit, copy and print controls. the idea is to help customers bring organised measurements and questions into the shop. the site also links to your WhatsApp chat for enquiries. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L49" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="50" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M49" s="6" t="str">
+        <ns0:v>Tap to call +447455981419: tel:+447455981419
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Bradgate%20Lace%207%20Odeon%20Arcade%20Cank%20Street%20Leicester%20LE1%205HJ
+WhatsApp chat: https://wa.me/447455981419</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="50" ht="210" customHeight="1">
       <ns0:c r="A50" s="6" t="n">
         <ns0:v>44</ns0:v>
       </ns0:c>
@@ -2009,19 +2254,25 @@
       </ns0:c>
       <ns0:c r="I50" s="6" t="str">
         <ns0:v>Phone make, model and fault enquiry guide
-Copyable repair discussion notes</ns0:v>
+Copyable repair discussion notes
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J50" s="6" t="str">
         <ns0:v>Help customers describe a screen, charging or camera problem before contacting the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K50" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Humberstone Mobile. it includes phone make, model and fault enquiry guide and copyable repair discussion notes. the idea is to help customers describe a screen, charging or camera problem before contacting the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Humberstone Mobile. it includes phone make, model and fault enquiry guide and copyable repair discussion notes. the idea is to help customers describe a screen, charging or camera problem before contacting the shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L50" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="51" ht="150" customHeight="1">
+      <ns0:c r="M50" s="6" t="str">
+        <ns0:v>Tap to call +447849027337: tel:+447849027337
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Humberstone%20Mobile%2028%20Humberstone%20Road%20Leicester%20LE5%200AR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="51" ht="210" customHeight="1">
       <ns0:c r="A51" s="6" t="n">
         <ns0:v>45</ns0:v>
       </ns0:c>
@@ -2046,19 +2297,25 @@
       </ns0:c>
       <ns0:c r="I51" s="6" t="str">
         <ns0:v>Searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks
-Food photograph views and an existing Uber Eats link</ns0:v>
+Food photograph views and an existing Uber Eats link
+Direct link to Uber Eats ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J51" s="6" t="str">
         <ns0:v>Help customers find a relevant lunch choice before visiting or opening the ordering provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K51" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Kicheri. it includes searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks and food photograph views and an existing Uber Eats link. the idea is to help customers find a relevant lunch choice before visiting or opening the ordering provider. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Kicheri. it includes searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks and food photograph views and an existing Uber Eats link. the idea is to help customers find a relevant lunch choice before visiting or opening the ordering provider. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L51" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="52" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M51" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/kicheri/1-bAM0_uSrq0eeCYGP3RQg
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Kicheri%2029%20Loseby%20Lane%20Leicester%20LE1%205DR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="52" ht="210" customHeight="1">
       <ns0:c r="A52" s="6" t="n">
         <ns0:v>46</ns0:v>
       </ns0:c>
@@ -2080,19 +2337,24 @@
       <ns0:c r="I52" s="6" t="str">
         <ns0:v>Service selector including BIAB Manicure and Gel Manicure
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open By.meadowmae’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J52" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K52" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for By.meadowmae. visitors can compare options such as BIAB Manicure and Gel Manicure, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for By.meadowmae. visitors can compare options such as BIAB Manicure and Gel Manicure, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L52" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="53" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M52" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/183660_by-meadowmae_nail-salon_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=7%20Parkstone%20Road%20Leicester%20LE5%201NP</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="53" ht="210" customHeight="1">
       <ns0:c r="A53" s="6" t="n">
         <ns0:v>47</ns0:v>
       </ns0:c>
@@ -2114,19 +2376,24 @@
       <ns0:c r="I53" s="6" t="str">
         <ns0:v>Service selector including Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Cargo Male Grooming’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J53" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K53" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Cargo Male Grooming. visitors can compare options such as Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Cargo Male Grooming. visitors can compare options such as Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L53" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="54" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M53" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/115069_cargo-male-grooming_barber_73715_groby
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=24%20Ratby%20Road%20Groby%20Leicester%20LE6%200GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="54" ht="210" customHeight="1">
       <ns0:c r="A54" s="6" t="n">
         <ns0:v>48</ns0:v>
       </ns0:c>
@@ -2154,19 +2421,25 @@
       </ns0:c>
       <ns0:c r="I54" s="6" t="str">
         <ns0:v>Visit planner for breakfast, lunch or a drink break
-Question list for dates, group size, outdoor seating and access</ns0:v>
+Question list for dates, group size, outdoor seating and access
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J54" s="6" t="str">
         <ns0:v>Help visitors organise their café questions before calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K54" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Cade Dido. it includes visit planner for breakfast, lunch or a drink break and question list for dates, group size, outdoor seating and access. the idea is to help visitors organise their café questions before calling. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Cade Dido. it includes visit planner for breakfast, lunch or a drink break and question list for dates, group size, outdoor seating and access. the idea is to help visitors organise their café questions before calling. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L54" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="55" ht="150" customHeight="1">
+      <ns0:c r="M54" s="6" t="str">
+        <ns0:v>Tap to call +447553914619: tel:+447553914619
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Cafe+Dido+12+Loseby+Lane+Leicester+LE1+5DR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="55" ht="210" customHeight="1">
       <ns0:c r="A55" s="6" t="n">
         <ns0:v>49</ns0:v>
       </ns0:c>
@@ -2192,19 +2465,24 @@
       <ns0:c r="I55" s="6" t="str">
         <ns0:v>Service selector including Ladies Cut &amp; Finish and Blow dry
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Grace Hairstylist’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J55" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K55" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Grace Hairstylist. visitors can compare options such as Ladies Cut &amp; Finish and Blow dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Grace Hairstylist. visitors can compare options such as Ladies Cut &amp; Finish and Blow dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L55" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="56" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M55" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/grace-hairstylist-leicester-browns-107-clarendon-park-road-w3ytcuxn
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Browns%2C%20107%20Clarendon%20Park%20Road%2C%20Leicester%20LE2%203AH</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="56" ht="210" customHeight="1">
       <ns0:c r="A56" s="6" t="n">
         <ns0:v>50</ns0:v>
       </ns0:c>
@@ -2230,19 +2508,24 @@
       <ns0:c r="I56" s="6" t="str">
         <ns0:v>Service selector including Cut &amp; Finish and Gents Cut &amp; Finish
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Josh’s Hair Hideaway’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J56" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K56" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Josh’s Hair Hideaway. visitors can compare options such as Cut &amp; Finish and Gents Cut &amp; Finish, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Josh’s Hair Hideaway. visitors can compare options such as Cut &amp; Finish and Gents Cut &amp; Finish, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L56" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="57" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M56" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/joshs-hair-hideaway-leicester-uk-39-courtenay-road-r4zvys8z
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=39%20Courtenay%20Road%2C%20Leicester%20LE3%209TA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="57" ht="210" customHeight="1">
       <ns0:c r="A57" s="6" t="n">
         <ns0:v>51</ns0:v>
       </ns0:c>
@@ -2268,19 +2551,24 @@
       <ns0:c r="I57" s="6" t="str">
         <ns0:v>Service selector including 30 min Mini fill and Brow wax and tint
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Pretty Suite by Abbie’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J57" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K57" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Pretty Suite by Abbie. visitors can compare options such as 30 min Mini fill and Brow wax and tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Pretty Suite by Abbie. visitors can compare options such as 30 min Mini fill and Brow wax and tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L57" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="58" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M57" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/pretty-suite-by-abbie-leicester-hill-rise-tw0ac4s3
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Hill%20Rise%2C%20Leicester%20LE4</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="58" ht="210" customHeight="1">
       <ns0:c r="A58" s="6" t="n">
         <ns0:v>52</ns0:v>
       </ns0:c>
@@ -2305,19 +2593,23 @@
       </ns0:c>
       <ns0:c r="I58" s="6" t="str">
         <ns0:v>Guide to snacks, newspapers, mobile top-ups and bill services
-Visit checklist with questions for the selected services</ns0:v>
+Visit checklist with questions for the selected services
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J58" s="6" t="str">
         <ns0:v>Help shoppers check what they need from the kiosk before making a trip.</ns0:v>
       </ns0:c>
       <ns0:c r="K58" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Haymarket Kiosk. it includes guide to snacks, newspapers, mobile top-ups and bill services and visit checklist with questions for the selected services. the idea is to help shoppers check what they need from the kiosk before making a trip. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Haymarket Kiosk. it includes guide to snacks, newspapers, mobile top-ups and bill services and visit checklist with questions for the selected services. the idea is to help shoppers check what they need from the kiosk before making a trip. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L58" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="59" ht="150" customHeight="1">
+      <ns0:c r="M58" s="6" t="str">
+        <ns0:v>Tap to call +441162536033: tel:+441162536033</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="59" ht="210" customHeight="1">
       <ns0:c r="A59" s="6" t="n">
         <ns0:v>53</ns0:v>
       </ns0:c>
@@ -2343,19 +2635,24 @@
       <ns0:c r="I59" s="6" t="str">
         <ns0:v>Service selector including Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Aimee Charlotte Beauty’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J59" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K59" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Aimee Charlotte Beauty. visitors can compare options such as Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Aimee Charlotte Beauty. visitors can compare options such as Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L59" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="60" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M59" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/aimee-charlotte-beauty-anstey-megslashes-37-the-nook-c4dfe1bt
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=MegsLashes%2C%2037%20The%20Nook%2C%20Anstey%20LE7%207AZ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="60" ht="210" customHeight="1">
       <ns0:c r="A60" s="6" t="n">
         <ns0:v>54</ns0:v>
       </ns0:c>
@@ -2381,19 +2678,24 @@
       <ns0:c r="I60" s="6" t="str">
         <ns0:v>Service selector including LVL Lash Lift and Individual eyelash extensions - Full set
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Anelita Beauty’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J60" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K60" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Anelita Beauty. visitors can compare options such as LVL Lash Lift and Individual eyelash extensions - Full set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Anelita Beauty. visitors can compare options such as LVL Lash Lift and Individual eyelash extensions - Full set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L60" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="61" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M60" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/anelita-beauty-leicester-30a-blaby-road-y1gkfn59
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=30A%20Blaby%20Road%2C%20Leicester%20LE18%204PA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="61" ht="210" customHeight="1">
       <ns0:c r="A61" s="6" t="n">
         <ns0:v>55</ns0:v>
       </ns0:c>
@@ -2419,19 +2721,24 @@
       <ns0:c r="I61" s="6" t="str">
         <ns0:v>Service selector including Hair up and Tapes Half head Maintenance
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Hair by Tia’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J61" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K61" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Hair by Tia. visitors can compare options such as Hair up and Tapes Half head Maintenance, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Hair by Tia. visitors can compare options such as Hair up and Tapes Half head Maintenance, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L61" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="62" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M61" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/hair-by-tia-leicester-uk-100-lorne-road-glbzje22
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=100%20Lorne%20Road%2C%20Leicester%20LE2%201YG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="62" ht="210" customHeight="1">
       <ns0:c r="A62" s="6" t="n">
         <ns0:v>56</ns0:v>
       </ns0:c>
@@ -2456,19 +2763,25 @@
       </ns0:c>
       <ns0:c r="I62" s="6" t="str">
         <ns0:v>Produce, grocery and fresh bread category guide
-Copyable shopping interests list</ns0:v>
+Copyable shopping interests list
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J62" s="6" t="str">
         <ns0:v>Help customers organise the parts of their shop they want to ask about.</ns0:v>
       </ns0:c>
       <ns0:c r="K62" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for International Food Centre. it includes produce, grocery and fresh bread category guide and copyable shopping interests list. the idea is to help customers organise the parts of their shop they want to ask about. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for International Food Centre. it includes produce, grocery and fresh bread category guide and copyable shopping interests list. the idea is to help customers organise the parts of their shop they want to ask about. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L62" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="63" ht="150" customHeight="1">
+      <ns0:c r="M62" s="6" t="str">
+        <ns0:v>Tap to call +441162552149: tel:+441162552149
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=International+Food+Centre+Narborough+Road+Leicester+LE3+0LE</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="63" ht="210" customHeight="1">
       <ns0:c r="A63" s="6" t="n">
         <ns0:v>57</ns0:v>
       </ns0:c>
@@ -2493,19 +2806,25 @@
       </ns0:c>
       <ns0:c r="I63" s="6" t="str">
         <ns0:v>Vegetarian dish examples grouped by comfort food and soup
-Café photograph viewer and Free Lane visit information</ns0:v>
+Café photograph viewer and Free Lane visit information
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J63" s="6" t="str">
         <ns0:v>Give visitors a feel for the cooking and help them recognise the café.</ns0:v>
       </ns0:c>
       <ns0:c r="K63" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for The Good Earth. it includes vegetarian dish examples grouped by comfort food and soup and café photograph viewer and Free Lane visit information. the idea is to give visitors a feel for the cooking and help them recognise the café. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for The Good Earth. it includes vegetarian dish examples grouped by comfort food and soup and café photograph viewer and Free Lane visit information. the idea is to give visitors a feel for the cooking and help them recognise the café. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L63" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="64" ht="150" customHeight="1">
+      <ns0:c r="M63" s="6" t="str">
+        <ns0:v>Tap to call +441162626260: tel:+441162626260
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=The+Good+Earth+19+Free+Lane+Leicester+LE1+1JX</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="64" ht="210" customHeight="1">
       <ns0:c r="A64" s="6" t="n">
         <ns0:v>58</ns0:v>
       </ns0:c>
@@ -2526,19 +2845,25 @@
       <ns0:c r="H64" s="6" t="str"/>
       <ns0:c r="I64" s="6" t="str">
         <ns0:v>Fruit, meat and chicken, and bread category choices
-Copyable shopping note</ns0:v>
+Copyable shopping note
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J64" s="6" t="str">
         <ns0:v>Help customers bring together the items they want to discuss in the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K64" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Leicester Fresh Food. it includes fruit, meat and chicken, and bread category choices and copyable shopping note. the idea is to help customers bring together the items they want to discuss in the shop. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Leicester Fresh Food. it includes fruit, meat and chicken, and bread category choices and copyable shopping note. the idea is to help customers bring together the items they want to discuss in the shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L64" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="65" ht="150" customHeight="1">
+      <ns0:c r="M64" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Leicester+Fresh+Food+33+Narborough+Road+Leicester+LE3+0LE
+Tap to call +447999979796: tel:+447999979796</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="65" ht="210" customHeight="1">
       <ns0:c r="A65" s="6" t="n">
         <ns0:v>59</ns0:v>
       </ns0:c>
@@ -2563,19 +2888,25 @@
       </ns0:c>
       <ns0:c r="I65" s="6" t="str">
         <ns0:v>Treatment information and Church Gate location details
-Links to the existing business website and directions</ns0:v>
+Links to the existing business website and directions
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J65" s="6" t="str">
         <ns0:v>Give people a clear starting point for asking about treatments and planning a visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K65" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Soi 52. it includes treatment information and Church Gate location details and links to the existing business website and directions. the idea is to give people a clear starting point for asking about treatments and planning a visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Soi 52. it includes treatment information and Church Gate location details and links to the existing business website and directions. the idea is to give people a clear starting point for asking about treatments and planning a visit. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L65" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="66" ht="150" customHeight="1">
+      <ns0:c r="M65" s="6" t="str">
+        <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Soi52%2052%20Church%20Gate%20Leicester%20LE1%204AJ
+Tap to call +447886366933: tel:+447886366933</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="66" ht="210" customHeight="1">
       <ns0:c r="A66" s="6" t="n">
         <ns0:v>60</ns0:v>
       </ns0:c>
@@ -2597,19 +2928,24 @@
       <ns0:c r="I66" s="6" t="str">
         <ns0:v>Service selector including Wash Cut &amp; Blowdry and Signature Blowout
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Soie Hair’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J66" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K66" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Soie Hair. visitors can compare options such as Wash Cut &amp; Blowdry and Signature Blowout, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Soie Hair. visitors can compare options such as Wash Cut &amp; Blowdry and Signature Blowout, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L66" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="67" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M66" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/188904_soie-hair_hair-salon_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=2%20South%20Knighton%20Road%20Leicester%20LE2%203LN</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="67" ht="210" customHeight="1">
       <ns0:c r="A67" s="6" t="n">
         <ns0:v>61</ns0:v>
       </ns0:c>
@@ -2635,19 +2971,26 @@
       <ns0:c r="I67" s="6" t="str">
         <ns0:v>Service selector including Hair cut and Skin fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Star Barbers Oadby’s existing Booksy booking profile
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J67" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K67" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Star Barbers Oadby. visitors can compare options such as Hair cut and Skin fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Star Barbers Oadby. visitors can compare options such as Hair cut and Skin fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L67" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="68" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M67" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/98224_star-barbers-oadby_barber_79319_oadby
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=58%20Chestnut%20Avenue%20Oadby%20Leicester%20LE2%205JG
+Tap to call +441164026122: tel:+441164026122</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="68" ht="210" customHeight="1">
       <ns0:c r="A68" s="6" t="n">
         <ns0:v>62</ns0:v>
       </ns0:c>
@@ -2669,19 +3012,24 @@
       <ns0:c r="I68" s="6" t="str">
         <ns0:v>Service selector including Skin fade and Taper fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open M K BARBER’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J68" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K68" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for M K BARBER. visitors can compare options such as Skin fade and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for M K BARBER. visitors can compare options such as Skin fade and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L68" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="69" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M68" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/153839_m-k-barber_barber_79753_wigston
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=45%20Bell%20Street%20Wigston%20LE18%201AD</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="69" ht="210" customHeight="1">
       <ns0:c r="A69" s="6" t="n">
         <ns0:v>63</ns0:v>
       </ns0:c>
@@ -2702,19 +3050,27 @@
       <ns0:c r="H69" s="6" t="str"/>
       <ns0:c r="I69" s="6" t="str">
         <ns0:v>Coffee, specials and açaí menu filters
-Four-topping açaí bowl outline builder</ns0:v>
+Four-topping açaí bowl outline builder
+Direct link to Uber Eats ordering menu
+Direct link to Square gift card page
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J69" s="6" t="str">
         <ns0:v>Let visitors explore a bowl combination before checking the existing ordering options.</ns0:v>
       </ns0:c>
       <ns0:c r="K69" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Alcove. it includes coffee, specials and açaí menu filters and four-topping açaí bowl outline builder. the idea is to let visitors explore a bowl combination before checking the existing ordering options. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Alcove. it includes coffee, specials and açaí menu filters and four-topping açaí bowl outline builder. the idea is to let visitors explore a bowl combination before checking the existing ordering options. the site also links to your existing Uber Eats menu for ordering, and your Square gift card page. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L69" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="70" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M69" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/alcove/8TM387sUXl-NeVJvhYXdIA
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Alcove+27+St+Nicholas+Place+Leicester+LE1+4LD
+Square gift card page: https://app.squareup.com/gift/MLDHD6J3GQ4YJ/order</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="70" ht="210" customHeight="1">
       <ns0:c r="A70" s="6" t="n">
         <ns0:v>64</ns0:v>
       </ns0:c>
@@ -2736,19 +3092,24 @@
       <ns0:c r="I70" s="6" t="str">
         <ns0:v>Service selector including Gents Haircut and Skin Fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open The Mane Room Leicester’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J70" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K70" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for The Mane Room Leicester. visitors can compare options such as Gents Haircut and Skin Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for The Mane Room Leicester. visitors can compare options such as Gents Haircut and Skin Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L70" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="71" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M70" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/130067_the-mane-room-leicester_barber_79753_wigston
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=94%20Leicester%20Road%20Wigston%20LE18%201DR</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="71" ht="210" customHeight="1">
       <ns0:c r="A71" s="6" t="n">
         <ns0:v>65</ns0:v>
       </ns0:c>
@@ -2770,19 +3131,24 @@
       <ns0:c r="I71" s="6" t="str">
         <ns0:v>Service selector including Gents Haircut and Skin or Zero Fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Mancave Barber Lounge’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J71" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K71" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Mancave Barber Lounge. visitors can compare options such as Gents Haircut and Skin or Zero Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Mancave Barber Lounge. visitors can compare options such as Gents Haircut and Skin or Zero Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L71" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="72" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M71" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/20487_mancave-barber-lounge_barber_79753_wigston
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=5%20Bell%20Street%20Wigston%20LE18%201AD</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="72" ht="210" customHeight="1">
       <ns0:c r="A72" s="6" t="n">
         <ns0:v>66</ns0:v>
       </ns0:c>
@@ -2808,19 +3174,26 @@
       <ns0:c r="I72" s="6" t="str">
         <ns0:v>Service selector including BIAB overlay and BIAB infill
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open 11:11 Studios’s existing Fresha booking profile
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J72" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K72" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for 11:11 Studios. visitors can compare options such as BIAB overlay and BIAB infill, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for 11:11 Studios. visitors can compare options such as BIAB overlay and BIAB infill, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L72" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="73" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M72" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/11-11-studios-leicester-10-turville-road-d3i3gen7
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=10%20Turville%20Road%20Leicester%20LE3%201NY
+Tap to call +447835773090: tel:+447835773090</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="73" ht="210" customHeight="1">
       <ns0:c r="A73" s="6" t="n">
         <ns0:v>67</ns0:v>
       </ns0:c>
@@ -2846,19 +3219,24 @@
       <ns0:c r="I73" s="6" t="str">
         <ns0:v>Service selector including Ladies Cut and Blow dry and Gents cut no wash
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open MPHair’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J73" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K73" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for MPHair. visitors can compare options such as Ladies Cut and Blow dry and Gents cut no wash, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for MPHair. visitors can compare options such as Ladies Cut and Blow dry and Gents cut no wash, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L73" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="74" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M73" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/mphair-glenfield-102-dominion-road-dixl6g64
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=102%20Dominion%20Road%20Unit%203%2C%20Glenfield%20LE3%208FB</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="74" ht="210" customHeight="1">
       <ns0:c r="A74" s="6" t="n">
         <ns0:v>68</ns0:v>
       </ns0:c>
@@ -2885,19 +3263,24 @@
       <ns0:c r="I74" s="6" t="str">
         <ns0:v>Service selector including BIAB Infill and Eyebrow shape &amp; Tint
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Be beautiful by Alex’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J74" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K74" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Be beautiful by Alex. visitors can compare options such as BIAB Infill and Eyebrow shape &amp; Tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Be beautiful by Alex. visitors can compare options such as BIAB Infill and Eyebrow shape &amp; Tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L74" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="75" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M74" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/be-beautiful-by-alex-glenfield-stamford-street-li3z5jdq
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=13%20Stamford%20Street%2C%20Glenfield%20LE3%208DL</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="75" ht="210" customHeight="1">
       <ns0:c r="A75" s="6" t="n">
         <ns0:v>69</ns0:v>
       </ns0:c>
@@ -2923,19 +3306,24 @@
       <ns0:c r="I75" s="6" t="str">
         <ns0:v>Service selector including Knotless/Box Braids and Make-up (For Occasions)
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Graced by Helen’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J75" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K75" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Graced by Helen. visitors can compare options such as Knotless/Box Braids and Make-up (For Occasions), see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Graced by Helen. visitors can compare options such as Knotless/Box Braids and Make-up (For Occasions), see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L75" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="76" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M75" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/graced-by-helen-leicester-aadams-apartments-uk-20-frog-island-b5u60lzv
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Aadams%20Apartments%2C%2020%20Frog%20Island%2C%20Leicester%20LE3%205AG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="76" ht="210" customHeight="1">
       <ns0:c r="A76" s="6" t="n">
         <ns0:v>70</ns0:v>
       </ns0:c>
@@ -2963,19 +3351,25 @@
       </ns0:c>
       <ns0:c r="I76" s="6" t="str">
         <ns0:v>Gift brief built around occasion and shopping interest
-Optional budget selection and a copyable summary</ns0:v>
+Optional budget selection and a copyable summary
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J76" s="6" t="str">
         <ns0:v>Help shoppers explain a birthday, thank-you or just-because gift idea.</ns0:v>
       </ns0:c>
       <ns0:c r="K76" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Pot Pourri Shop. it includes gift brief built around occasion and shopping interest and optional budget selection and a copyable summary. the idea is to help shoppers explain a birthday, thank-you or just-because gift idea. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Pot Pourri Shop. it includes gift brief built around occasion and shopping interest and optional budget selection and a copyable summary. the idea is to help shoppers explain a birthday, thank-you or just-because gift idea. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L76" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="77" ht="150" customHeight="1">
+      <ns0:c r="M76" s="6" t="str">
+        <ns0:v>Tap to call +441162626666: tel:+441162626666
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=The+Pot+Pourri+Shop+17+Free+Lane+Leicester+LE1+1JX</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="77" ht="210" customHeight="1">
       <ns0:c r="A77" s="6" t="n">
         <ns0:v>71</ns0:v>
       </ns0:c>
@@ -3000,19 +3394,25 @@
       </ns0:c>
       <ns0:c r="I77" s="6" t="str">
         <ns0:v>Nail inspiration choices from the salon gallery
-Call note combining the chosen look with preferred nail length</ns0:v>
+Call note combining the chosen look with preferred nail length
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J77" s="6" t="str">
         <ns0:v>Help clients describe the finish they have in mind before speaking to the salon.</ns0:v>
       </ns0:c>
       <ns0:c r="K77" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for London Nails. it includes nail inspiration choices from the salon gallery and call note combining the chosen look with preferred nail length. the idea is to help clients describe the finish they have in mind before speaking to the salon. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for London Nails. it includes nail inspiration choices from the salon gallery and call note combining the chosen look with preferred nail length. the idea is to help clients describe the finish they have in mind before speaking to the salon. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L77" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="78" ht="150" customHeight="1">
+      <ns0:c r="M77" s="6" t="str">
+        <ns0:v>Tap to call +447762262345: tel:+447762262345
+Open directions in Google Maps: https://maps.app.goo.gl/YkoSCLvR1rJMRjJc8?g_st=com.google.maps.preview.copy</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="78" ht="210" customHeight="1">
       <ns0:c r="A78" s="6" t="n">
         <ns0:v>72</ns0:v>
       </ns0:c>
@@ -3039,19 +3439,24 @@
       <ns0:c r="I78" s="6" t="str">
         <ns0:v>Service selector including Restyle and Patch test &amp; consultation
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Tiegan Seaton (Seats Hair Studio)’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J78" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K78" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Tiegan Seaton (Seats Hair Studio). visitors can compare options such as Restyle and Patch test &amp; consultation, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Tiegan Seaton (Seats Hair Studio). visitors can compare options such as Restyle and Patch test &amp; consultation, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L78" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="79" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M78" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/tiegan-seaton-seats-hair-studio-anstey-4b-cropston-road-mozb3qoa
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=4B%20Cropston%20Road%2C%20Anstey%20LE7%207BJ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="79" ht="210" customHeight="1">
       <ns0:c r="A79" s="6" t="n">
         <ns0:v>73</ns0:v>
       </ns0:c>
@@ -3077,19 +3482,24 @@
       <ns0:c r="I79" s="6" t="str">
         <ns0:v>Service selector including Shape up and Haircut
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Royalty Trimz’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J79" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K79" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Royalty Trimz. visitors can compare options such as Shape up and Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Royalty Trimz. visitors can compare options such as Shape up and Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L79" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="80" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M79" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/royalty-trimz-leicester-40-church-gate-xkxfpy1l
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=40%20Church%20Gate%2C%20Leicester%20LE1%204AF</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="80" ht="210" customHeight="1">
       <ns0:c r="A80" s="6" t="n">
         <ns0:v>74</ns0:v>
       </ns0:c>
@@ -3115,19 +3525,26 @@
       <ns0:c r="I80" s="6" t="str">
         <ns0:v>Service selector including Ladies Cut &amp; Blowdry and Long Hair Blowdry
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Hair Muse’s existing Fresha booking profile
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J80" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K80" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Hair Muse. visitors can compare options such as Ladies Cut &amp; Blowdry and Long Hair Blowdry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Hair Muse. visitors can compare options such as Ladies Cut &amp; Blowdry and Long Hair Blowdry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L80" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="81" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M80" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/hair-muse-leicester-247-clarendon-park-road-lqtsyymq
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=247%20Clarendon%20Park%20Road%20Leicester%20LE2%203AN
+Tap to call +441165075590: tel:+441165075590</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="81" ht="210" customHeight="1">
       <ns0:c r="A81" s="6" t="n">
         <ns0:v>75</ns0:v>
       </ns0:c>
@@ -3153,19 +3570,24 @@
       <ns0:c r="I81" s="6" t="str">
         <ns0:v>Service selector including Haircut · Senior barber and Haircut &amp; Beard · Senior barber
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Autofaders’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J81" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K81" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Autofaders. visitors can compare options such as Haircut · Senior barber and Haircut &amp; Beard · Senior barber, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Autofaders. visitors can compare options such as Haircut · Senior barber and Haircut &amp; Beard · Senior barber, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L81" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="82" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M81" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/autofaders-ltd-where-style-meets-precision-leicester-8c-devana-road-nxj56jn6
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=8c%20Devana%20Road%2C%20Leicester%20LE2%201PJ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="82" ht="210" customHeight="1">
       <ns0:c r="A82" s="6" t="n">
         <ns0:v>76</ns0:v>
       </ns0:c>
@@ -3192,19 +3614,24 @@
       <ns0:c r="I82" s="6" t="str">
         <ns0:v>Service selector including Makeup and Prom makeup
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open GlamUpWithEster’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J82" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K82" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for GlamUpWithEster. visitors can compare options such as Makeup and Prom makeup, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for GlamUpWithEster. visitors can compare options such as Makeup and Prom makeup, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L82" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="83" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M82" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/glamupwithester-leicester-airborne-rn00zt24
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Airborne%2C%20Leicester%20LE7</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="83" ht="210" customHeight="1">
       <ns0:c r="A83" s="6" t="n">
         <ns0:v>77</ns0:v>
       </ns0:c>
@@ -3226,19 +3653,24 @@
       <ns0:c r="I83" s="6" t="str">
         <ns0:v>Service selector including Builder Gel Infills and Acrylic Nails
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Mercy Nails’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J83" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K83" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Mercy Nails. visitors can compare options such as Builder Gel Infills and Acrylic Nails, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Mercy Nails. visitors can compare options such as Builder Gel Infills and Acrylic Nails, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L83" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="84" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M83" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/155807_mercy-nails_nail-salon_65190_glenfield
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=102%20Dominion%20Road%20Leicester%20LE3%208FB</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="84" ht="210" customHeight="1">
       <ns0:c r="A84" s="6" t="n">
         <ns0:v>78</ns0:v>
       </ns0:c>
@@ -3265,19 +3697,22 @@
       <ns0:c r="I84" s="6" t="str">
         <ns0:v>Service selector including Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Sapphire Treatments’s existing Fresha booking profile</ns0:v>
       </ns0:c>
       <ns0:c r="J84" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K84" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Sapphire Treatments. visitors can compare options such as Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Sapphire Treatments. visitors can compare options such as Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L84" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="85" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M84" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/sapphire-treatments-leicester-vsa5bzok</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="85" ht="210" customHeight="1">
       <ns0:c r="A85" s="6" t="n">
         <ns0:v>79</ns0:v>
       </ns0:c>
@@ -3304,19 +3739,24 @@
       <ns0:c r="I85" s="6" t="str">
         <ns0:v>Service selector including Wash Cut &amp; Blowdry and Mens Haircut
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open SamBrayHair’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J85" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K85" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for SamBrayHair. visitors can compare options such as Wash Cut &amp; Blowdry and Mens Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for SamBrayHair. visitors can compare options such as Wash Cut &amp; Blowdry and Mens Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L85" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="86" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M85" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/sambrayhair-thurmaston-uk-church-hill-road-w5hi6pp2
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Church%20Hill%20Road%20Thurmaston%20Leicester%20LE4%208DE</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="86" ht="210" customHeight="1">
       <ns0:c r="A86" s="6" t="n">
         <ns0:v>80</ns0:v>
       </ns0:c>
@@ -3342,19 +3782,24 @@
       <ns0:c r="I86" s="6" t="str">
         <ns0:v>Service selector including BIAB and BIAB Toes
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Jennifer Audrey Nails &amp; Beauty’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J86" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K86" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Jennifer Audrey Nails &amp; Beauty. visitors can compare options such as BIAB and BIAB Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Jennifer Audrey Nails &amp; Beauty. visitors can compare options such as BIAB and BIAB Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L86" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="87" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M86" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/jennifer-audrey-nails-beauty-leicester-thurmaston-fa8uc05k
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Thurmaston%2C%20Leicester%20LE4%208NQ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="87" ht="210" customHeight="1">
       <ns0:c r="A87" s="6" t="n">
         <ns0:v>81</ns0:v>
       </ns0:c>
@@ -3379,19 +3824,25 @@
       </ns0:c>
       <ns0:c r="I87" s="6" t="str">
         <ns0:v>Korean dish filters covering bibimbap, bulgogi, soups and more
-Meal shortlist with table BBQ, spice and allergy questions</ns0:v>
+Meal shortlist with table BBQ, spice and allergy questions
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J87" s="6" t="str">
         <ns0:v>Help a group organise dishes and the questions they want to discuss.</ns0:v>
       </ns0:c>
       <ns0:c r="K87" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Oppa Korean Restaurant. it includes korean dish filters covering bibimbap, bulgogi, soups and more and meal shortlist with table BBQ, spice and allergy questions. the idea is to help a group organise dishes and the questions they want to discuss. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Oppa Korean Restaurant. it includes korean dish filters covering bibimbap, bulgogi, soups and more and meal shortlist with table BBQ, spice and allergy questions. the idea is to help a group organise dishes and the questions they want to discuss. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L87" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="88" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M87" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/oppa-korean-bbq-restaurant
+Tap to call +441164295128: tel:+441164295128</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="88" ht="210" customHeight="1">
       <ns0:c r="A88" s="6" t="n">
         <ns0:v>82</ns0:v>
       </ns0:c>
@@ -3417,19 +3868,25 @@
       </ns0:c>
       <ns0:c r="I88" s="6" t="str">
         <ns0:v>Cheese and deli guide with accompaniment ideas
-Gathering question list covering guest count, flavour preferences and serving questions</ns0:v>
+Gathering question list covering guest count, flavour preferences and serving questions
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J88" s="6" t="str">
         <ns0:v>Help customers ask for a cheese selection suited to their gathering.</ns0:v>
       </ns0:c>
       <ns0:c r="K88" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Sherwin's Cheese Company. it includes cheese and deli guide with accompaniment ideas and gathering question list covering guest count, flavour preferences and serving questions. the idea is to help customers ask for a cheese selection suited to their gathering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Sherwin's Cheese Company. it includes cheese and deli guide with accompaniment ideas and gathering question list covering guest count, flavour preferences and serving questions. the idea is to help customers ask for a cheese selection suited to their gathering. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L88" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="89" ht="150" customHeight="1">
+      <ns0:c r="M88" s="6" t="str">
+        <ns0:v>Tap to call +441162629236: tel:+441162629236
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Sherwins+Cheese+Company+Leicester+Market+Food+Hall+33+Market+Place+LE1+5GG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="89" ht="210" customHeight="1">
       <ns0:c r="A89" s="6" t="n">
         <ns0:v>83</ns0:v>
       </ns0:c>
@@ -3454,19 +3911,25 @@
       </ns0:c>
       <ns0:c r="I89" s="6" t="str">
         <ns0:v>Service search and filters for Dan, Tate, Dom and Alfie
-Named barber service listings with the existing Fresha route</ns0:v>
+Named barber service listings with the existing Fresha route
+Booking buttons open Amic Studios’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J89" s="6" t="str">
         <ns0:v>Help clients find the barber and service they want before opening the booking page.</ns0:v>
       </ns0:c>
       <ns0:c r="K89" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Amic Studios. it includes service search and filters for Dan, Tate, Dom and Alfie and named barber service listings with the existing Fresha route. the idea is to help clients find the barber and service they want before opening the booking page. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Amic Studios. it includes service search and filters for Dan, Tate, Dom and Alfie and named barber service listings with the existing Fresha route. the idea is to help clients find the barber and service they want before opening the booking page. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L89" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="90" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M89" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/en-GB/a/amic-studios-birstall-2b-stonehill-avenue-ekar337w
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Amic%20Studios%202B%20Stonehill%20Avenue%20Birstall%20Leicester</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="90" ht="210" customHeight="1">
       <ns0:c r="A90" s="6" t="n">
         <ns0:v>84</ns0:v>
       </ns0:c>
@@ -3492,19 +3955,24 @@
       <ns0:c r="I90" s="6" t="str">
         <ns0:v>Service selector including Gel polish - one colour and Removals with new set
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open IRL Nails and Beauty’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J90" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K90" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for IRL Nails and Beauty. visitors can compare options such as Gel polish - one colour and Removals with new set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for IRL Nails and Beauty. visitors can compare options such as Gel polish - one colour and Removals with new set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L90" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="91" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M90" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/irl-nails-and-beauty-leicester-naver-road-mumgjpxd
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Naver%20Road%2C%20Leicester%20LE19%204DG</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="91" ht="210" customHeight="1">
       <ns0:c r="A91" s="6" t="n">
         <ns0:v>85</ns0:v>
       </ns0:c>
@@ -3530,19 +3998,24 @@
       <ns0:c r="I91" s="6" t="str">
         <ns0:v>Service selector including Ladies Cut &amp; Blow Dry and Gents Cut
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Hair By Wikki’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J91" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K91" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Hair By Wikki. visitors can compare options such as Ladies Cut &amp; Blow Dry and Gents Cut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Hair By Wikki. visitors can compare options such as Ladies Cut &amp; Blow Dry and Gents Cut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L91" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="92" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M91" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/hair-by-wikki-leicester-50a-hinckley-road-mtq61cm7
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=50A%20Hinckley%20Road%2C%20Leicester%20LE3%200RB</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="92" ht="210" customHeight="1">
       <ns0:c r="A92" s="6" t="n">
         <ns0:v>86</ns0:v>
       </ns0:c>
@@ -3563,19 +4036,25 @@
       <ns0:c r="H92" s="6" t="str"/>
       <ns0:c r="I92" s="6" t="str">
         <ns0:v>Searchable menu selection with burger, wrap, pizza and grill filters
-Existing Deliveroo link alongside location information</ns0:v>
+Existing Deliveroo link alongside location information
+Direct link to Deliveroo ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J92" s="6" t="str">
         <ns0:v>Help customers find a meal category quickly before checking the ordering menu.</ns0:v>
       </ns0:c>
       <ns0:c r="K92" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for LALA’S Restaurant. it includes searchable menu selection with burger, wrap, pizza and grill filters and existing Deliveroo link alongside location information. the idea is to help customers find a meal category quickly before checking the ordering menu. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for LALA’S Restaurant. it includes searchable menu selection with burger, wrap, pizza and grill filters and existing Deliveroo link alongside location information. the idea is to help customers find a meal category quickly before checking the ordering menu. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L92" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="93" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M92" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/leicester/leicester-city-centre/lalas-restaurant-17-halford-street
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Lalas%20Restaurant%2017%20Halford%20Street%20Leicester%20LE1%201JA</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="93" ht="210" customHeight="1">
       <ns0:c r="A93" s="6" t="n">
         <ns0:v>87</ns0:v>
       </ns0:c>
@@ -3597,19 +4076,24 @@
       <ns0:c r="I93" s="6" t="str">
         <ns0:v>Service selector including Cut and Finish and Cut and Finish w/ Beard Trim
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open VOSS. Barbering and Men’s Hair Specialist’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J93" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K93" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for VOSS. Barbering and Men’s Hair Specialist. visitors can compare options such as Cut and Finish and Cut and Finish w/ Beard Trim, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for VOSS. Barbering and Men’s Hair Specialist. visitors can compare options such as Cut and Finish and Cut and Finish w/ Beard Trim, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L93" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="94" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M93" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/93977_voss-barbering-and-mens-hair-specialist_barber_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=A%20Barber%20Room%20181%20Clarendon%20Park%20Road%20Leicester%20LE2%203AJ</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="94" ht="210" customHeight="1">
       <ns0:c r="A94" s="6" t="n">
         <ns0:v>88</ns0:v>
       </ns0:c>
@@ -3630,19 +4114,25 @@
       <ns0:c r="H94" s="6" t="str"/>
       <ns0:c r="I94" s="6" t="str">
         <ns0:v>Searchable hot and cold mezze selection
-Existing Uber Eats link and Gallowtree Gate visit information</ns0:v>
+Existing Uber Eats link and Gallowtree Gate visit information
+Direct link to Uber Eats ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J94" s="6" t="str">
         <ns0:v>Help visitors explore mezze choices before ordering or visiting.</ns0:v>
       </ns0:c>
       <ns0:c r="K94" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Falafelland. it includes searchable hot and cold mezze selection and existing Uber Eats link and Gallowtree Gate visit information. the idea is to help visitors explore mezze choices before ordering or visiting. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Falafelland. it includes searchable hot and cold mezze selection and existing Uber Eats link and Gallowtree Gate visit information. the idea is to help visitors explore mezze choices before ordering or visiting. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L94" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="95" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M94" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/falafel-land/yf2cbpeTV4ivf_iQszd5ww
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Falafel%20Land%2045%2047%20Gallowtree%20Gate%20Leicester%20LE1%205AD</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="95" ht="210" customHeight="1">
       <ns0:c r="A95" s="6" t="n">
         <ns0:v>89</ns0:v>
       </ns0:c>
@@ -3664,19 +4154,24 @@
       <ns0:c r="I95" s="6" t="str">
         <ns0:v>Service selector including Beard Trim and Condition and Taper fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Amo’s Cutthroat’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J95" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K95" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Amo’s Cutthroat. visitors can compare options such as Beard Trim and Condition and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Amo’s Cutthroat. visitors can compare options such as Beard Trim and Condition and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L95" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="96" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M95" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/155778_amos-cutthroat_barber_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=154%20East%20Park%20Road%20Leicester%20LE5%204QB</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="96" ht="210" customHeight="1">
       <ns0:c r="A96" s="6" t="n">
         <ns0:v>90</ns0:v>
       </ns0:c>
@@ -3698,19 +4193,24 @@
       <ns0:c r="I96" s="6" t="str">
         <ns0:v>Service selector including Haircut with Martin and Haircut with Alex
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Til Next Time Barbershop’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J96" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K96" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Til Next Time Barbershop. visitors can compare options such as Haircut with Martin and Haircut with Alex, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Til Next Time Barbershop. visitors can compare options such as Haircut with Martin and Haircut with Alex, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L96" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="97" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M96" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/34218_til-next-time-barbershop_barber_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=6B%20Hotel%20Street%20Leicester%20LE1%205AW</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="97" ht="210" customHeight="1">
       <ns0:c r="A97" s="6" t="n">
         <ns0:v>91</ns0:v>
       </ns0:c>
@@ -3735,19 +4235,27 @@
       </ns0:c>
       <ns0:c r="I97" s="6" t="str">
         <ns0:v>Searchable Uyghur menu across noodles, dumplings, skewers and vegetables
-Links to the existing business and ordering pages</ns0:v>
+Links to the existing business and ordering pages
+Direct link to Uber Eats ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J97" s="6" t="str">
         <ns0:v>Help diners explore unfamiliar dishes and find the next step for a visit or order.</ns0:v>
       </ns0:c>
       <ns0:c r="K97" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Karamay Hot Pot. it includes searchable Uyghur menu across noodles, dumplings, skewers and vegetables and links to the existing business and ordering pages. the idea is to help diners explore unfamiliar dishes and find the next step for a visit or order. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Karamay Hot Pot. it includes searchable Uyghur menu across noodles, dumplings, skewers and vegetables and links to the existing business and ordering pages. the idea is to help diners explore unfamiliar dishes and find the next step for a visit or order. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L97" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="98" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M97" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/karamay-uyghur-cuisine-%E5%85%8B%E6%8B%89%E7%8E%9B%E4%BE%9D%E6%96%B0%E7%96%86%E9%A4%90%E5%8E%85/ABmj9kB5QTisZFhkrFZD3Q
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Karamay%2063%20London%20Road%20Leicester%20LE2%200PE
+Tap to call +441162918060: tel:+441162918060</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="98" ht="210" customHeight="1">
       <ns0:c r="A98" s="6" t="n">
         <ns0:v>92</ns0:v>
       </ns0:c>
@@ -3773,19 +4281,24 @@
       <ns0:c r="I98" s="6" t="str">
         <ns0:v>Service selector including BIAB Manicure and BIAB Manicure &amp; Simple Nail Art
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open By Nancy’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J98" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K98" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for By Nancy. visitors can compare options such as BIAB Manicure and BIAB Manicure &amp; Simple Nail Art, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for By Nancy. visitors can compare options such as BIAB Manicure and BIAB Manicure &amp; Simple Nail Art, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L98" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="99" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M98" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/by-nancy-south-wigston-2-orange-street-vpssmvw9
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=2%20Orange%20Street%20Belle%20Ame%20Salon%2C%20South%20Wigston%20LE18%204QB</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="99" ht="210" customHeight="1">
       <ns0:c r="A99" s="6" t="n">
         <ns0:v>93</ns0:v>
       </ns0:c>
@@ -3811,19 +4324,24 @@
       <ns0:c r="I99" s="6" t="str">
         <ns0:v>Service selector including Double classic infill and Korean lash lift
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open elmaybeauty.x’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J99" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K99" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for elmaybeauty.x. visitors can compare options such as Double classic infill and Korean lash lift, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for elmaybeauty.x. visitors can compare options such as Double classic infill and Korean lash lift, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L99" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="100" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M99" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/elmaybeauty-x-wigston-hazelwood-road-suc2o819
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Hazelwood%20Road%2C%20Wigston%20LE18%204LS</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="100" ht="210" customHeight="1">
       <ns0:c r="A100" s="6" t="n">
         <ns0:v>94</ns0:v>
       </ns0:c>
@@ -3850,19 +4368,23 @@
       </ns0:c>
       <ns0:c r="I100" s="6" t="str">
         <ns0:v>Visit checklist for a chosen date and group size
-Questions covering Belgian beers, weekend plans, access and arrival</ns0:v>
+Questions covering Belgian beers, weekend plans, access and arrival
+Tap-to-call link to the business phone number</ns0:v>
       </ns0:c>
       <ns0:c r="J100" s="6" t="str">
         <ns0:v>Help groups organise what to check with the venue before a visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K100" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Café Bruxelles. it includes visit checklist for a chosen date and group size and questions covering Belgian beers, weekend plans, access and arrival. the idea is to help groups organise what to check with the venue before a visit. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Café Bruxelles. it includes visit checklist for a chosen date and group size and questions covering Belgian beers, weekend plans, access and arrival. the idea is to help groups organise what to check with the venue before a visit. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L100" s="6" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
       </ns0:c>
-    </ns0:row>
-    <ns0:row r="101" ht="150" customHeight="1">
+      <ns0:c r="M100" s="6" t="str">
+        <ns0:v>Tap to call +441162531325: tel:+441162531325</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="101" ht="210" customHeight="1">
       <ns0:c r="A101" s="6" t="n">
         <ns0:v>95</ns0:v>
       </ns0:c>
@@ -3888,19 +4410,27 @@
       </ns0:c>
       <ns0:c r="I101" s="6" t="str">
         <ns0:v>Filter for vegetarian menu listings
-Item detail views across breakfast, paninis, wraps and salads</ns0:v>
+Item detail views across breakfast, paninis, wraps and salads
+Direct link to Deliveroo ordering menu
+Tap-to-call link to the business phone number
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J101" s="6" t="str">
         <ns0:v>Help customers narrow down lunch options before checking ingredients and ordering.</ns0:v>
       </ns0:c>
       <ns0:c r="K101" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Deliish. it includes filter for vegetarian menu listings and item detail views across breakfast, paninis, wraps and salads. the idea is to help customers narrow down lunch options before checking ingredients and ordering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Deliish. it includes filter for vegetarian menu listings and item detail views across breakfast, paninis, wraps and salads. the idea is to help customers narrow down lunch options before checking ingredients and ordering. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L101" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="102" ht="150" customHeight="1">
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M101" s="6" t="str">
+        <ns0:v>Deliveroo ordering menu: https://deliveroo.co.uk/menu/Leicester/leicester-city-centre/deliish
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Deliish%206-8%20Rutland%20Street%20Leicester%20LE1%201RA
+Tap to call +441162628674: tel:+441162628674</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="102" ht="210" customHeight="1">
       <ns0:c r="A102" s="6" t="n">
         <ns0:v>96</ns0:v>
       </ns0:c>
@@ -3922,19 +4452,24 @@
       <ns0:c r="I102" s="6" t="str">
         <ns0:v>Service selector including Brow architecture · mapping and shaping and Lash Removal
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Ink&amp;Beauty Factory’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J102" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K102" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Ink&amp;Beauty Factory. visitors can compare options such as Brow architecture · mapping and shaping and Lash Removal, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Ink&amp;Beauty Factory. visitors can compare options such as Brow architecture · mapping and shaping and Lash Removal, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L102" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="103" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M102" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/177384_ink-beauty-factory_brows-lashes_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=91%20Hopefield%20Road%20Leicester%20LE3%202BL</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="103" ht="210" customHeight="1">
       <ns0:c r="A103" s="6" t="n">
         <ns0:v>97</ns0:v>
       </ns0:c>
@@ -3960,19 +4495,24 @@
       <ns0:c r="I103" s="6" t="str">
         <ns0:v>Service selector including Haircut (Leicester) and Haircut and beard trim
 Listed prices and appointment lengths update with the selected service
-Link to the existing Fresha booking page</ns0:v>
+Booking buttons open Shortys - Leicester’s existing Fresha booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J103" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K103" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Shortys - Leicester. visitors can compare options such as Haircut (Leicester) and Haircut and beard trim, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Shortys - Leicester. visitors can compare options such as Haircut (Leicester) and Haircut and beard trim, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L103" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="104" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M103" s="6" t="str">
+        <ns0:v>Fresha booking profile: https://www.fresha.com/a/shortys-leicester-leicester-hair-1rd-42-44-rutland-street-jq5wg2jp
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Hair%401rd%2C%2042-44%20Rutland%20Street%2C%20Leicester%20LE1%201RD</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="104" ht="210" customHeight="1">
       <ns0:c r="A104" s="6" t="n">
         <ns0:v>98</ns0:v>
       </ns0:c>
@@ -3998,19 +4538,24 @@
       <ns0:c r="I104" s="6" t="str">
         <ns0:v>Service selector including SkinFade and Classic Haircut
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Taurus barbers’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J104" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K104" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Taurus barbers. visitors can compare options such as SkinFade and Classic Haircut, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Taurus barbers. visitors can compare options such as SkinFade and Classic Haircut, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L104" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="105" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M104" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/181375_taurus-barbers_barber_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=27%20Francis%20Street%20Stoneygate%20Leicester%20LE2%202BE</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="105" ht="210" customHeight="1">
       <ns0:c r="A105" s="6" t="n">
         <ns0:v>99</ns0:v>
       </ns0:c>
@@ -4032,19 +4577,24 @@
       <ns0:c r="I105" s="6" t="str">
         <ns0:v>Service selector including Haircut and Skin-Fade/Taper fade
 Listed prices and appointment lengths update with the selected service
-Link to the existing Booksy booking page</ns0:v>
+Booking buttons open Hair Roots &amp; Co’s existing Booksy booking profile
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J105" s="6" t="str">
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K105" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Hair Roots &amp; Co. visitors can compare options such as Haircut and Skin-Fade/Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Hair Roots &amp; Co. visitors can compare options such as Haircut and Skin-Fade/Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L105" s="6" t="str">
-        <ns0:v>Prices and appointment lengths reflect saved provider listings. Selections are not transferred to the booking provider; no live availability is shown. Email signup is a demonstration.</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="106" ht="150" customHeight="1">
+        <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M105" s="6" t="str">
+        <ns0:v>Booksy booking profile: https://booksy.com/en-gb/187348_hair-roots-co_barber_31021_leicester
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=749%20Aylestone%20Road%20Leicester</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="106" ht="210" customHeight="1">
       <ns0:c r="A106" s="6" t="n">
         <ns0:v>100</ns0:v>
       </ns0:c>
@@ -4065,16 +4615,22 @@
       <ns0:c r="H106" s="6" t="str"/>
       <ns0:c r="I106" s="6" t="str">
         <ns0:v>Searchable brunch selection grouped into bowls, toast, brunch and bread
-Existing ordering route and Braunstone Gate visit information</ns0:v>
+Existing ordering route and Braunstone Gate visit information
+Direct link to Uber Eats ordering menu
+Directions button opens the business location in Google Maps</ns0:v>
       </ns0:c>
       <ns0:c r="J106" s="6" t="str">
         <ns0:v>Help visitors find the kind of brunch they fancy before visiting or ordering.</ns0:v>
       </ns0:c>
       <ns0:c r="K106" s="6" t="str">
-        <ns0:v>i’ve put together a website preview for Ninety Six Degrees. it includes searchable brunch selection grouped into bowls, toast, brunch and bread and existing ordering route and Braunstone Gate visit information. the idea is to help visitors find the kind of brunch they fancy before visiting or ordering. this is a preview to show the idea, with any forms still in demo mode.</ns0:v>
+        <ns0:v>i’ve put together a website preview for Ninety Six Degrees. it includes searchable brunch selection grouped into bowls, toast, brunch and bread and existing ordering route and Braunstone Gate visit information. the idea is to help visitors find the kind of brunch they fancy before visiting or ordering. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L106" s="6" t="str">
-        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
+        <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
+      </ns0:c>
+      <ns0:c r="M106" s="6" t="str">
+        <ns0:v>Uber Eats ordering menu: https://www.ubereats.com/gb/store/ninety-six-degrees/HJ1Ch8tHWh-rSsmDa1Wn1w
+Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Ninety%20Six%20Degrees%2042%20Braunstone%20Gate%20Leicester%20LE3%205LG</ns0:v>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>
@@ -4182,7 +4738,7 @@
   </ns0:hyperlinks>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ns0:tableParts count="1">
-    <ns0:tablePart ns1:id="Ra09ae118ee1f481b"/>
+    <ns0:tablePart ns1:id="R0e0959c6f8474b9a"/>
   </ns0:tableParts>
 </ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
Update first 100 contacts with sourced gap research
</commit_message>
<xml_diff>
--- a/website-demos/business-contacts.xlsx
+++ b/website-demos/business-contacts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="R92b2a0cdd0cf4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="First 100" sheetId="1" r:id="Rd3090be7a0ab4d5b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -351,7 +351,7 @@
     </ns0:row>
     <ns0:row r="3">
       <ns0:c r="A3" t="str">
-        <ns0:v>25 October 2026. All 100 reconciled: 52 from the 414 master, 48 later additions. 81 phone / 19 email / 20 owner, director or operator leads. Roles and caveats in N:T.</ns0:v>
+        <ns0:v>25 October 2026. All 100 reconciled: 52 from the 414 master, 48 later additions. 86 phone / 20 email / 30 owner, director or operator leads. Gap follow-up completed. Roles and caveats in N:T.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="4">
@@ -453,7 +453,7 @@
         <ns0:v>Help visitors explain the look and appointment they have in mind before calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K7" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Andrew Leonards Hairdressing. it includes service guide for cuts, colour and occasions and appointment discussion notes with a preferred date. the idea is to help visitors explain the look and appointment they have in mind before calling. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Andrew Leonards Hairdressing. It includes service guide for cuts, colour and occasions and appointment discussion notes with a preferred date. The idea is to help visitors explain the look and appointment they have in mind before calling. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L7" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -478,10 +478,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S7" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T7" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="8" ht="210" customHeight="1">
@@ -516,7 +516,7 @@
         <ns0:v>Make a catering conversation easier to start with the key details already together.</ns0:v>
       </ns0:c>
       <ns0:c r="K8" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Bar Sandwich. it includes lunch categories for sandwiches, soup and buffets and group lunch planner with headcount, date and dietary questions. the idea is to make a catering conversation easier to start with the key details already together. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Bar Sandwich. It includes lunch categories for sandwiches, soup and buffets and group lunch planner with headcount, date and dietary questions. The idea is to make a catering conversation easier to start with the key details already together. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L8" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -541,10 +541,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S8" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T8" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="9" ht="210" customHeight="1">
@@ -564,7 +564,7 @@
         <ns0:v>https://venturasolutions.co.uk/5-coats/</ns0:v>
       </ns0:c>
       <ns0:c r="F9" s="7" t="str">
-        <ns0:v>Phone 07887 347304: BID exact19HighStreet entry; conflicting directory number remains to resolve. Phone 07887 304347: Conflicting directory number; confirm before use.</ns0:v>
+        <ns0:v>Phone 07887 347304: BID exact19HighStreet entry; conflicting directory number remains to resolve. Phone 07887 304347: Conflicting directory number; confirm before use. </ns0:v>
       </ns0:c>
       <ns0:c r="G9" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -582,7 +582,7 @@
         <ns0:v>Let people pick out a lunch or cake idea before visiting High Street.</ns0:v>
       </ns0:c>
       <ns0:c r="K9" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for 5 Coats. it includes lunch, cake and drink category filters and café shortlist with item details and a copyable visit note. the idea is to let people pick out a lunch or cake idea before visiting High Street. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for 5 Coats. It includes lunch, cake and drink category filters and café shortlist with item details and a copyable visit note. The idea is to let people pick out a lunch or cake idea before visiting High Street. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L9" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -607,10 +607,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S9" s="7" t="str">
-        <ns0:v>hey angelina,</ns0:v>
+        <ns0:v>Hi Angelina,</ns0:v>
       </ns0:c>
       <ns0:c r="T9" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="10" ht="210" customHeight="1">
@@ -630,7 +630,7 @@
         <ns0:v>https://venturasolutions.co.uk/chloe-nails/</ns0:v>
       </ns0:c>
       <ns0:c r="F10" s="7" t="str">
-        <ns0:v>Phone 07436 856789: Retained September directory phone; not freshly visible/confirmed.</ns0:v>
+        <ns0:v>Phone 07436 856789: Retained September directory phone; not freshly visible/confirmed. </ns0:v>
       </ns0:c>
       <ns0:c r="G10" s="7" t="str">
         <ns0:v>2026-09-26</ns0:v>
@@ -647,7 +647,7 @@
         <ns0:v>Help clients think through their treatment and removal questions before opening Booksy.</ns0:v>
       </ns0:c>
       <ns0:c r="K10" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Chloe's Nails. it includes acrylic, BIAB, gel and pedicure treatment guide and existing product guidance, nail inspiration gallery and Booksy links. the idea is to help clients think through their treatment and removal questions before opening Booksy. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Chloe's Nails. It includes acrylic, BIAB, gel and pedicure treatment guide and existing product guidance, nail inspiration gallery and Booksy links. The idea is to help clients think through their treatment and removal questions before opening Booksy. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L10" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -672,10 +672,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S10" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T10" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="11" ht="210" customHeight="1">
@@ -710,7 +710,7 @@
         <ns0:v>Help customers explain the products and quantities they want to ask the counter about.</ns0:v>
       </ns0:c>
       <ns0:c r="K11" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Tomasz Kotula Butcher. it includes product enquiry list with quantities across Polish deli categories and english or Polish enquiry summaries with collection and delivery questions. the idea is to help customers explain the products and quantities they want to ask the counter about. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Tomasz Kotula Butcher. It includes product enquiry list with quantities across Polish deli categories and English or Polish enquiry summaries with collection and delivery questions. The idea is to help customers explain the products and quantities they want to ask the counter about. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L11" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -735,10 +735,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S11" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T11" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="12" ht="210" customHeight="1">
@@ -773,7 +773,7 @@
         <ns0:v>Give visitors a starting point for browsing the shop or finding a gift.</ns0:v>
       </ns0:c>
       <ns0:c r="K12" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for The Very Bazaar. it includes discovery guide across jewellery, crystals, clothing, gifts and incense and personal shopping or gift choice with a copyable visit list. the idea is to give visitors a starting point for browsing the shop or finding a gift. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for The Very Bazaar. It includes discovery guide across jewellery, crystals, clothing, gifts and incense and personal shopping or gift choice with a copyable visit list. The idea is to give visitors a starting point for browsing the shop or finding a gift. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L12" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -798,10 +798,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S12" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T12" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="13" ht="210" customHeight="1">
@@ -820,7 +820,9 @@
       <ns0:c r="E13" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/croft-hotel/</ns0:v>
       </ns0:c>
-      <ns0:c r="F13" s="7" t="str"/>
+      <ns0:c r="F13" s="7" t="str">
+        <ns0:v>Historical Croft Hotel emails were explicitly marked obsolete by the directory and excluded.</ns0:v>
+      </ns0:c>
       <ns0:c r="G13" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
       </ns0:c>
@@ -837,7 +839,7 @@
         <ns0:v>Help guests compare room types before checking current dates and rates.</ns0:v>
       </ns0:c>
       <ns0:c r="K13" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Croft Hotel. it includes room search and filters for single, twin, double and family options and bed arrangements beside links to the existing Booking.com profile. the idea is to help guests compare room types before checking current dates and rates. the site also links to your Booking.com page to check room availability. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Croft Hotel. It includes room search and filters for single, twin, double and family options and bed arrangements beside links to the existing Booking.com profile. The idea is to help guests compare room types before checking current dates and rates. The site also links to your Booking.com page to check room availability. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L13" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -863,10 +865,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S13" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T13" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="14" ht="210" customHeight="1">
@@ -886,7 +888,7 @@
         <ns0:v>https://venturasolutions.co.uk/duffys/</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="7" t="str">
-        <ns0:v>Email info@firebugbar.co.uk: Festival venue-space contact for Duffy’s; shared Firebug address, not Matt’s verified personal inbox. Purpose-specific contact.</ns0:v>
+        <ns0:v>Email info@firebugbar.co.uk: Festival venue-space contact for Duffy’s; shared Firebug address, not Matt’s verified personal inbox. Purpose-specific contact. </ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="7" t="str">
         <ns0:v>2026-10-10; 2026-10-25</ns0:v>
@@ -904,7 +906,7 @@
         <ns0:v>Help visitors find a relevant gig and organise the questions they need to ask.</ns0:v>
       </ns0:c>
       <ns0:c r="K14" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Duffy's. it includes gig list searchable by artist and filterable by month and gig details and a visit note for group, access or ticket questions. the idea is to help visitors find a relevant gig and organise the questions they need to ask. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Duffy's. It includes gig list searchable by artist and filterable by month and gig details and a visit note for group, access or ticket questions. The idea is to help visitors find a relevant gig and organise the questions they need to ask. Customers can open the business location in Google Maps for directions. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L14" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -929,7 +931,7 @@
         <ns0:v>info@firebugbar.co.uk: Festival venue-space contact for Duffy’s; shared Firebug address, not Matt’s verified personal inbox. Purpose-specific contact.</ns0:v>
       </ns0:c>
       <ns0:c r="S14" s="7" t="str">
-        <ns0:v>hey matt,</ns0:v>
+        <ns0:v>Hi Matt,</ns0:v>
       </ns0:c>
       <ns0:c r="T14" s="7" t="str">
         <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
@@ -951,7 +953,9 @@
       <ns0:c r="E15" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/sams-beauty-den/</ns0:v>
       </ns0:c>
-      <ns0:c r="F15" s="7" t="str"/>
+      <ns0:c r="F15" s="7" t="str">
+        <ns0:v>Phone +44 7932 067588: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G15" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -968,7 +972,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K15" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Sam’s Beauty Den in Butchers Salon. visitors can compare options such as Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Sam’s Beauty Den in Butchers Salon. Visitors can compare options such as Eyebrow, upper lip &amp; chin wax and Relaxing Full Body Massage, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L15" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -991,10 +995,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S15" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T15" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="16" ht="210" customHeight="1">
@@ -1029,7 +1033,7 @@
         <ns0:v>Help diners put a few Japanese dishes together before their visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K16" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Mitsuki. it includes sushi, bento and ramen category filters and dish detail views and a copyable favourites list. the idea is to help diners put a few Japanese dishes together before their visit. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Mitsuki. It includes sushi, bento and ramen category filters and dish detail views and a copyable favourites list. The idea is to help diners put a few Japanese dishes together before their visit. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L16" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -1038,14 +1042,14 @@
         <ns0:v>Tap to call 01162554805: tel:01162554805</ns0:v>
       </ns0:c>
       <ns0:c r="N16" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Chee Kwan Chang</ns0:v>
       </ns0:c>
       <ns0:c r="O16" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. No current public owner or manager verified in the logged search.</ns0:v>
+        <ns0:v>Active company director. MITSUKI GEN LIMITED; exact 109 London Road. Active appointment follows earlier resignation. Operational buying responsibility is not established.</ns0:v>
       </ns0:c>
       <ns0:c r="P16" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-27</ns0:v>
+        <ns0:v>https://find-and-update.company-information.service.gov.uk/company/13573025/officers
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q16" s="7" t="str">
         <ns0:v>None verified</ns0:v>
@@ -1054,10 +1058,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S16" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T16" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="17" ht="210" customHeight="1">
@@ -1076,7 +1080,9 @@
       <ns0:c r="E17" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/kurda/</ns0:v>
       </ns0:c>
-      <ns0:c r="F17" s="7" t="str"/>
+      <ns0:c r="F17" s="7" t="str">
+        <ns0:v>A secondary company directory suggests Kurdo Nawzad Nwri; primary verification was unavailable. Not adopted as a verified owner.</ns0:v>
+      </ns0:c>
       <ns0:c r="G17" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
       </ns0:c>
@@ -1094,7 +1100,7 @@
         <ns0:v>Help groups decide what to ask about before speaking to the restaurant.</ns0:v>
       </ns0:c>
       <ns0:c r="K17" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Kurda Restaurant. it includes sharing platter guide organised by group size and meal discussion note with food choice, guest count and preferred date. the idea is to help groups decide what to ask about before speaking to the restaurant. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Kurda Restaurant. It includes sharing platter guide organised by group size and meal discussion note with food choice, guest count and preferred date. The idea is to help groups decide what to ask about before speaking to the restaurant. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L17" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1121,10 +1127,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S17" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T17" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="18" ht="210" customHeight="1">
@@ -1144,7 +1150,7 @@
         <ns0:v>https://venturasolutions.co.uk/tatra/</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="7" t="str">
-        <ns0:v>Email tatraeasterncorner@gmail.com: Publicdirectoryemail also indexedbyTripadvisor; deliveryuntested.</ns0:v>
+        <ns0:v>Email tatraeasterncorner@gmail.com: Publicdirectoryemail also indexedbyTripadvisor; deliveryuntested. </ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1164,7 +1170,7 @@
         <ns0:v>Make it easier to start a conversation about a celebration or catering enquiry.</ns0:v>
       </ns0:c>
       <ns0:c r="K18" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Tatra Eastern Corner. it includes menu sections with dish photographs and event enquiry outline covering occasion, guests, food and collection preferences. the idea is to make it easier to start a conversation about a celebration or catering enquiry. the site also links to your existing table request page. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Tatra Eastern Corner. It includes menu sections with dish photographs and event enquiry outline covering occasion, guests, food and collection preferences. The idea is to make it easier to start a conversation about a celebration or catering enquiry. The site also links to your existing table request page. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L18" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1191,10 +1197,10 @@
         <ns0:v>tatraeasterncorner@gmail.com: Publicdirectoryemail also indexedbyTripadvisor; deliveryuntested.</ns0:v>
       </ns0:c>
       <ns0:c r="S18" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T18" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="19" ht="210" customHeight="1">
@@ -1214,7 +1220,7 @@
         <ns0:v>https://venturasolutions.co.uk/palya/</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="7" t="str">
-        <ns0:v>Email contact@palyascatering.co.uk: Direct customer contact. Email support@palyascatering.co.uk: App support address; not necessarily sales/owner.</ns0:v>
+        <ns0:v>Email contact@palyascatering.co.uk: Direct customer contact. Email support@palyascatering.co.uk: App support address; not necessarily sales/owner. </ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="7" t="str">
         <ns0:v>2026-10-11</ns0:v>
@@ -1234,7 +1240,7 @@
         <ns0:v>Bring the important event details together before a catering conversation.</ns0:v>
       </ns0:c>
       <ns0:c r="K19" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for PALYA'S Catering. it includes daily versus weekly and monthly meal sections and catering brief with occasion, date, guest count, location and dietary requests. the idea is to bring the important event details together before a catering conversation. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for PALYA'S Catering. It includes daily versus weekly and monthly meal sections and catering brief with occasion, date, guest count, location and dietary requests. The idea is to bring the important event details together before a catering conversation. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L19" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1261,10 +1267,10 @@
 support@palyascatering.co.uk: App support address; not necessarily sales/owner.</ns0:v>
       </ns0:c>
       <ns0:c r="S19" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T19" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="20" ht="210" customHeight="1">
@@ -1301,7 +1307,7 @@
         <ns0:v>Help customers narrow down a café visit and explain what they need when calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K20" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Piero Snack Bar. it includes breakfast, lunch and drinks filters and café call outline with visit type, group size and questions. the idea is to help customers narrow down a café visit and explain what they need when calling. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Piero Snack Bar. It includes breakfast, lunch and drinks filters and café call outline with visit type, group size and questions. The idea is to help customers narrow down a café visit and explain what they need when calling. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L20" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1328,10 +1334,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S20" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T20" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="21" ht="210" customHeight="1">
@@ -1351,7 +1357,7 @@
         <ns0:v>https://venturasolutions.co.uk/country-fayre/</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="7" t="str">
-        <ns0:v>Email country-fayre@btconnect.com: Directory-published email only; owner confirmation required.</ns0:v>
+        <ns0:v>Email country-fayre@btconnect.com: Directory-published email only; owner confirmation required. </ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1370,7 +1376,7 @@
         <ns0:v>Separate everyday purchases from trade and celebration enquiries.</ns0:v>
       </ns0:c>
       <ns0:c r="K21" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Country Fayre Foods. it includes product range explorer for cheese, meats, pastry and dairy and different enquiry paths for home shopping, trade supply and celebration cheese cakes. the idea is to separate everyday purchases from trade and celebration enquiries. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Country Fayre Foods. It includes product range explorer for cheese, meats, pastry and dairy and different enquiry paths for home shopping, trade supply and celebration cheese cakes. The idea is to separate everyday purchases from trade and celebration enquiries. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L21" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -1396,7 +1402,7 @@
         <ns0:v>country-fayre@btconnect.com: Directory-published email only; owner confirmation required.</ns0:v>
       </ns0:c>
       <ns0:c r="S21" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T21" s="7" t="str">
         <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
@@ -1436,7 +1442,7 @@
         <ns0:v>Help customers narrow down dishes and prepare a clear meal enquiry.</ns0:v>
       </ns0:c>
       <ns0:c r="K22" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Taste of China. it includes searchable rice and noodle menu selection and meal note with group size, visit type and questions. the idea is to help customers narrow down dishes and prepare a clear meal enquiry. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Taste of China. It includes searchable rice and noodle menu selection and meal note with group size, visit type and questions. The idea is to help customers narrow down dishes and prepare a clear meal enquiry. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L22" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1447,14 +1453,14 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Taste+of+China+25+High+Street+Leicester+LE1+4FP</ns0:v>
       </ns0:c>
       <ns0:c r="N22" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Cheong Kee Tang; Suzanna Chiu Yee Wilkins</ns0:v>
       </ns0:c>
       <ns0:c r="O22" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. No public owner or manager with a confirmed current role found in scoped search.</ns0:v>
+        <ns0:v>Active company director. Exact 25 High Street. Suzanna has an active reappointment dated 9 June 2026. Operational buying responsibility is not established.</ns0:v>
       </ns0:c>
       <ns0:c r="P22" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-26</ns0:v>
+        <ns0:v>https://find-and-update.company-information.service.gov.uk/company/07281955/officers
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q22" s="7" t="str">
         <ns0:v>Cheong Kee Tang (Active company director at exact business address; current daily role unconfirmed.); Suzanna Chiu Yee Wilkins (Active director appointed9 June2026, exact business address; not assumed website buyer.)</ns0:v>
@@ -1463,10 +1469,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S22" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T22" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="23" ht="210" customHeight="1">
@@ -1486,7 +1492,7 @@
         <ns0:v>https://venturasolutions.co.uk/noodle-house/</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="7" t="str">
-        <ns0:v>Phone 0116 291 5254: Exact-address current search results also corroborated by RestaurantGuru; another old directory number conflicts, confirm before use.</ns0:v>
+        <ns0:v>Phone 0116 291 5254: Exact-address current search results also corroborated by RestaurantGuru; another old directory number conflicts, confirm before use. </ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1504,7 +1510,7 @@
         <ns0:v>Help people coordinate a group meal before checking the real ordering menu.</ns0:v>
       </ns0:c>
       <ns0:c r="K23" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Noodle House. it includes box mix, noodle, rice and soup filters and group shortlist with quantities for each selected dish. the idea is to help people coordinate a group meal before checking the real ordering menu. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Noodle House. It includes box mix, noodle, rice and soup filters and group shortlist with quantities for each selected dish. The idea is to help people coordinate a group meal before checking the real ordering menu. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L23" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1530,10 +1536,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S23" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T23" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="24" ht="210" customHeight="1">
@@ -1553,7 +1559,7 @@
         <ns0:v>https://venturasolutions.co.uk/paper-wings/</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="7" t="str">
-        <ns0:v>Email admin@paperwingscafe.co.uk: Official hire enquiry inbox.</ns0:v>
+        <ns0:v>Email admin@paperwingscafe.co.uk: Official hire enquiry inbox. </ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1571,7 +1577,7 @@
         <ns0:v>Make a workshop, meetup or celebration enquiry easier to explain.</ns0:v>
       </ns0:c>
       <ns0:c r="K24" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Paper Wings Café. it includes separate daytime upstairs and evening whole-space hire options and hire enquiry outline with event type, date, guests, duration and setup needs. the idea is to make a workshop, meetup or celebration enquiry easier to explain. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Paper Wings Café. It includes separate daytime upstairs and evening whole-space hire options and hire enquiry outline with event type, date, guests, duration and setup needs. The idea is to make a workshop, meetup or celebration enquiry easier to explain. Customers can open the business location in Google Maps for directions. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L24" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -1596,10 +1602,10 @@
         <ns0:v>admin@paperwingscafe.co.uk: Official hire enquiry inbox.</ns0:v>
       </ns0:c>
       <ns0:c r="S24" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T24" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="25" ht="210" customHeight="1">
@@ -1618,7 +1624,9 @@
       <ns0:c r="E25" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/oh-so-pretty/</ns0:v>
       </ns0:c>
-      <ns0:c r="F25" s="7" t="str"/>
+      <ns0:c r="F25" s="7" t="str">
+        <ns0:v>Phone +44 7356 019119: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G25" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -1635,7 +1643,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K25" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Oh So Pretty. visitors can compare options such as Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Oh So Pretty. Visitors can compare options such as Gel mani, BIAB &amp; simple design and Gel mani, BIAB &amp; complex design, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L25" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -1645,12 +1653,15 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=4%20Liskeard%20House%2C%20Wigston%20LE18%202GL</ns0:v>
       </ns0:c>
       <ns0:c r="N25" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Krish</ns0:v>
       </ns0:c>
       <ns0:c r="O25" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. </ns0:v>
-      </ns0:c>
-      <ns0:c r="P25" s="7" t="str"/>
+        <ns0:v>Owner. Explicit owner role in booking provider team section; surname not independently verified.</ns0:v>
+      </ns0:c>
+      <ns0:c r="P25" s="7" t="str">
+        <ns0:v>https://www.fresha.com/a/oh-so-pretty-wigston-4-liskeard-house-telbdqpd
+Checked: 2026-10-25</ns0:v>
+      </ns0:c>
       <ns0:c r="Q25" s="7" t="str">
         <ns0:v>Emily (Listed staff member, not a verified owner/decision maker.); Mia (Listed staff member, not a verified owner/decision maker.); Krish (Listed staff member, not a verified owner/decision maker.)</ns0:v>
       </ns0:c>
@@ -1658,10 +1669,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S25" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi Krish,</ns0:v>
       </ns0:c>
       <ns0:c r="T25" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="26" ht="210" customHeight="1">
@@ -1681,7 +1692,7 @@
         <ns0:v>https://venturasolutions.co.uk/fone-plus/</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="7" t="str">
-        <ns0:v>Email info@foneplus.co.uk: Published address; contact page link target is a placeholder.</ns0:v>
+        <ns0:v>Email info@foneplus.co.uk: Published address; contact page link target is a placeholder. </ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1699,7 +1710,7 @@
         <ns0:v>Help customers describe their device problem before contacting the Leicester shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K26" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Fone Plus. it includes repair enquiry guide for phones, tablets, computers and consoles and device model and fault selection with a reviewable enquiry summary. the idea is to help customers describe their device problem before contacting the Leicester shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Fone Plus. It includes repair enquiry guide for phones, tablets, computers and consoles and device model and fault selection with a reviewable enquiry summary. The idea is to help customers describe their device problem before contacting the Leicester shop. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L26" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -1726,10 +1737,10 @@
         <ns0:v>info@foneplus.co.uk: Published address; contact page link target is a placeholder.</ns0:v>
       </ns0:c>
       <ns0:c r="S26" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T26" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="27" ht="210" customHeight="1">
@@ -1749,7 +1760,7 @@
         <ns0:v>https://venturasolutions.co.uk/roma/</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="7" t="str">
-        <ns0:v>Email caferomaenquiries@gmail.com: Claimed listing public email; no message sent.</ns0:v>
+        <ns0:v>Email caferomaenquiries@gmail.com: Claimed listing public email; no message sent. </ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -1769,7 +1780,7 @@
         <ns0:v>Help visitors choose the right service and prepare their dining questions.</ns0:v>
       </ns0:c>
       <ns0:c r="K27" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Roma. it includes brunch, lunch and evening menu sections and dining enquiry notes with occasion and guests, plus the existing Dojo booking link. the idea is to help visitors choose the right service and prepare their dining questions. the site also links to your Dojo page for table bookings. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Roma. It includes brunch, lunch and evening menu sections and dining enquiry notes with occasion and guests, plus the existing Dojo booking link. The idea is to help visitors choose the right service and prepare their dining questions. The site also links to your Dojo page for table bookings. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L27" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1796,10 +1807,10 @@
         <ns0:v>caferomaenquiries@gmail.com: Claimed listing public email; no message sent.</ns0:v>
       </ns0:c>
       <ns0:c r="S27" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T27" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="28" ht="210" customHeight="1">
@@ -1831,7 +1842,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K28" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Cabello Mens Hairsalon. visitors can compare options such as Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Cabello Mens Hairsalon. Visitors can compare options such as Skin Fade/ Taper Fade with Freddie and Skin Fade &amp; Beard Trim with Freddie, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L28" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -1854,10 +1865,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S28" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T28" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="29" ht="210" customHeight="1">
@@ -1892,7 +1903,7 @@
         <ns0:v>Help customers ask for a suitable cut without needing to know every product name.</ns0:v>
       </ns0:c>
       <ns0:c r="K29" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Frank Lee And Son. it includes range guide including beef, pork, lamb and alternative cuts and copyable butcher ask list based on cooking method, people and recipe questions. the idea is to help customers ask for a suitable cut without needing to know every product name. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Frank Lee And Son. It includes range guide including beef, pork, lamb and alternative cuts and copyable butcher ask list based on cooking method, people and recipe questions. The idea is to help customers ask for a suitable cut without needing to know every product name. Customers can open the business location in Google Maps for directions. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L29" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -1901,14 +1912,14 @@
         <ns0:v>Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Frank%20Lee%20and%20Son%20Leicester%20Market%20Food%20Hall%20LE1%205GG</ns0:v>
       </ns0:c>
       <ns0:c r="N29" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Frank Adrian Lee</ns0:v>
       </ns0:c>
       <ns0:c r="O29" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. Public owner or manager not verified.</ns0:v>
+        <ns0:v>Active company director. Matching company name and Leicester business; registered office is an accountant address. Anona Lee resigned in July 2026 and is excluded. Operational buying responsibility is not established.</ns0:v>
       </ns0:c>
       <ns0:c r="P29" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-26</ns0:v>
+        <ns0:v>https://find-and-update.company-information.service.gov.uk/company/01577726/officers
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q29" s="7" t="str">
         <ns0:v>None verified</ns0:v>
@@ -1917,10 +1928,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S29" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T29" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="30" ht="210" customHeight="1">
@@ -1956,7 +1967,7 @@
         <ns0:v>Make unfamiliar dishes easier to explore before asking at the counter.</ns0:v>
       </ns0:c>
       <ns0:c r="K30" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Guilin Street Food. it includes regional noodle guide with English and Chinese dish names and counter checklist for a chosen dish, group size, spice and ingredient questions. the idea is to make unfamiliar dishes easier to explore before asking at the counter. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Guilin Street Food. It includes regional noodle guide with English and Chinese dish names and counter checklist for a chosen dish, group size, spice and ingredient questions. The idea is to make unfamiliar dishes easier to explore before asking at the counter. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L30" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -1982,10 +1993,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S30" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T30" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="31" ht="210" customHeight="1">
@@ -2021,7 +2032,7 @@
         <ns0:v>Help customers arrive with useful questions about choosing and preparing their fish.</ns0:v>
       </ns0:c>
       <ns0:c r="K31" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Leicester Wholesale Fish Direct. it includes fish, shellfish and crustacean range guide and question list covering cooking plan, preparation, weight and handling. the idea is to help customers arrive with useful questions about choosing and preparing their fish. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Leicester Wholesale Fish Direct. It includes fish, shellfish and crustacean range guide and question list covering cooking plan, preparation, weight and handling. The idea is to help customers arrive with useful questions about choosing and preparing their fish. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L31" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -2047,10 +2058,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S31" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T31" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="32" ht="210" customHeight="1">
@@ -2086,7 +2097,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K32" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Violet’s Hair Studio. visitors can compare options such as Cut &amp; Blow Dry and Blow Dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Violet’s Hair Studio. Visitors can compare options such as Cut &amp; Blow Dry and Blow Dry, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L32" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -2109,10 +2120,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S32" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T32" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="33" ht="210" customHeight="1">
@@ -2148,7 +2159,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K33" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Beauty by Mel. visitors can compare options such as Back, Neck &amp; Shoulders and Gel Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Beauty by Mel. Visitors can compare options such as Back, Neck &amp; Shoulders and Gel Toes, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L33" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -2171,10 +2182,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S33" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T33" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="34" ht="210" customHeight="1">
@@ -2205,7 +2216,7 @@
         <ns0:v>Help someone who likes a particular fruit find relevant drinks quickly.</ns0:v>
       </ns0:c>
       <ns0:c r="K34" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Blossom Boba. it includes fruit tea finder for a chosen flavour and single flavour versus flavour pair matching. the idea is to help someone who likes a particular fruit find relevant drinks quickly. the site also links to your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Blossom Boba. It includes fruit tea finder for a chosen flavour and single flavour versus flavour pair matching. The idea is to help someone who likes a particular fruit find relevant drinks quickly. The site also links to your existing Just Eat menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L34" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2230,10 +2241,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S34" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T34" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="35" ht="210" customHeight="1">
@@ -2270,7 +2281,7 @@
         <ns0:v>Help customers put their meal preferences into one clear discussion note.</ns0:v>
       </ns0:c>
       <ns0:c r="K35" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Latin Kitchen. it includes plated food versus handheld food filters and dish planner with side choice, quantities and group questions. the idea is to help customers put their meal preferences into one clear discussion note. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Latin Kitchen. It includes plated food versus handheld food filters and dish planner with side choice, quantities and group questions. The idea is to help customers put their meal preferences into one clear discussion note. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L35" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2297,10 +2308,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S35" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T35" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="36" ht="210" customHeight="1">
@@ -2337,7 +2348,7 @@
         <ns0:v>Help diners keep their favourite dishes together while choosing a meal.</ns0:v>
       </ns0:c>
       <ns0:c r="K36" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Sakura. it includes searchable sushi, bento, noodle and starter selection and copyable meal shortlist with a personal reminder. the idea is to help diners keep their favourite dishes together while choosing a meal. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Sakura. It includes searchable sushi, bento, noodle and starter selection and copyable meal shortlist with a personal reminder. The idea is to help diners keep their favourite dishes together while choosing a meal. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L36" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2364,10 +2375,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S36" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T36" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="37" ht="210" customHeight="1">
@@ -2386,7 +2397,9 @@
       <ns0:c r="E37" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/silver-street-cafe/</ns0:v>
       </ns0:c>
-      <ns0:c r="F37" s="7" t="str"/>
+      <ns0:c r="F37" s="7" t="str">
+        <ns0:v>A similarly named company director was found, but connection to this exact cafe was not established; excluded.</ns0:v>
+      </ns0:c>
       <ns0:c r="G37" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
       </ns0:c>
@@ -2402,7 +2415,7 @@
         <ns0:v>Help visitors organise a breakfast choice before checking it with the café.</ns0:v>
       </ns0:c>
       <ns0:c r="K37" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Silver Street Cafe. it includes search and filters for breakfast plates and hot cobs and copyable café shortlist with group size and beans or tomatoes preference. the idea is to help visitors organise a breakfast choice before checking it with the café. the site also links to your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Silver Street Cafe. It includes search and filters for breakfast plates and hot cobs and copyable café shortlist with group size and beans or tomatoes preference. The idea is to help visitors organise a breakfast choice before checking it with the café. The site also links to your existing Just Eat menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L37" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2427,10 +2440,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S37" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T37" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="38" ht="210" customHeight="1">
@@ -2450,7 +2463,7 @@
         <ns0:v>https://venturasolutions.co.uk/the-beauty-lab-thurmaston/</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="7" t="str">
-        <ns0:v>Email thebeautylable3@icloud.com: Public current SumUp contact. Dated actual browser read; no booking, delivery test or outreach permission inferred. Current SumUp service source differs from older Fresha pricing.</ns0:v>
+        <ns0:v>Phone +44 7501 827293: Published provider phone, not evidence of WhatsApp. Email thebeautylable3@icloud.com: Public current SumUp contact. Dated actual browser read; no booking, delivery test or outreach permission inferred. Current SumUp service source differs from older Fresha pricing. </ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -2469,7 +2482,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K38" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for The Beauty Lab. visitors can compare options such as Brow wax and Brow wax &amp; tint, see the listed price and appointment length, then open your SumUp Bookings booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing SumUp Bookings page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for The Beauty Lab. Visitors can compare options such as Brow wax and Brow wax &amp; tint, see the listed price and appointment length, then open your SumUp Bookings booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing SumUp Bookings page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L38" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -2492,10 +2505,10 @@
         <ns0:v>thebeautylable3@icloud.com: Public current SumUp contact. Dated actual browser read; no booking, delivery test or outreach permission inferred. Current SumUp service source differs from older Fresha pricing.</ns0:v>
       </ns0:c>
       <ns0:c r="S38" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T38" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="39" ht="210" customHeight="1">
@@ -2515,7 +2528,7 @@
         <ns0:v>https://venturasolutions.co.uk/steak-and-lounge/</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="7" t="str">
-        <ns0:v>Email info@maffoodandbeverages.com: Official published email; delivery not tested.</ns0:v>
+        <ns0:v>Email info@maffoodandbeverages.com: Official published email; delivery not tested. </ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -2533,7 +2546,7 @@
         <ns0:v>Help diners explore the type of evening they want before checking availability.</ns0:v>
       </ns0:c>
       <ns0:c r="K39" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Steak &amp; Lounge. it includes food category explorer across steaks, starters, sizzlers and more and food photograph viewer and links to the existing booking route. the idea is to help diners explore the type of evening they want before checking availability. the site also links to your OpenTable page for table bookings. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Steak &amp; Lounge. It includes food category explorer across steaks, starters, sizzlers and more and food photograph viewer and links to the existing booking route. The idea is to help diners explore the type of evening they want before checking availability. The site also links to your OpenTable page for table bookings. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L39" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2543,14 +2556,14 @@
 Tap to call +441162622666: tel:+441162622666</ns0:v>
       </ns0:c>
       <ns0:c r="N39" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Fiaz Abdul Majid</ns0:v>
       </ns0:c>
       <ns0:c r="O39" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. Exact-name and company candidate search did not verify a current local decision-maker.</ns0:v>
+        <ns0:v>Active company director. Exact 43 Abbey Street. Operational buying responsibility is not established.</ns0:v>
       </ns0:c>
       <ns0:c r="P39" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-26</ns0:v>
+        <ns0:v>https://find-and-update.company-information.service.gov.uk/company/11262058/officers
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q39" s="7" t="str">
         <ns0:v>None verified</ns0:v>
@@ -2559,10 +2572,10 @@
         <ns0:v>info@maffoodandbeverages.com: Official published email; delivery not tested.</ns0:v>
       </ns0:c>
       <ns0:c r="S39" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T39" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Contact fields have public-source leads; see role and source caveats.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="40" ht="210" customHeight="1">
@@ -2582,7 +2595,7 @@
         <ns0:v>https://venturasolutions.co.uk/raykdi/</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="7" t="str">
-        <ns0:v>Phone 07707 181303: Exact 9 Bath House Lane directory phone; Low confidence because the same directory mislabels Indian cuisine as Thai. Verify recipient before use.</ns0:v>
+        <ns0:v>Phone 07707 181303: Exact 9 Bath House Lane directory phone; Low confidence because the same directory mislabels Indian cuisine as Thai. Verify recipient before use. </ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="7" t="str">
         <ns0:v>2026-10-11</ns0:v>
@@ -2601,7 +2614,7 @@
         <ns0:v>Help customers explore the chaat menu and keep the dishes they want to try together.</ns0:v>
       </ns0:c>
       <ns0:c r="K40" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Raykdi. it includes menu category filters and item detail views and copyable dish shortlist. the idea is to help customers explore the chaat menu and keep the dishes they want to try together. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Raykdi. It includes menu category filters and item detail views and copyable dish shortlist. The idea is to help customers explore the chaat menu and keep the dishes they want to try together. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L40" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2628,10 +2641,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S40" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T40" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="41" ht="210" customHeight="1">
@@ -2651,7 +2664,7 @@
         <ns0:v>https://venturasolutions.co.uk/keith-ashmore/</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="7" t="str">
-        <ns0:v>Phone 0116 251 7272: Directory landline conflicts with preferred market mobile; confirm.</ns0:v>
+        <ns0:v>Phone 0116 251 7272: Directory landline conflicts with preferred market mobile; confirm. </ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -2670,7 +2683,7 @@
         <ns0:v>Help customers explain what they are cooking and get advice at the counter.</ns0:v>
       </ns0:c>
       <ns0:c r="K41" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Keith Ashmore. it includes range guide covering beef, lamb, pork, poultry and offal and butcher question list shaped by meal type, people and preparation needs. the idea is to help customers explain what they are cooking and get advice at the counter. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Keith Ashmore. It includes range guide covering beef, lamb, pork, poultry and offal and butcher question list shaped by meal type, people and preparation needs. The idea is to help customers explain what they are cooking and get advice at the counter. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L41" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -2696,10 +2709,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S41" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T41" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="42" ht="210" customHeight="1">
@@ -2735,7 +2748,7 @@
         <ns0:v>Help visitors choose a few brunch and drink ideas before arriving.</ns0:v>
       </ns0:c>
       <ns0:c r="K42" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for La Foret Cafe. it includes brunch, lunch and drinks filters and café list for shortlisted dishes and drinks. the idea is to help visitors choose a few brunch and drink ideas before arriving. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for La Foret Cafe. It includes brunch, lunch and drinks filters and café list for shortlisted dishes and drinks. The idea is to help visitors choose a few brunch and drink ideas before arriving. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L42" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2745,14 +2758,14 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=11+King+Street%2C+Leicester</ns0:v>
       </ns0:c>
       <ns0:c r="N42" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Radhouene Mhadhbi</ns0:v>
       </ns0:c>
       <ns0:c r="O42" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. No public owner or manager with a confirmed current role found in scoped search.</ns0:v>
+        <ns0:v>Active company director. Exact 11 King Street. Operational buying responsibility is not established.</ns0:v>
       </ns0:c>
       <ns0:c r="P42" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-26</ns0:v>
+        <ns0:v>https://find-and-update.company-information.service.gov.uk/company/12466337/officers
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q42" s="7" t="str">
         <ns0:v>None verified</ns0:v>
@@ -2761,10 +2774,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S42" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T42" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="43" ht="210" customHeight="1">
@@ -2802,7 +2815,7 @@
         <ns0:v>Help visitors distinguish a brunch plan from an evening meal.</ns0:v>
       </ns0:c>
       <ns0:c r="K43" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for LYNN. it includes separate brunch and bistro views with dish search and meal note that includes occasion, day and group size. the idea is to help visitors distinguish a brunch plan from an evening meal. the site also links to your SevenRooms page for table bookings, and your existing Just Eat menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for LYNN. It includes separate brunch and bistro views with dish search and meal note that includes occasion, day and group size. The idea is to help visitors distinguish a brunch plan from an evening meal. The site also links to your SevenRooms page for table bookings, and your existing Just Eat menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L43" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -2830,10 +2843,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S43" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T43" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="44" ht="210" customHeight="1">
@@ -2868,7 +2881,7 @@
         <ns0:v>Help visitors ask about the dishes they have seen without assuming they are available today.</ns0:v>
       </ns0:c>
       <ns0:c r="K44" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Milan Di Damao. it includes searchable nasta, chai and Indo-Chinese dish references and copyable ask list with visit day, time of day and availability questions. the idea is to help visitors ask about the dishes they have seen without assuming they are available today. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Milan Di Damao. It includes searchable nasta, chai and Indo-Chinese dish references and copyable ask list with visit day, time of day and availability questions. The idea is to help visitors ask about the dishes they have seen without assuming they are available today. Customers can open the business location in Google Maps for directions. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L44" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -2893,10 +2906,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S44" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T44" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="45" ht="210" customHeight="1">
@@ -2915,7 +2928,9 @@
       <ns0:c r="E45" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/beautylicious/</ns0:v>
       </ns0:c>
-      <ns0:c r="F45" s="7" t="str"/>
+      <ns0:c r="F45" s="7" t="str">
+        <ns0:v>Phone +44 7773 723925: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G45" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -2932,7 +2947,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K45" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Beautylicious. visitors can compare options such as Eyebrows · threading and Eyebrows · waxing, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Beautylicious. Visitors can compare options such as Eyebrows · threading and Eyebrows · waxing, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L45" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -2955,10 +2970,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S45" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T45" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="46" ht="210" customHeight="1">
@@ -2977,7 +2992,9 @@
       <ns0:c r="E46" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/queen-lashes/</ns0:v>
       </ns0:c>
-      <ns0:c r="F46" s="7" t="str"/>
+      <ns0:c r="F46" s="7" t="str">
+        <ns0:v>Phone +44 7927 801351: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G46" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -2994,7 +3011,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K46" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Queen Lashes. visitors can compare options such as Russian Infills and Classic Full Set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Queen Lashes. Visitors can compare options such as Russian Infills and Classic Full Set, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L46" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3017,10 +3034,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S46" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T46" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="47" ht="210" customHeight="1">
@@ -3050,7 +3067,7 @@
         <ns0:v>Help shoppers describe the kind of outfit they are looking for.</ns0:v>
       </ns0:c>
       <ns0:c r="K47" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for RKD. it includes menswear and womenswear browsing choices and casual or formal preferences with a copyable visit shortlist. the idea is to help shoppers describe the kind of outfit they are looking for. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for RKD. It includes menswear and womenswear browsing choices and casual or formal preferences with a copyable visit shortlist. The idea is to help shoppers describe the kind of outfit they are looking for. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L47" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -3073,10 +3090,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S47" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T47" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="48" ht="210" customHeight="1">
@@ -3111,7 +3128,7 @@
         <ns0:v>Help visitors plan a trip that combines gaming, a café stop and browsing.</ns0:v>
       </ns0:c>
       <ns0:c r="K48" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Super Game Shack Level 2. it includes arcade, café and shop visit guide and copyable list of activities to explore. the idea is to help visitors plan a trip that combines gaming, a café stop and browsing. customers can open the business location in Google Maps for directions. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Super Game Shack Level 2. It includes arcade, café and shop visit guide and copyable list of activities to explore. The idea is to help visitors plan a trip that combines gaming, a café stop and browsing. Customers can open the business location in Google Maps for directions. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L48" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -3136,10 +3153,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S48" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T48" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="49" ht="210" customHeight="1">
@@ -3176,7 +3193,7 @@
         <ns0:v>Help customers bring organised measurements and questions into the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K49" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Bradgate Lace. it includes window measurement notes with room labels and centimetre or inch units and multiple window entries with edit, copy and print controls. the idea is to help customers bring organised measurements and questions into the shop. the site also links to your WhatsApp chat for enquiries. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Bradgate Lace. It includes window measurement notes with room labels and centimetre or inch units and multiple window entries with edit, copy and print controls. The idea is to help customers bring organised measurements and questions into the shop. The site also links to your WhatsApp chat for enquiries. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L49" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -3203,10 +3220,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S49" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T49" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="50" ht="210" customHeight="1">
@@ -3242,7 +3259,7 @@
         <ns0:v>Help customers describe a screen, charging or camera problem before contacting the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K50" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Humberstone Mobile. it includes phone make, model and fault enquiry guide and copyable repair discussion notes. the idea is to help customers describe a screen, charging or camera problem before contacting the shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Humberstone Mobile. It includes phone make, model and fault enquiry guide and copyable repair discussion notes. The idea is to help customers describe a screen, charging or camera problem before contacting the shop. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L50" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -3268,10 +3285,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S50" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T50" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="51" ht="210" customHeight="1">
@@ -3307,7 +3324,7 @@
         <ns0:v>Help customers find a relevant lunch choice before visiting or opening the ordering provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K51" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Kicheri. it includes searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks and food photograph views and an existing Uber Eats link. the idea is to help customers find a relevant lunch choice before visiting or opening the ordering provider. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Kicheri. It includes searchable menu grouped into breakfasts, omelettes, create-your-own options and drinks and food photograph views and an existing Uber Eats link. The idea is to help customers find a relevant lunch choice before visiting or opening the ordering provider. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L51" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -3333,10 +3350,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S51" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T51" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="52" ht="210" customHeight="1">
@@ -3368,7 +3385,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K52" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for By.meadowmae. visitors can compare options such as BIAB Manicure and Gel Manicure, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for By.meadowmae. Visitors can compare options such as BIAB Manicure and Gel Manicure, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L52" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3391,10 +3408,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S52" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T52" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="53" ht="210" customHeight="1">
@@ -3426,7 +3443,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K53" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Cargo Male Grooming. visitors can compare options such as Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Cargo Male Grooming. Visitors can compare options such as Haircut &amp; Style with Alfie and Haircut &amp; Beard with Alfie, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L53" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3452,10 +3469,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S53" s="7" t="str">
-        <ns0:v>hey alfie,</ns0:v>
+        <ns0:v>Hi Alfie,</ns0:v>
       </ns0:c>
       <ns0:c r="T53" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="54" ht="210" customHeight="1">
@@ -3475,7 +3492,7 @@
         <ns0:v>https://venturasolutions.co.uk/cafe-dido/</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="7" t="str">
-        <ns0:v>Phone 0116 225 0446: Older directory landline; conflicts with newer mobile.</ns0:v>
+        <ns0:v>Phone 0116 225 0446: Older directory landline; conflicts with newer mobile. </ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -3494,7 +3511,7 @@
         <ns0:v>Help visitors organise their café questions before calling.</ns0:v>
       </ns0:c>
       <ns0:c r="K54" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Cade Dido. it includes visit planner for breakfast, lunch or a drink break and question list for dates, group size, outdoor seating and access. the idea is to help visitors organise their café questions before calling. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Cade Dido. It includes visit planner for breakfast, lunch or a drink break and question list for dates, group size, outdoor seating and access. The idea is to help visitors organise their café questions before calling. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L54" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -3520,10 +3537,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S54" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T54" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="55" ht="210" customHeight="1">
@@ -3542,7 +3559,9 @@
       <ns0:c r="E55" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/grace-hairstylist/</ns0:v>
       </ns0:c>
-      <ns0:c r="F55" s="7" t="str"/>
+      <ns0:c r="F55" s="7" t="str">
+        <ns0:v>Phone +44 7857 422506: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G55" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3559,7 +3578,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K55" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Grace Hairstylist. visitors can compare options such as Ladies Cut &amp; Finish and Blow dry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Grace Hairstylist. Visitors can compare options such as Ladies Cut &amp; Finish and Blow dry, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L55" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3582,10 +3601,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S55" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T55" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="56" ht="210" customHeight="1">
@@ -3604,7 +3623,9 @@
       <ns0:c r="E56" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/joshs-hair-hideaway/</ns0:v>
       </ns0:c>
-      <ns0:c r="F56" s="7" t="str"/>
+      <ns0:c r="F56" s="7" t="str">
+        <ns0:v>Phone +44 7949 179382: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G56" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3621,7 +3642,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K56" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Josh’s Hair Hideaway. visitors can compare options such as Cut &amp; Finish and Gents Cut &amp; Finish, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Josh’s Hair Hideaway. Visitors can compare options such as Cut &amp; Finish and Gents Cut &amp; Finish, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L56" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3644,10 +3665,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S56" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T56" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="57" ht="210" customHeight="1">
@@ -3666,7 +3687,9 @@
       <ns0:c r="E57" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/pretty-suite-by-abbie/</ns0:v>
       </ns0:c>
-      <ns0:c r="F57" s="7" t="str"/>
+      <ns0:c r="F57" s="7" t="str">
+        <ns0:v>Phone +44 7709 212108: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G57" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3683,7 +3706,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K57" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Pretty Suite by Abbie. visitors can compare options such as 30 min Mini fill and Brow wax and tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Pretty Suite by Abbie. Visitors can compare options such as 30 min Mini fill and Brow wax and tint, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L57" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3693,12 +3716,15 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Hill%20Rise%2C%20Leicester%20LE4</ns0:v>
       </ns0:c>
       <ns0:c r="N57" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Abbie</ns0:v>
       </ns0:c>
       <ns0:c r="O57" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. </ns0:v>
-      </ns0:c>
-      <ns0:c r="P57" s="7" t="str"/>
+        <ns0:v>Salon owner. Explicit owner role in booking provider team section; surname not independently verified.</ns0:v>
+      </ns0:c>
+      <ns0:c r="P57" s="7" t="str">
+        <ns0:v>https://www.fresha.com/a/pretty-suite-by-abbie-leicester-hill-rise-tw0ac4s3
+Checked: 2026-10-25</ns0:v>
+      </ns0:c>
       <ns0:c r="Q57" s="7" t="str">
         <ns0:v>Megan (Listed staff member, not a verified owner/decision maker.); Jemma (Listed staff member, not a verified owner/decision maker.); Mia (Listed staff member, not a verified owner/decision maker.); Abbie (Listed staff member, not a verified owner/decision maker.)</ns0:v>
       </ns0:c>
@@ -3706,10 +3732,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S57" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi Abbie,</ns0:v>
       </ns0:c>
       <ns0:c r="T57" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="58" ht="210" customHeight="1">
@@ -3744,7 +3770,7 @@
         <ns0:v>Help shoppers check what they need from the kiosk before making a trip.</ns0:v>
       </ns0:c>
       <ns0:c r="K58" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Haymarket Kiosk. it includes guide to snacks, newspapers, mobile top-ups and bill services and visit checklist with questions for the selected services. the idea is to help shoppers check what they need from the kiosk before making a trip. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Haymarket Kiosk. It includes guide to snacks, newspapers, mobile top-ups and bill services and visit checklist with questions for the selected services. The idea is to help shoppers check what they need from the kiosk before making a trip. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L58" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -3769,10 +3795,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S58" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T58" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="59" ht="210" customHeight="1">
@@ -3791,7 +3817,9 @@
       <ns0:c r="E59" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/aimee-charlotte-beauty/</ns0:v>
       </ns0:c>
-      <ns0:c r="F59" s="7" t="str"/>
+      <ns0:c r="F59" s="7" t="str">
+        <ns0:v>Phone +44 7584 858257: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G59" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3808,7 +3836,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K59" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Aimee Charlotte Beauty. visitors can compare options such as Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Aimee Charlotte Beauty. Visitors can compare options such as Builder In A Bottle &amp; Gel Polish and Builder In A Bottle French, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L59" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3831,10 +3859,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S59" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T59" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="60" ht="210" customHeight="1">
@@ -3853,7 +3881,9 @@
       <ns0:c r="E60" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/anelita-beauty/</ns0:v>
       </ns0:c>
-      <ns0:c r="F60" s="7" t="str"/>
+      <ns0:c r="F60" s="7" t="str">
+        <ns0:v>Phone +44 7549 914795: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G60" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3870,7 +3900,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K60" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Anelita Beauty. visitors can compare options such as LVL Lash Lift and Individual eyelash extensions - Full set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Anelita Beauty. Visitors can compare options such as LVL Lash Lift and Individual eyelash extensions - Full set, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L60" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3893,10 +3923,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S60" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T60" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="61" ht="210" customHeight="1">
@@ -3915,7 +3945,9 @@
       <ns0:c r="E61" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/hair-by-tia/</ns0:v>
       </ns0:c>
-      <ns0:c r="F61" s="7" t="str"/>
+      <ns0:c r="F61" s="7" t="str">
+        <ns0:v>Phone +44 7947 720560: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G61" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -3932,7 +3964,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K61" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Hair by Tia. visitors can compare options such as Hair up and Tapes Half head Maintenance, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Hair by Tia. Visitors can compare options such as Hair up and Tapes Half head Maintenance, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L61" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -3955,10 +3987,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S61" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T61" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="62" ht="210" customHeight="1">
@@ -3994,7 +4026,7 @@
         <ns0:v>Help customers organise the parts of their shop they want to ask about.</ns0:v>
       </ns0:c>
       <ns0:c r="K62" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for International Food Centre. it includes produce, grocery and fresh bread category guide and copyable shopping interests list. the idea is to help customers organise the parts of their shop they want to ask about. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for International Food Centre. It includes produce, grocery and fresh bread category guide and copyable shopping interests list. The idea is to help customers organise the parts of their shop they want to ask about. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L62" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4020,10 +4052,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S62" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T62" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="63" ht="210" customHeight="1">
@@ -4059,7 +4091,7 @@
         <ns0:v>Give visitors a feel for the cooking and help them recognise the café.</ns0:v>
       </ns0:c>
       <ns0:c r="K63" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for The Good Earth. it includes vegetarian dish examples grouped by comfort food and soup and café photograph viewer and Free Lane visit information. the idea is to give visitors a feel for the cooking and help them recognise the café. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for The Good Earth. It includes vegetarian dish examples grouped by comfort food and soup and café photograph viewer and Free Lane visit information. The idea is to give visitors a feel for the cooking and help them recognise the café. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L63" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4085,10 +4117,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S63" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T63" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="64" ht="210" customHeight="1">
@@ -4120,7 +4152,7 @@
         <ns0:v>Help customers bring together the items they want to discuss in the shop.</ns0:v>
       </ns0:c>
       <ns0:c r="K64" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Leicester Fresh Food. it includes fruit, meat and chicken, and bread category choices and copyable shopping note. the idea is to help customers bring together the items they want to discuss in the shop. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Leicester Fresh Food. It includes fruit, meat and chicken, and bread category choices and copyable shopping note. The idea is to help customers bring together the items they want to discuss in the shop. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L64" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4146,10 +4178,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S64" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T64" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="65" ht="210" customHeight="1">
@@ -4185,7 +4217,7 @@
         <ns0:v>Give people a clear starting point for asking about treatments and planning a visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K65" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Soi 52. it includes treatment information and Church Gate location details and links to the existing business website and directions. the idea is to give people a clear starting point for asking about treatments and planning a visit. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Soi 52. It includes treatment information and Church Gate location details and links to the existing business website and directions. The idea is to give people a clear starting point for asking about treatments and planning a visit. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L65" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4211,10 +4243,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S65" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T65" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="66" ht="210" customHeight="1">
@@ -4246,7 +4278,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K66" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Soie Hair. visitors can compare options such as Wash Cut &amp; Blowdry and Signature Blowout, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Soie Hair. Visitors can compare options such as Wash Cut &amp; Blowdry and Signature Blowout, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L66" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4269,10 +4301,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S66" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T66" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="67" ht="210" customHeight="1">
@@ -4309,7 +4341,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K67" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Star Barbers Oadby. visitors can compare options such as Hair cut and Skin fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Star Barbers Oadby. Visitors can compare options such as Hair cut and Skin fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L67" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4336,10 +4368,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S67" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T67" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="68" ht="210" customHeight="1">
@@ -4371,7 +4403,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K68" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for M K BARBER. visitors can compare options such as Skin fade and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for M K BARBER. Visitors can compare options such as Skin fade and Taper fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L68" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4394,10 +4426,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S68" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T68" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="69" ht="210" customHeight="1">
@@ -4430,7 +4462,7 @@
         <ns0:v>Let visitors explore a bowl combination before checking the existing ordering options.</ns0:v>
       </ns0:c>
       <ns0:c r="K69" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Alcove. it includes coffee, specials and açaí menu filters and four-topping açaí bowl outline builder. the idea is to let visitors explore a bowl combination before checking the existing ordering options. the site also links to your existing Uber Eats menu for ordering, and your Square gift card page. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Alcove. It includes coffee, specials and açaí menu filters and four-topping açaí bowl outline builder. The idea is to let visitors explore a bowl combination before checking the existing ordering options. The site also links to your existing Uber Eats menu for ordering, and your Square gift card page. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L69" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -4451,16 +4483,16 @@
 Checked: 2026-09-26</ns0:v>
       </ns0:c>
       <ns0:c r="Q69" s="7" t="str">
-        <ns0:v>None verified</ns0:v>
+        <ns0:v>Reece (Venue event manager; not verified owner)</ns0:v>
       </ns0:c>
       <ns0:c r="R69" s="7" t="str">
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S69" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T69" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="70" ht="210" customHeight="1">
@@ -4471,7 +4503,7 @@
         <ns0:v>The Mane Room Leicester</ns0:v>
       </ns0:c>
       <ns0:c r="C70" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>0116 319 1818</ns0:v>
       </ns0:c>
       <ns0:c r="D70" s="8" t="str">
         <ns0:v>Not found</ns0:v>
@@ -4479,9 +4511,15 @@
       <ns0:c r="E70" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/the-mane-room/</ns0:v>
       </ns0:c>
-      <ns0:c r="F70" s="7" t="str"/>
-      <ns0:c r="G70" s="7" t="str"/>
-      <ns0:c r="H70" s="7" t="str"/>
+      <ns0:c r="F70" s="7" t="str">
+        <ns0:v>Phone 0116 319 1818: Exact 94 Leicester Road directory match; also listed by Endole. Not call-tested. </ns0:v>
+      </ns0:c>
+      <ns0:c r="G70" s="7" t="str">
+        <ns0:v>2026-10-25</ns0:v>
+      </ns0:c>
+      <ns0:c r="H70" s="7" t="str">
+        <ns0:v>https://www.192.com/atoz/business/wigston-le18/hairdressers-unisex/the-mane-room-leicester-ltd/36f8d6e751a3651fbd51cb48f732f16631ead2d0/comp/</ns0:v>
+      </ns0:c>
       <ns0:c r="I70" s="7" t="str">
         <ns0:v>Service selector including Gents Haircut and Skin Fade
 Listed prices and appointment lengths update with the selected service
@@ -4492,7 +4530,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K70" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for The Mane Room Leicester. visitors can compare options such as Gents Haircut and Skin Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for The Mane Room Leicester. Visitors can compare options such as Gents Haircut and Skin Fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L70" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4518,10 +4556,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S70" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T70" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="71" ht="210" customHeight="1">
@@ -4532,7 +4570,7 @@
         <ns0:v>Mancave Barber Lounge</ns0:v>
       </ns0:c>
       <ns0:c r="C71" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>0116 319 3353</ns0:v>
       </ns0:c>
       <ns0:c r="D71" s="8" t="str">
         <ns0:v>Not found</ns0:v>
@@ -4540,9 +4578,15 @@
       <ns0:c r="E71" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/mancave-barber-lounge/</ns0:v>
       </ns0:c>
-      <ns0:c r="F71" s="7" t="str"/>
-      <ns0:c r="G71" s="7" t="str"/>
-      <ns0:c r="H71" s="7" t="str"/>
+      <ns0:c r="F71" s="7" t="str">
+        <ns0:v>Phone 0116 319 3353: Exact 5 Bell Street; corroborated by Waze and Yell. Not call-tested. Unrelated Canadian Mancave contact and redirected old website excluded. Current operator caveat retained.</ns0:v>
+      </ns0:c>
+      <ns0:c r="G71" s="7" t="str">
+        <ns0:v>2026-10-25</ns0:v>
+      </ns0:c>
+      <ns0:c r="H71" s="7" t="str">
+        <ns0:v>https://wigston.cylex-uk.co.uk/company/mancave-barber-lounge-26998055.html</ns0:v>
+      </ns0:c>
       <ns0:c r="I71" s="7" t="str">
         <ns0:v>Service selector including Gents Haircut and Skin or Zero Fade
 Listed prices and appointment lengths update with the selected service
@@ -4553,7 +4597,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K71" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Mancave Barber Lounge. visitors can compare options such as Gents Haircut and Skin or Zero Fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Mancave Barber Lounge. Visitors can compare options such as Gents Haircut and Skin or Zero Fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L71" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4579,10 +4623,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S71" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T71" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="72" ht="210" customHeight="1">
@@ -4619,7 +4663,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K72" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for 11:11 Studios. visitors can compare options such as BIAB overlay and BIAB infill, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for 11:11 Studios. Visitors can compare options such as BIAB overlay and BIAB infill, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L72" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4643,10 +4687,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S72" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T72" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="73" ht="210" customHeight="1">
@@ -4665,7 +4709,9 @@
       <ns0:c r="E73" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/mphair/</ns0:v>
       </ns0:c>
-      <ns0:c r="F73" s="7" t="str"/>
+      <ns0:c r="F73" s="7" t="str">
+        <ns0:v>Phone +44 7914 342985: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G73" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -4682,7 +4728,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K73" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for MPHair. visitors can compare options such as Ladies Cut and Blow dry and Gents cut no wash, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for MPHair. Visitors can compare options such as Ladies Cut and Blow dry and Gents cut no wash, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L73" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4705,10 +4751,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S73" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T73" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="74" ht="210" customHeight="1">
@@ -4728,7 +4774,7 @@
         <ns0:v>https://venturasolutions.co.uk/be-beautiful-by-alex/</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="7" t="str">
-        <ns0:v>Email bebeautifulbyalex@hotmail.com: Published business email. Primary-linked page ID, business phone and host address matched. No delivery or outreach permission inferred.</ns0:v>
+        <ns0:v>Phone +44 7896 468368: Published provider phone, not evidence of WhatsApp. Email bebeautifulbyalex@hotmail.com: Published business email. Primary-linked page ID, business phone and host address matched. No delivery or outreach permission inferred. </ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -4747,7 +4793,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K74" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Be beautiful by Alex. visitors can compare options such as BIAB Infill and Eyebrow shape &amp; Tint, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Be beautiful by Alex. Visitors can compare options such as BIAB Infill and Eyebrow shape &amp; Tint, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L74" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4770,10 +4816,10 @@
         <ns0:v>bebeautifulbyalex@hotmail.com: Published business email. Primary-linked page ID, business phone and host address matched. No delivery or outreach permission inferred.</ns0:v>
       </ns0:c>
       <ns0:c r="S74" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T74" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="75" ht="210" customHeight="1">
@@ -4792,7 +4838,9 @@
       <ns0:c r="E75" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/graced-by-helen/</ns0:v>
       </ns0:c>
-      <ns0:c r="F75" s="7" t="str"/>
+      <ns0:c r="F75" s="7" t="str">
+        <ns0:v>Phone +44 7903 370240: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G75" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -4809,7 +4857,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K75" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Graced by Helen. visitors can compare options such as Knotless/Box Braids and Make-up (For Occasions), see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Graced by Helen. Visitors can compare options such as Knotless/Box Braids and Make-up (For Occasions), see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L75" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -4832,10 +4880,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S75" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T75" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="76" ht="210" customHeight="1">
@@ -4855,7 +4903,7 @@
         <ns0:v>https://venturasolutions.co.uk/pot-pourri-shop/</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="7" t="str">
-        <ns0:v>Phone 07746 005228: Search snippet alternative; confirm recipient before use.</ns0:v>
+        <ns0:v>Phone 07746 005228: Search snippet alternative; confirm recipient before use. </ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -4874,7 +4922,7 @@
         <ns0:v>Help shoppers explain a birthday, thank-you or just-because gift idea.</ns0:v>
       </ns0:c>
       <ns0:c r="K76" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Pot Pourri Shop. it includes gift brief built around occasion and shopping interest and optional budget selection and a copyable summary. the idea is to help shoppers explain a birthday, thank-you or just-because gift idea. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Pot Pourri Shop. It includes gift brief built around occasion and shopping interest and optional budget selection and a copyable summary. The idea is to help shoppers explain a birthday, thank-you or just-because gift idea. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L76" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4900,10 +4948,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S76" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T76" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="77" ht="210" customHeight="1">
@@ -4939,7 +4987,7 @@
         <ns0:v>Help clients describe the finish they have in mind before speaking to the salon.</ns0:v>
       </ns0:c>
       <ns0:c r="K77" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for London Nails. it includes nail inspiration choices from the salon gallery and call note combining the chosen look with preferred nail length. the idea is to help clients describe the finish they have in mind before speaking to the salon. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for London Nails. It includes nail inspiration choices from the salon gallery and call note combining the chosen look with preferred nail length. The idea is to help clients describe the finish they have in mind before speaking to the salon. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L77" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -4965,10 +5013,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S77" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T77" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="78" ht="210" customHeight="1">
@@ -4988,7 +5036,7 @@
         <ns0:v>https://venturasolutions.co.uk/tiegan-seaton/</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="7" t="str">
-        <ns0:v>Email Seatshairstudio@icloud.com: Source-specific public business contact. Seat’s Facebook phone differs from provider phone and does not overwrite it. No WhatsApp, delivery test or outreach permission inferred.</ns0:v>
+        <ns0:v>Phone +44 7903 864581: Published provider phone, not evidence of WhatsApp. Phone 07394 504034: Source-specific public business contact. Seat’s Facebook phone differs from provider phone and does not overwrite it. No WhatsApp, delivery test or outreach permission inferred. Email Seatshairstudio@icloud.com: Source-specific public business contact. Seat’s Facebook phone differs from provider phone and does not overwrite it. No WhatsApp, delivery test or outreach permission inferred. </ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -5007,7 +5055,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K78" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Tiegan Seaton (Seats Hair Studio). visitors can compare options such as Restyle and Patch test &amp; consultation, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Tiegan Seaton (Seats Hair Studio). Visitors can compare options such as Restyle and Patch test &amp; consultation, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L78" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5030,10 +5078,10 @@
         <ns0:v>Seatshairstudio@icloud.com: Source-specific public business contact. Seat’s Facebook phone differs from provider phone and does not overwrite it. No WhatsApp, delivery test or outreach permission inferred.</ns0:v>
       </ns0:c>
       <ns0:c r="S78" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T78" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="79" ht="210" customHeight="1">
@@ -5052,7 +5100,9 @@
       <ns0:c r="E79" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/royalty-trimz/</ns0:v>
       </ns0:c>
-      <ns0:c r="F79" s="7" t="str"/>
+      <ns0:c r="F79" s="7" t="str">
+        <ns0:v>Phone +44 7716 285487: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G79" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -5069,7 +5119,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K79" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Royalty Trimz. visitors can compare options such as Shape up and Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Royalty Trimz. Visitors can compare options such as Shape up and Haircut, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L79" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5092,10 +5142,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S79" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T79" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="80" ht="210" customHeight="1">
@@ -5132,7 +5182,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K80" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Hair Muse. visitors can compare options such as Ladies Cut &amp; Blowdry and Long Hair Blowdry, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Hair Muse. Visitors can compare options such as Ladies Cut &amp; Blowdry and Long Hair Blowdry, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L80" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5159,10 +5209,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S80" s="7" t="str">
-        <ns0:v>hey jodie and phoebe,</ns0:v>
+        <ns0:v>Hi Jodie and Phoebe,</ns0:v>
       </ns0:c>
       <ns0:c r="T80" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="81" ht="210" customHeight="1">
@@ -5182,7 +5232,7 @@
         <ns0:v>https://venturasolutions.co.uk/autofaders/</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="7" t="str">
-        <ns0:v>Email autofader@hotmail.com: Public booking-profile business contact at exact 8c Devana Road; named owner recipient and inbox delivery untested.</ns0:v>
+        <ns0:v>Phone +44 116 221 6774: Published provider phone, not evidence of WhatsApp. Phone 07718 596614: Additional published business number; previous numbers retained. Email autofader@hotmail.com: Public booking-profile business contact at exact 8c Devana Road; named owner recipient and inbox delivery untested. </ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -5201,7 +5251,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K81" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Autofaders. visitors can compare options such as Haircut · Senior barber and Haircut &amp; Beard · Senior barber, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Autofaders. Visitors can compare options such as Haircut · Senior barber and Haircut &amp; Beard · Senior barber, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L81" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5224,10 +5274,10 @@
         <ns0:v>autofader@hotmail.com: Public booking-profile business contact at exact 8c Devana Road; named owner recipient and inbox delivery untested.</ns0:v>
       </ns0:c>
       <ns0:c r="S81" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T81" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="82" ht="210" customHeight="1">
@@ -5247,7 +5297,7 @@
         <ns0:v>https://venturasolutions.co.uk/glamupwithester/</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="7" t="str">
-        <ns0:v>Email makeupwithester@gmail.com: Published specifically for bridal booking enquiries through December2027. General sales outreach suitability unverified. No delivery test or outreach permission inferred.</ns0:v>
+        <ns0:v>Phone +44 7432 132050: Published provider phone, not evidence of WhatsApp. Email makeupwithester@gmail.com: Published specifically for bridal booking enquiries through December2027. General sales outreach suitability unverified. No delivery test or outreach permission inferred. </ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -5266,7 +5316,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K82" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for GlamUpWithEster. visitors can compare options such as Makeup and Prom makeup, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for GlamUpWithEster. Visitors can compare options such as Makeup and Prom makeup, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L82" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5289,10 +5339,10 @@
         <ns0:v>makeupwithester@gmail.com: Published specifically for bridal booking enquiries through December2027. General sales outreach suitability unverified. No delivery test or outreach permission inferred.</ns0:v>
       </ns0:c>
       <ns0:c r="S82" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T82" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="83" ht="210" customHeight="1">
@@ -5324,7 +5374,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K83" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Mercy Nails. visitors can compare options such as Builder Gel Infills and Acrylic Nails, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Mercy Nails. Visitors can compare options such as Builder Gel Infills and Acrylic Nails, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L83" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5347,10 +5397,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S83" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T83" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="84" ht="210" customHeight="1">
@@ -5370,7 +5420,7 @@
         <ns0:v>https://venturasolutions.co.uk/sapphire-treatments/</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="7" t="str">
-        <ns0:v>Email sapphiretreatments@icloud.com: Published public business contact from provider-linked Facebook; inbox delivery and named recipient not tested.</ns0:v>
+        <ns0:v>Phone +44 7802 254291: Published provider phone, not evidence of WhatsApp. Email sapphiretreatments@icloud.com: Published public business contact from provider-linked Facebook; inbox delivery and named recipient not tested. </ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
@@ -5388,7 +5438,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K84" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Sapphire Treatments. visitors can compare options such as Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Sapphire Treatments. Visitors can compare options such as Relax &amp; Revive; Leg &amp; Foot and Tension Relief: Back, Neck &amp; Scalp Retreat, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L84" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5410,10 +5460,10 @@
         <ns0:v>sapphiretreatments@icloud.com: Published public business contact from provider-linked Facebook; inbox delivery and named recipient not tested.</ns0:v>
       </ns0:c>
       <ns0:c r="S84" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T84" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="85" ht="210" customHeight="1">
@@ -5433,7 +5483,7 @@
         <ns0:v>https://venturasolutions.co.uk/sambrayhair/</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="7" t="str">
-        <ns0:v>Email Sambray92@hotmail.com: Published business email. Primary-linked page ID, address and phone matched. No delivery or outreach permission inferred.</ns0:v>
+        <ns0:v>Email Sambray92@hotmail.com: Published business email. Primary-linked page ID, address and phone matched. No delivery or outreach permission inferred. </ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="7" t="str">
         <ns0:v>2026-10-24</ns0:v>
@@ -5452,7 +5502,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K85" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for SamBrayHair. visitors can compare options such as Wash Cut &amp; Blowdry and Mens Haircut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for SamBrayHair. Visitors can compare options such as Wash Cut &amp; Blowdry and Mens Haircut, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L85" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5462,12 +5512,15 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=Church%20Hill%20Road%20Thurmaston%20Leicester%20LE4%208DE</ns0:v>
       </ns0:c>
       <ns0:c r="N85" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Samantha</ns0:v>
       </ns0:c>
       <ns0:c r="O85" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. </ns0:v>
-      </ns0:c>
-      <ns0:c r="P85" s="7" t="str"/>
+        <ns0:v>Salon owner. Explicit owner role in booking provider team section; surname not independently verified.</ns0:v>
+      </ns0:c>
+      <ns0:c r="P85" s="7" t="str">
+        <ns0:v>https://www.fresha.com/a/sambrayhair-thurmaston-uk-church-hill-road-w5hi6pp2
+Checked: 2026-10-25</ns0:v>
+      </ns0:c>
       <ns0:c r="Q85" s="7" t="str">
         <ns0:v>Samantha (Listed staff member, not a verified owner/decision maker.)</ns0:v>
       </ns0:c>
@@ -5475,10 +5528,10 @@
         <ns0:v>Sambray92@hotmail.com: Published business email. Primary-linked page ID, address and phone matched. No delivery or outreach permission inferred.</ns0:v>
       </ns0:c>
       <ns0:c r="S85" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi Samantha,</ns0:v>
       </ns0:c>
       <ns0:c r="T85" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Contact fields have public-source leads; see role and source caveats.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="86" ht="210" customHeight="1">
@@ -5514,7 +5567,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K86" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Jennifer Audrey Nails &amp; Beauty. visitors can compare options such as BIAB and BIAB Toes, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Jennifer Audrey Nails &amp; Beauty. Visitors can compare options such as BIAB and BIAB Toes, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L86" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5537,10 +5590,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S86" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T86" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="87" ht="210" customHeight="1">
@@ -5576,7 +5629,7 @@
         <ns0:v>Help a group organise dishes and the questions they want to discuss.</ns0:v>
       </ns0:c>
       <ns0:c r="K87" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Oppa Korean Restaurant. it includes korean dish filters covering bibimbap, bulgogi, soups and more and meal shortlist with table BBQ, spice and allergy questions. the idea is to help a group organise dishes and the questions they want to discuss. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Oppa Korean Restaurant. It includes korean dish filters covering bibimbap, bulgogi, soups and more and meal shortlist with table BBQ, spice and allergy questions. The idea is to help a group organise dishes and the questions they want to discuss. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L87" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -5602,10 +5655,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S87" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T87" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="88" ht="210" customHeight="1">
@@ -5625,7 +5678,7 @@
         <ns0:v>https://venturasolutions.co.uk/sherwins/</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="7" t="str">
-        <ns0:v>Email ali.ireland55@yahoo.com: Published by cheese producer as Sherwins retailer contact; personal-style address used publicly for this business. Conflicting operator attribution: current market page names Tim Pole, tourism names Alison and Adam Ireland. Confirm current email routing.</ns0:v>
+        <ns0:v>Email ali.ireland55@yahoo.com: Published by cheese producer as Sherwins retailer contact; personal-style address used publicly for this business. Conflicting operator attribution: current market page names Tim Pole, tourism names Alison and Adam Ireland. Confirm current email routing. </ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -5644,7 +5697,7 @@
         <ns0:v>Help customers ask for a cheese selection suited to their gathering.</ns0:v>
       </ns0:c>
       <ns0:c r="K88" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Sherwin's Cheese Company. it includes cheese and deli guide with accompaniment ideas and gathering question list covering guest count, flavour preferences and serving questions. the idea is to help customers ask for a cheese selection suited to their gathering. customers can tap to call the business and open directions in Google Maps. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Sherwin's Cheese Company. It includes cheese and deli guide with accompaniment ideas and gathering question list covering guest count, flavour preferences and serving questions. The idea is to help customers ask for a cheese selection suited to their gathering. Customers can tap to call the business and open directions in Google Maps. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L88" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -5670,7 +5723,7 @@
         <ns0:v>ali.ireland55@yahoo.com: Published by cheese producer as Sherwins retailer contact; personal-style address used publicly for this business. Conflicting operator attribution: current market page names Tim Pole, tourism names Alison and Adam Ireland. Confirm current email routing.</ns0:v>
       </ns0:c>
       <ns0:c r="S88" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T88" s="7" t="str">
         <ns0:v>Conflict documented in batch 3 QC advisory; unresolved</ns0:v>
@@ -5692,7 +5745,9 @@
       <ns0:c r="E89" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/amic-studios/</ns0:v>
       </ns0:c>
-      <ns0:c r="F89" s="7" t="str"/>
+      <ns0:c r="F89" s="7" t="str">
+        <ns0:v>Phone +44 116 507 9854: Current exact public Amic Studios Birstall provider phone. Phone alone does not establish WhatsApp; no call or outreach. </ns0:v>
+      </ns0:c>
       <ns0:c r="G89" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -5709,7 +5764,7 @@
         <ns0:v>Help clients find the barber and service they want before opening the booking page.</ns0:v>
       </ns0:c>
       <ns0:c r="K89" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Amic Studios. it includes service search and filters for Dan, Tate, Dom and Alfie and named barber service listings with the existing Fresha route. the idea is to help clients find the barber and service they want before opening the booking page. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Amic Studios. It includes service search and filters for Dan, Tate, Dom and Alfie and named barber service listings with the existing Fresha route. The idea is to help clients find the barber and service they want before opening the booking page. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L89" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5735,10 +5790,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S89" s="7" t="str">
-        <ns0:v>hey alfie,</ns0:v>
+        <ns0:v>Hi Alfie,</ns0:v>
       </ns0:c>
       <ns0:c r="T89" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="90" ht="210" customHeight="1">
@@ -5757,7 +5812,9 @@
       <ns0:c r="E90" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/irl-nails-and-beauty/</ns0:v>
       </ns0:c>
-      <ns0:c r="F90" s="7" t="str"/>
+      <ns0:c r="F90" s="7" t="str">
+        <ns0:v>Phone +44 7754 989436: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G90" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -5774,7 +5831,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K90" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for IRL Nails and Beauty. visitors can compare options such as Gel polish - one colour and Removals with new set, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for IRL Nails and Beauty. Visitors can compare options such as Gel polish - one colour and Removals with new set, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L90" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5797,10 +5854,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S90" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T90" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="91" ht="210" customHeight="1">
@@ -5819,7 +5876,9 @@
       <ns0:c r="E91" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/hair-by-wikki/</ns0:v>
       </ns0:c>
-      <ns0:c r="F91" s="7" t="str"/>
+      <ns0:c r="F91" s="7" t="str">
+        <ns0:v>Phone +44 7806 744847: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G91" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -5836,7 +5895,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K91" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Hair By Wikki. visitors can compare options such as Ladies Cut &amp; Blow Dry and Gents Cut, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Hair By Wikki. Visitors can compare options such as Ladies Cut &amp; Blow Dry and Gents Cut, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L91" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5859,10 +5918,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S91" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T91" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="92" ht="210" customHeight="1">
@@ -5894,7 +5953,7 @@
         <ns0:v>Help customers find a meal category quickly before checking the ordering menu.</ns0:v>
       </ns0:c>
       <ns0:c r="K92" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for LALA’S Restaurant. it includes searchable menu selection with burger, wrap, pizza and grill filters and existing Deliveroo link alongside location information. the idea is to help customers find a meal category quickly before checking the ordering menu. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for LALA’S Restaurant. It includes searchable menu selection with burger, wrap, pizza and grill filters and existing Deliveroo link alongside location information. The idea is to help customers find a meal category quickly before checking the ordering menu. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L92" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -5917,10 +5976,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S92" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T92" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="93" ht="210" customHeight="1">
@@ -5939,7 +5998,9 @@
       <ns0:c r="E93" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/voss/</ns0:v>
       </ns0:c>
-      <ns0:c r="F93" s="7" t="str"/>
+      <ns0:c r="F93" s="7" t="str">
+        <ns0:v>Phone 07554 852052: Additional published business number; previous numbers retained. </ns0:v>
+      </ns0:c>
       <ns0:c r="G93" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -5956,7 +6017,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K93" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for VOSS. Barbering and Men’s Hair Specialist. visitors can compare options such as Cut and Finish and Cut and Finish w/ Beard Trim, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for VOSS. Barbering and Men’s Hair Specialist. Visitors can compare options such as Cut and Finish and Cut and Finish w/ Beard Trim, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L93" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -5982,10 +6043,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S93" s="7" t="str">
-        <ns0:v>hey william,</ns0:v>
+        <ns0:v>Hi William,</ns0:v>
       </ns0:c>
       <ns0:c r="T93" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="94" ht="210" customHeight="1">
@@ -6004,7 +6065,9 @@
       <ns0:c r="E94" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/falafelland/</ns0:v>
       </ns0:c>
-      <ns0:c r="F94" s="7" t="str"/>
+      <ns0:c r="F94" s="7" t="str">
+        <ns0:v>Unverified phone candidate 07984 063411 appears only on a pricing directory: https://uk.pricelisto.com/menu-prices/falafelland-uk . Not included as a usable phone; confirm independently.</ns0:v>
+      </ns0:c>
       <ns0:c r="G94" s="7" t="str"/>
       <ns0:c r="H94" s="7" t="str"/>
       <ns0:c r="I94" s="7" t="str">
@@ -6017,7 +6080,7 @@
         <ns0:v>Help visitors explore mezze choices before ordering or visiting.</ns0:v>
       </ns0:c>
       <ns0:c r="K94" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Falafelland. it includes searchable hot and cold mezze selection and existing Uber Eats link and Gallowtree Gate visit information. the idea is to help visitors explore mezze choices before ordering or visiting. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Falafelland. It includes searchable hot and cold mezze selection and existing Uber Eats link and Gallowtree Gate visit information. The idea is to help visitors explore mezze choices before ordering or visiting. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L94" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -6043,10 +6106,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S94" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T94" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="95" ht="210" customHeight="1">
@@ -6078,7 +6141,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K95" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Amo’s Cutthroat. visitors can compare options such as Beard Trim and Condition and Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Amo’s Cutthroat. Visitors can compare options such as Beard Trim and Condition and Taper fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L95" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6101,10 +6164,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S95" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T95" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="96" ht="210" customHeight="1">
@@ -6136,7 +6199,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K96" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Til Next Time Barbershop. visitors can compare options such as Haircut with Martin and Haircut with Alex, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Til Next Time Barbershop. Visitors can compare options such as Haircut with Martin and Haircut with Alex, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L96" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6159,10 +6222,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S96" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T96" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: phone, published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="97" ht="210" customHeight="1">
@@ -6176,17 +6239,20 @@
         <ns0:v>0116 291 8060</ns0:v>
       </ns0:c>
       <ns0:c r="D97" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>feina89722@gmail.com</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/karamay/</ns0:v>
       </ns0:c>
-      <ns0:c r="F97" s="7" t="str"/>
+      <ns0:c r="F97" s="7" t="str">
+        <ns0:v>Email feina89722@gmail.com: Directory-listed business inbox, corroborated by ThreeBestRated; exact 63 London Road and phone match. Named recipient and deliverability untested. Confirm current routing. London branch and recruitment emails excluded; dissolved historical company not used to infer current owner.</ns0:v>
+      </ns0:c>
       <ns0:c r="G97" s="7" t="str">
-        <ns0:v>2026-10-11</ns0:v>
+        <ns0:v>2026-10-11; 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="H97" s="7" t="str">
-        <ns0:v>https://visitleicester.info/point-of-interest/karamay/</ns0:v>
+        <ns0:v>https://visitleicester.info/point-of-interest/karamay/
+https://www.bizseek.co.uk/karamay-uyghur-cuisine-0116-429-9129</ns0:v>
       </ns0:c>
       <ns0:c r="I97" s="7" t="str">
         <ns0:v>Searchable Uyghur menu across noodles, dumplings, skewers and vegetables
@@ -6199,7 +6265,7 @@
         <ns0:v>Help diners explore unfamiliar dishes and find the next step for a visit or order.</ns0:v>
       </ns0:c>
       <ns0:c r="K97" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Karamay Hot Pot. it includes searchable Uyghur menu across noodles, dumplings, skewers and vegetables and links to the existing business and ordering pages. the idea is to help diners explore unfamiliar dishes and find the next step for a visit or order. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Karamay Hot Pot. It includes searchable Uyghur menu across noodles, dumplings, skewers and vegetables and links to the existing business and ordering pages. The idea is to help diners explore unfamiliar dishes and find the next step for a visit or order. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L97" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -6223,13 +6289,13 @@
         <ns0:v>None verified</ns0:v>
       </ns0:c>
       <ns0:c r="R97" s="7" t="str">
-        <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
+        <ns0:v>feina89722@gmail.com: Directory-listed business inbox, corroborated by ThreeBestRated; exact 63 London Road and phone match. Named recipient and deliverability untested. Confirm current routing.</ns0:v>
       </ns0:c>
       <ns0:c r="S97" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T97" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="98" ht="210" customHeight="1">
@@ -6248,7 +6314,9 @@
       <ns0:c r="E98" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/by-nancy/</ns0:v>
       </ns0:c>
-      <ns0:c r="F98" s="7" t="str"/>
+      <ns0:c r="F98" s="7" t="str">
+        <ns0:v>Phone +44 7725 441079: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G98" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -6265,7 +6333,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K98" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for By Nancy. visitors can compare options such as BIAB Manicure and BIAB Manicure &amp; Simple Nail Art, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for By Nancy. Visitors can compare options such as BIAB Manicure and BIAB Manicure &amp; Simple Nail Art, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L98" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6275,12 +6343,15 @@
 Open directions in Google Maps: https://www.google.com/maps/search/?api=1&amp;query=2%20Orange%20Street%20Belle%20Ame%20Salon%2C%20South%20Wigston%20LE18%204QB</ns0:v>
       </ns0:c>
       <ns0:c r="N98" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Nancy</ns0:v>
       </ns0:c>
       <ns0:c r="O98" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. </ns0:v>
-      </ns0:c>
-      <ns0:c r="P98" s="7" t="str"/>
+        <ns0:v>Owner. Explicit owner role in booking provider team section; surname not independently verified.</ns0:v>
+      </ns0:c>
+      <ns0:c r="P98" s="7" t="str">
+        <ns0:v>https://www.fresha.com/a/by-nancy-south-wigston-2-orange-street-vpssmvw9
+Checked: 2026-10-25</ns0:v>
+      </ns0:c>
       <ns0:c r="Q98" s="7" t="str">
         <ns0:v>Nancy (Listed staff member, not a verified owner/decision maker.)</ns0:v>
       </ns0:c>
@@ -6288,10 +6359,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S98" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi Nancy,</ns0:v>
       </ns0:c>
       <ns0:c r="T98" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="99" ht="210" customHeight="1">
@@ -6310,7 +6381,9 @@
       <ns0:c r="E99" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/elmaybeauty-x/</ns0:v>
       </ns0:c>
-      <ns0:c r="F99" s="7" t="str"/>
+      <ns0:c r="F99" s="7" t="str">
+        <ns0:v>Phone +44 7519 349743: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G99" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -6327,7 +6400,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K99" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for elmaybeauty.x. visitors can compare options such as Double classic infill and Korean lash lift, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for elmaybeauty.x. Visitors can compare options such as Double classic infill and Korean lash lift, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L99" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6350,10 +6423,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S99" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T99" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="100" ht="210" customHeight="1">
@@ -6373,7 +6446,7 @@
         <ns0:v>https://venturasolutions.co.uk/bruxelles/</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="7" t="str">
-        <ns0:v>Phone 0116 224 3013: Secondary directory number; current routing unconfirmed. Email hello@bruxelles-leicester.com: Directory current field; domain is construction shell, inbox untested.</ns0:v>
+        <ns0:v>Phone 0116 224 3013: Secondary directory number; current routing unconfirmed. Email hello@bruxelles-leicester.com: Directory current field; domain is construction shell, inbox untested. Undated proprietor listing and dissolved historical company excluded from current owner field.</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -6390,7 +6463,7 @@
         <ns0:v>Help groups organise what to check with the venue before a visit.</ns0:v>
       </ns0:c>
       <ns0:c r="K100" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Café Bruxelles. it includes visit checklist for a chosen date and group size and questions covering Belgian beers, weekend plans, access and arrival. the idea is to help groups organise what to check with the venue before a visit. customers can tap the phone number to call the business. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Café Bruxelles. It includes visit checklist for a chosen date and group size and questions covering Belgian beers, weekend plans, access and arrival. The idea is to help groups organise what to check with the venue before a visit. Customers can tap the phone number to call the business. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L100" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming.</ns0:v>
@@ -6415,10 +6488,10 @@
         <ns0:v>hello@bruxelles-leicester.com: Directory current field; domain is construction shell, inbox untested.</ns0:v>
       </ns0:c>
       <ns0:c r="S100" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T100" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="101" ht="210" customHeight="1">
@@ -6438,7 +6511,7 @@
         <ns0:v>https://venturasolutions.co.uk/deliish/</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="7" t="str">
-        <ns0:v>Email enquiries@deli-ish.co.uk: Exact-address TripAdvisor public email; inbox not tested.</ns0:v>
+        <ns0:v>Email enquiries@deli-ish.co.uk: Exact-address TripAdvisor public email; inbox not tested. </ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="7" t="str">
         <ns0:v>2026-10-10</ns0:v>
@@ -6458,7 +6531,7 @@
         <ns0:v>Help customers narrow down lunch options before checking ingredients and ordering.</ns0:v>
       </ns0:c>
       <ns0:c r="K101" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Deliish. it includes filter for vegetarian menu listings and item detail views across breakfast, paninis, wraps and salads. the idea is to help customers narrow down lunch options before checking ingredients and ordering. the site also links to your existing Deliveroo menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Deliish. It includes filter for vegetarian menu listings and item detail views across breakfast, paninis, wraps and salads. The idea is to help customers narrow down lunch options before checking ingredients and ordering. The site also links to your existing Deliveroo menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L101" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -6469,14 +6542,14 @@
 Tap to call +441162628674: tel:+441162628674</ns0:v>
       </ns0:c>
       <ns0:c r="N101" s="7" t="str">
-        <ns0:v>Not verified</ns0:v>
+        <ns0:v>Tom (surname not verified)</ns0:v>
       </ns0:c>
       <ns0:c r="O101" s="7" t="str">
-        <ns0:v>Owner or decision maker not verified. Exact-name and company candidate search did not verify a current local decision-maker.</ns0:v>
+        <ns0:v>Owner named in supplier testimonial. Undated testimonial; historical attribution only. Current ownership must be confirmed before personalising.</ns0:v>
       </ns0:c>
       <ns0:c r="P101" s="7" t="str">
-        <ns0:v>
-Checked: 2026-09-26</ns0:v>
+        <ns0:v>https://eatpos.co.uk/testimonials/deliish/
+Checked: 2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="Q101" s="7" t="str">
         <ns0:v>Tom and Maz (EPOS supplier testimonial names experienced operators; undated/historical attribution, current ownership unverified.)</ns0:v>
@@ -6485,10 +6558,10 @@
         <ns0:v>enquiries@deli-ish.co.uk: Exact-address TripAdvisor public email; inbox not tested.</ns0:v>
       </ns0:c>
       <ns0:c r="S101" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T101" s="7" t="str">
-        <ns0:v>Saved 414 research reviewed; source date retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Contact fields have public-source leads; see role and source caveats.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="102" ht="210" customHeight="1">
@@ -6499,7 +6572,7 @@
         <ns0:v>Ink&amp;Beauty Factory</ns0:v>
       </ns0:c>
       <ns0:c r="C102" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>07479 443197</ns0:v>
       </ns0:c>
       <ns0:c r="D102" s="8" t="str">
         <ns0:v>Not found</ns0:v>
@@ -6507,9 +6580,15 @@
       <ns0:c r="E102" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/ink-beauty-factory/</ns0:v>
       </ns0:c>
-      <ns0:c r="F102" s="7" t="str"/>
-      <ns0:c r="G102" s="7" t="str"/>
-      <ns0:c r="H102" s="7" t="str"/>
+      <ns0:c r="F102" s="7" t="str">
+        <ns0:v>Phone 07479 443197: Directory mirrors business posts; LE3 2BL and booking profile match. Not call-tested. </ns0:v>
+      </ns0:c>
+      <ns0:c r="G102" s="7" t="str">
+        <ns0:v>2026-10-25</ns0:v>
+      </ns0:c>
+      <ns0:c r="H102" s="7" t="str">
+        <ns0:v>https://www.beautynailhairsalons.com/GB/Leicester/107976825101348/Ink%26Beauty-Factory---Ewelina-Ewiak</ns0:v>
+      </ns0:c>
       <ns0:c r="I102" s="7" t="str">
         <ns0:v>Service selector including Brow architecture · mapping and shaping and Lash Removal
 Listed prices and appointment lengths update with the selected service
@@ -6520,7 +6599,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K102" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Ink&amp;Beauty Factory. visitors can compare options such as Brow architecture · mapping and shaping and Lash Removal, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Ink&amp;Beauty Factory. Visitors can compare options such as Brow architecture · mapping and shaping and Lash Removal, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L102" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6537,16 +6616,16 @@
       </ns0:c>
       <ns0:c r="P102" s="7" t="str"/>
       <ns0:c r="Q102" s="7" t="str">
-        <ns0:v>Ewelina Ewiak (Listed staff member, not a verified owner/decision maker.)</ns0:v>
+        <ns0:v>Ewelina Ewiak (Listed staff member, not a verified owner/decision maker.); Ewelina Ewiak (Named beauty practitioner; ownership not verified)</ns0:v>
       </ns0:c>
       <ns0:c r="R102" s="7" t="str">
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S102" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T102" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="103" ht="210" customHeight="1">
@@ -6565,7 +6644,9 @@
       <ns0:c r="E103" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/shortys-leicester/</ns0:v>
       </ns0:c>
-      <ns0:c r="F103" s="7" t="str"/>
+      <ns0:c r="F103" s="7" t="str">
+        <ns0:v>Phone +44 7384 597469: Published provider phone, not evidence of WhatsApp. </ns0:v>
+      </ns0:c>
       <ns0:c r="G103" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
@@ -6582,7 +6663,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K103" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Shortys - Leicester. visitors can compare options such as Haircut (Leicester) and Haircut and beard trim, see the listed price and appointment length, then open your Fresha booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Shortys - Leicester. Visitors can compare options such as Haircut (Leicester) and Haircut and beard trim, see the listed price and appointment length, then open your Fresha booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Fresha page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L103" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6605,10 +6686,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S103" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T103" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="104" ht="210" customHeight="1">
@@ -6644,7 +6725,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K104" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Taurus barbers. visitors can compare options such as SkinFade and Classic Haircut, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Taurus barbers. Visitors can compare options such as SkinFade and Classic Haircut, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L104" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6667,10 +6748,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S104" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T104" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="105" ht="210" customHeight="1">
@@ -6681,7 +6762,7 @@
         <ns0:v>Hair Roots &amp; Co</ns0:v>
       </ns0:c>
       <ns0:c r="C105" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>0116 319 5520</ns0:v>
       </ns0:c>
       <ns0:c r="D105" s="8" t="str">
         <ns0:v>Not found</ns0:v>
@@ -6689,9 +6770,15 @@
       <ns0:c r="E105" s="9" t="str">
         <ns0:v>https://venturasolutions.co.uk/hair-roots-co/</ns0:v>
       </ns0:c>
-      <ns0:c r="F105" s="7" t="str"/>
-      <ns0:c r="G105" s="7" t="str"/>
-      <ns0:c r="H105" s="7" t="str"/>
+      <ns0:c r="F105" s="7" t="str">
+        <ns0:v>Phone 0116 319 5520: Exact 749 Aylestone Road directory listing. Confirm current routing. </ns0:v>
+      </ns0:c>
+      <ns0:c r="G105" s="7" t="str">
+        <ns0:v>2026-10-25</ns0:v>
+      </ns0:c>
+      <ns0:c r="H105" s="7" t="str">
+        <ns0:v>https://www.yell.com/biz/hair-roots-leicester-8837240/</ns0:v>
+      </ns0:c>
       <ns0:c r="I105" s="7" t="str">
         <ns0:v>Service selector including Haircut and Skin-Fade/Taper fade
 Listed prices and appointment lengths update with the selected service
@@ -6702,7 +6789,7 @@
         <ns0:v>Help clients compare the service, listed price and appointment length before opening the existing booking provider.</ns0:v>
       </ns0:c>
       <ns0:c r="K105" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Hair Roots &amp; Co. visitors can compare options such as Haircut and Skin-Fade/Taper fade, see the listed price and appointment length, then open your Booksy booking page. the idea is to help them choose the right type of appointment before booking. the booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Hair Roots &amp; Co. Visitors can compare options such as Haircut and Skin-Fade/Taper fade, see the listed price and appointment length, then open your Booksy booking page. The idea is to help them choose the right type of appointment before booking. The booking buttons link directly to your existing Booksy page, where customers can choose their service and appointment. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L105" s="7" t="str">
         <ns0:v>The button opens the business booking page, not a preselected service. Service choices, dates and customer details are not transferred. Listed prices and durations are saved references; the provider confirms current details. Email signup is a demonstration.</ns0:v>
@@ -6725,10 +6812,10 @@
         <ns0:v>No published email verified in the scoped research; no guessed address.</ns0:v>
       </ns0:c>
       <ns0:c r="S105" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T105" s="7" t="str">
-        <ns0:v>Later addition: saved provider evidence plus public contact search on 25 October 2026; no verified owner email recovered</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Not found in public sources checked: published email, owner.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="106" ht="210" customHeight="1">
@@ -6739,7 +6826,7 @@
         <ns0:v>Ninety Six Degrees</ns0:v>
       </ns0:c>
       <ns0:c r="C106" s="8" t="str">
-        <ns0:v>Not found</ns0:v>
+        <ns0:v>0116 255 5474</ns0:v>
       </ns0:c>
       <ns0:c r="D106" s="8" t="str">
         <ns0:v>cafe96degrees@gmail.com</ns0:v>
@@ -6748,13 +6835,14 @@
         <ns0:v>https://venturasolutions.co.uk/ninety-six-degrees/</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="7" t="str">
-        <ns0:v>Email cafe96degrees@gmail.com: Claimed exact-address business listing email; not established as Ed’s direct inbox; delivery untested.</ns0:v>
+        <ns0:v>Phone 0116 255 5474: Exact 42 Braunstone Gate listing; corroborated by Sluurpy. Not call-tested. Email cafe96degrees@gmail.com: Claimed exact-address business listing email; not established as Ed’s direct inbox; delivery untested. </ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="7" t="str">
         <ns0:v>2026-10-25</ns0:v>
       </ns0:c>
       <ns0:c r="H106" s="7" t="str">
-        <ns0:v>https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d12099644-Reviews-Ninety_Six_Degrees-Leicester_Leicestershire_England.html</ns0:v>
+        <ns0:v>https://leicester.cylex-uk.co.uk/bede-island/cafe.html
+https://www.tripadvisor.co.uk/Restaurant_Review-g186334-d12099644-Reviews-Ninety_Six_Degrees-Leicester_Leicestershire_England.html</ns0:v>
       </ns0:c>
       <ns0:c r="I106" s="7" t="str">
         <ns0:v>Searchable brunch selection grouped into bowls, toast, brunch and bread
@@ -6766,7 +6854,7 @@
         <ns0:v>Help visitors find the kind of brunch they fancy before visiting or ordering.</ns0:v>
       </ns0:c>
       <ns0:c r="K106" s="7" t="str">
-        <ns0:v>i’ve put together a website preview for Ninety Six Degrees. it includes searchable brunch selection grouped into bowls, toast, brunch and bread and existing ordering route and Braunstone Gate visit information. the idea is to help visitors find the kind of brunch they fancy before visiting or ordering. the site also links to your existing Uber Eats menu for ordering. this is a preview, with any forms still in demo mode.</ns0:v>
+        <ns0:v>I’ve put together a website preview for Ninety Six Degrees. It includes searchable brunch selection grouped into bowls, toast, brunch and bread and existing ordering route and Braunstone Gate visit information. The idea is to help visitors find the kind of brunch they fancy before visiting or ordering. The site also links to your existing Uber Eats menu for ordering. This is a preview, with any forms still in demo mode.</ns0:v>
       </ns0:c>
       <ns0:c r="L106" s="7" t="str">
         <ns0:v>Forms and email signups are demonstrations. No enquiry, order or booking is submitted by this demo. External provider links open separately; prices and availability need confirming. These links open the existing business/provider pages. Shortlists, quantities and enquiry notes are not automatically transferred.</ns0:v>
@@ -6792,10 +6880,10 @@
         <ns0:v>cafe96degrees@gmail.com: Claimed exact-address business listing email; not established as Ed’s direct inbox; delivery untested.</ns0:v>
       </ns0:c>
       <ns0:c r="S106" s="7" t="str">
-        <ns0:v>hey team,</ns0:v>
+        <ns0:v>Hi team,</ns0:v>
       </ns0:c>
       <ns0:c r="T106" s="7" t="str">
-        <ns0:v>Public source checked 25 October 2026; role and limits retained</ns0:v>
+        <ns0:v>Gap follow-up searched 25 October 2026. Contact fields have public-source leads; see role and source caveats.</ns0:v>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>
@@ -6903,7 +6991,7 @@
   </ns0:hyperlinks>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ns0:tableParts count="1">
-    <ns0:tablePart ns1:id="Recd277f211e74c18"/>
+    <ns0:tablePart ns1:id="R3d3b1e3410a1467c"/>
   </ns0:tableParts>
 </ns0:worksheet>
 </file>
</xml_diff>